<commit_message>
Filters: author design-level Parts/Reports/page-search cases (Option A, VIU-Pending)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AZ5XzKsK9wv7M41cSPaMyg
</commit_message>
<xml_diff>
--- a/testrail-import/filters-v1-testrail-import.xlsx
+++ b/testrail-import/filters-v1-testrail-import.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J80"/>
+  <dimension ref="A1:J123"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -4118,243 +4118,2304 @@
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
+          <t>Parts Inventory page shows Bin Location, Category, Supply and Vendor filters</t>
+        </is>
+      </c>
+      <c r="B76" s="2" t="inlineStr">
+        <is>
+          <t>Parts Page Filters</t>
+        </is>
+      </c>
+      <c r="C76" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D76" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E76" s="2" t="inlineStr">
+        <is>
+          <t>1. You are signed in to the ShopView App on a desktop browser.
+2. You are on the Parts area of the app with some sample data present.</t>
+        </is>
+      </c>
+      <c r="F76" s="2" t="inlineStr">
+        <is>
+          <t>1. Open the Parts area and go to the Inventory page.
+2. Look at the filter buttons shown above the parts table.</t>
+        </is>
+      </c>
+      <c r="G76" s="2" t="inlineStr">
+        <is>
+          <t>1. The Inventory page shows four filter buttons in a row: Bin Location, Category, Supply and Vendor (each with a small icon and a down arrow).
+2. The table below shows the columns: Description, Part number, Tags, Category, Manufacturer, Vendor, Bin Location / Quantity and Action.
+3. A blue New Inventory Part button is shown at the top right.</t>
+        </is>
+      </c>
+      <c r="H76" s="2" t="inlineStr">
+        <is>
+          <t>Filters (Epic key TBD); Figma 11884-16885 (Parts filters); design-notes.md §B.5 #1</t>
+        </is>
+      </c>
+      <c r="I76" s="2" t="inlineStr"/>
+      <c r="J76" s="2" t="inlineStr"/>
+    </row>
+    <row r="77">
+      <c r="A77" s="2" t="inlineStr">
+        <is>
+          <t>Parts Part Sales page shows Status, Customer, Created by and Date filters</t>
+        </is>
+      </c>
+      <c r="B77" s="2" t="inlineStr">
+        <is>
+          <t>Parts Page Filters</t>
+        </is>
+      </c>
+      <c r="C77" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D77" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E77" s="2" t="inlineStr">
+        <is>
+          <t>1. You are signed in to the ShopView App on a desktop browser.
+2. You are on the Parts area of the app with some sample data present.</t>
+        </is>
+      </c>
+      <c r="F77" s="2" t="inlineStr">
+        <is>
+          <t>1. Open the Parts area and go to the Part Sales page.
+2. Look at the filter buttons shown above the part sales table.</t>
+        </is>
+      </c>
+      <c r="G77" s="2" t="inlineStr">
+        <is>
+          <t>1. The Part Sales page shows four filter buttons: Status, Customer, Created by and Date.
+2. The table shows the columns: Number, Status, Customer, Asset, VIN/Serial #, Created By, Total Price, Created On, Parts and Returns.
+3. A blue New Part Sale button is shown at the top right.</t>
+        </is>
+      </c>
+      <c r="H77" s="2" t="inlineStr">
+        <is>
+          <t>Filters (Epic key TBD); Figma 11884-16885 (Parts filters); design-notes.md §B.5 #2</t>
+        </is>
+      </c>
+      <c r="I77" s="2" t="inlineStr"/>
+      <c r="J77" s="2" t="inlineStr"/>
+    </row>
+    <row r="78">
+      <c r="A78" s="2" t="inlineStr">
+        <is>
+          <t>Parts Catalog page shows Manufacturer and Category filters</t>
+        </is>
+      </c>
+      <c r="B78" s="2" t="inlineStr">
+        <is>
+          <t>Parts Page Filters</t>
+        </is>
+      </c>
+      <c r="C78" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D78" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E78" s="2" t="inlineStr">
+        <is>
+          <t>1. You are signed in to the ShopView App on a desktop browser.
+2. You are on the Parts area of the app with some sample data present.</t>
+        </is>
+      </c>
+      <c r="F78" s="2" t="inlineStr">
+        <is>
+          <t>1. Open the Parts area and go to the Catalog page.
+2. Look at the filter buttons shown above the catalog table.</t>
+        </is>
+      </c>
+      <c r="G78" s="2" t="inlineStr">
+        <is>
+          <t>1. The Catalog page shows two filter buttons: Manufacturer and Category.
+2. The table shows the columns: (row checkbox), Description, Part Number, Tags and Category.
+3. A blue New Catalog Part button is shown at the top right.</t>
+        </is>
+      </c>
+      <c r="H78" s="2" t="inlineStr">
+        <is>
+          <t>Filters (Epic key TBD); Figma 11884-16885 (Parts filters); design-notes.md §B.5 #3</t>
+        </is>
+      </c>
+      <c r="I78" s="2" t="inlineStr"/>
+      <c r="J78" s="2" t="inlineStr"/>
+    </row>
+    <row r="79">
+      <c r="A79" s="2" t="inlineStr">
+        <is>
+          <t>Parts Returns tab shows Vendor, Category and Part Type filters</t>
+        </is>
+      </c>
+      <c r="B79" s="2" t="inlineStr">
+        <is>
+          <t>Parts Page Filters</t>
+        </is>
+      </c>
+      <c r="C79" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D79" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E79" s="2" t="inlineStr">
+        <is>
+          <t>1. You are signed in to the ShopView App on a desktop browser.
+2. You are on the Parts area of the app with some sample data present.</t>
+        </is>
+      </c>
+      <c r="F79" s="2" t="inlineStr">
+        <is>
+          <t>1. Open the Parts area and go to the Returns page.
+2. Make sure the Returns tab is selected (the page has Returns and Credits tabs).
+3. Look at the filter buttons shown above the returns table.</t>
+        </is>
+      </c>
+      <c r="G79" s="2" t="inlineStr">
+        <is>
+          <t>1. The Returns tab shows three filter buttons: Vendor, Category and Part Type.
+2. The table shows the columns: Work Order, Vendor Invoice, Vendor, Part Number, Description, Quantity, Cost, Total Cost, Return Reason, Status and Requested.
+3. A blue Create Return button is shown at the top right.</t>
+        </is>
+      </c>
+      <c r="H79" s="2" t="inlineStr">
+        <is>
+          <t>Filters (Epic key TBD); Figma 11884-16885 (Parts filters); design-notes.md §B.5 #4</t>
+        </is>
+      </c>
+      <c r="I79" s="2" t="inlineStr"/>
+      <c r="J79" s="2" t="inlineStr"/>
+    </row>
+    <row r="80">
+      <c r="A80" s="2" t="inlineStr">
+        <is>
+          <t>Parts Credits tab shows Vendor, Date and Processed by filters</t>
+        </is>
+      </c>
+      <c r="B80" s="2" t="inlineStr">
+        <is>
+          <t>Parts Page Filters</t>
+        </is>
+      </c>
+      <c r="C80" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D80" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E80" s="2" t="inlineStr">
+        <is>
+          <t>1. You are signed in to the ShopView App on a desktop browser.
+2. You are on the Parts area of the app with some sample data present.</t>
+        </is>
+      </c>
+      <c r="F80" s="2" t="inlineStr">
+        <is>
+          <t>1. Open the Parts area and go to the Returns page.
+2. Select the Credits tab.
+3. Look at the filter buttons shown above the credits table.</t>
+        </is>
+      </c>
+      <c r="G80" s="2" t="inlineStr">
+        <is>
+          <t>1. The Credits tab shows three filter buttons: Vendor, Date and Processed by.
+2. The table shows the columns: Credit Memo Number, Vendor, Work Order, Vendor Invoice, Date, Processed By, Total Cost and Notes.
+3. A blue Create Credit button is shown at the top right.</t>
+        </is>
+      </c>
+      <c r="H80" s="2" t="inlineStr">
+        <is>
+          <t>Filters (Epic key TBD); Figma 11884-16885 (Parts filters); design-notes.md §B.5 #5</t>
+        </is>
+      </c>
+      <c r="I80" s="2" t="inlineStr"/>
+      <c r="J80" s="2" t="inlineStr"/>
+    </row>
+    <row r="81">
+      <c r="A81" s="2" t="inlineStr">
+        <is>
+          <t>Parts Purchase Orders page shows Vendor, Status, Date and Ordered by filters</t>
+        </is>
+      </c>
+      <c r="B81" s="2" t="inlineStr">
+        <is>
+          <t>Parts Page Filters</t>
+        </is>
+      </c>
+      <c r="C81" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D81" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E81" s="2" t="inlineStr">
+        <is>
+          <t>1. You are signed in to the ShopView App on a desktop browser.
+2. You are on the Parts area of the app with some sample data present.</t>
+        </is>
+      </c>
+      <c r="F81" s="2" t="inlineStr">
+        <is>
+          <t>1. Open the Parts area and go to the Purchase Orders page.
+2. Look at the filter buttons shown above the purchase orders table.</t>
+        </is>
+      </c>
+      <c r="G81" s="2" t="inlineStr">
+        <is>
+          <t>1. The Purchase Orders page shows four filter buttons: Vendor, Status, Date and Ordered by.
+2. The table shows the columns: Work Order, Purchase Order Number, Vendor, Order Status, Created On, Ordered By, Total Price and Note.
+3. A blue New Purchase Order button is shown at the top right.</t>
+        </is>
+      </c>
+      <c r="H81" s="2" t="inlineStr">
+        <is>
+          <t>Filters (Epic key TBD); Figma 11884-16885 (Parts filters); design-notes.md §B.5 #6</t>
+        </is>
+      </c>
+      <c r="I81" s="2" t="inlineStr"/>
+      <c r="J81" s="2" t="inlineStr"/>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="inlineStr">
+        <is>
+          <t>Vendor Invoices page shows Vendor, Invoice date, Date received, Received by</t>
+        </is>
+      </c>
+      <c r="B82" s="2" t="inlineStr">
+        <is>
+          <t>Parts Page Filters</t>
+        </is>
+      </c>
+      <c r="C82" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D82" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E82" s="2" t="inlineStr">
+        <is>
+          <t>1. You are signed in to the ShopView App on a desktop browser.
+2. You are on the Parts area of the app with some sample data present.</t>
+        </is>
+      </c>
+      <c r="F82" s="2" t="inlineStr">
+        <is>
+          <t>1. Open the Parts area and go to the Vendor Invoices page.
+2. Look at the filter buttons shown above the vendor invoices table.</t>
+        </is>
+      </c>
+      <c r="G82" s="2" t="inlineStr">
+        <is>
+          <t>1. The Vendor Invoices page shows four filter buttons: Vendor, Invoice date, Date received and Received by.
+2. The table shows the columns: Work Order, Invoice Number, Order Number, Received By, Vendor Name, Date Received, Invoice Date, Due Date, Total Cost and Note.
+3. There is no New button on this page (only the search and filter icons).</t>
+        </is>
+      </c>
+      <c r="H82" s="2" t="inlineStr">
+        <is>
+          <t>Filters (Epic key TBD); Figma 11884-16885 (Parts filters); design-notes.md §B.5 #7</t>
+        </is>
+      </c>
+      <c r="I82" s="2" t="inlineStr"/>
+      <c r="J82" s="2" t="inlineStr"/>
+    </row>
+    <row r="83">
+      <c r="A83" s="2" t="inlineStr">
+        <is>
+          <t>Parts Vendors list page shows Vendor and State/Province filters</t>
+        </is>
+      </c>
+      <c r="B83" s="2" t="inlineStr">
+        <is>
+          <t>Parts Page Filters</t>
+        </is>
+      </c>
+      <c r="C83" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D83" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E83" s="2" t="inlineStr">
+        <is>
+          <t>1. You are signed in to the ShopView App on a desktop browser.
+2. You are on the Parts area of the app with some sample data present.</t>
+        </is>
+      </c>
+      <c r="F83" s="2" t="inlineStr">
+        <is>
+          <t>1. Open the Parts area and go to the Vendors list page.
+2. Look at the filter buttons shown above the vendors table.</t>
+        </is>
+      </c>
+      <c r="G83" s="2" t="inlineStr">
+        <is>
+          <t>1. The Vendors page shows two filter buttons: Vendor and State/Province.
+2. The table shows the columns: Name, Telephone, Email, Address 1, Address 2, City, State/Province and Zip/Postal Code.
+3. A blue New Vendor button is shown at the top right.</t>
+        </is>
+      </c>
+      <c r="H83" s="2" t="inlineStr">
+        <is>
+          <t>Filters (Epic key TBD); Figma 11884-16885 (Parts filters); design-notes.md §B.5 #8</t>
+        </is>
+      </c>
+      <c r="I83" s="2" t="inlineStr"/>
+      <c r="J83" s="2" t="inlineStr"/>
+    </row>
+    <row r="84">
+      <c r="A84" s="2" t="inlineStr">
+        <is>
+          <t>Part Type filter opens a Core / Non Core list with Clear selection</t>
+        </is>
+      </c>
+      <c r="B84" s="2" t="inlineStr">
+        <is>
+          <t>Parts Page Filters</t>
+        </is>
+      </c>
+      <c r="C84" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D84" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E84" s="2" t="inlineStr">
+        <is>
+          <t>1. You are signed in to the ShopView App on a desktop browser.
+2. You are on the Parts area of the app with some sample data present.</t>
+        </is>
+      </c>
+      <c r="F84" s="2" t="inlineStr">
+        <is>
+          <t>1. On the Parts Returns tab, click the Part Type filter button.
+2. Look at the small menu that opens.</t>
+        </is>
+      </c>
+      <c r="G84" s="2" t="inlineStr">
+        <is>
+          <t>1. A small menu opens with two options: Core and Non Core.
+2. A Clear selection action is shown at the bottom of the menu.
+3. Behaviour to confirm — pending Branko's product write-up; to be checked live once the feature is available. (whether the options are single- or multi-select, and how the list is filtered after choosing).</t>
+        </is>
+      </c>
+      <c r="H84" s="2" t="inlineStr">
+        <is>
+          <t>Filters (Epic key TBD); Figma 11884-16885 (Parts filters); design-notes.md §B.5 #9</t>
+        </is>
+      </c>
+      <c r="I84" s="2" t="inlineStr"/>
+      <c r="J84" s="2" t="inlineStr"/>
+    </row>
+    <row r="85">
+      <c r="A85" s="2" t="inlineStr">
+        <is>
+          <t>Parts pages show the shared search and filter toolbar icons</t>
+        </is>
+      </c>
+      <c r="B85" s="2" t="inlineStr">
+        <is>
+          <t>Parts Page Filters</t>
+        </is>
+      </c>
+      <c r="C85" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D85" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E85" s="2" t="inlineStr">
+        <is>
+          <t>1. You are signed in to the ShopView App on a desktop browser.
+2. You are on the Parts area of the app with some sample data present.</t>
+        </is>
+      </c>
+      <c r="F85" s="2" t="inlineStr">
+        <is>
+          <t>1. Open any Parts list page (for example Inventory).
+2. Look at the small icons on the right side of the toolbar.</t>
+        </is>
+      </c>
+      <c r="G85" s="2" t="inlineStr">
+        <is>
+          <t>1. The toolbar shows a Search (magnifier) icon and a filter (funnel) icon on every Parts list page.
+2. Some pages also show a column/layout toggle icon (for example Inventory).
+3. Behaviour to confirm — pending Branko's product write-up; to be checked live once the feature is available. (what the funnel and column icons do).</t>
+        </is>
+      </c>
+      <c r="H85" s="2" t="inlineStr">
+        <is>
+          <t>Filters (Epic key TBD); Figma 11884-16885 (Parts filters); design-notes.md §B.5 shared shell</t>
+        </is>
+      </c>
+      <c r="I85" s="2" t="inlineStr"/>
+      <c r="J85" s="2" t="inlineStr"/>
+    </row>
+    <row r="86">
+      <c r="A86" s="2" t="inlineStr">
+        <is>
+          <t>Choosing a Parts filter narrows the list on that page</t>
+        </is>
+      </c>
+      <c r="B86" s="2" t="inlineStr">
+        <is>
+          <t>Parts Page Filters</t>
+        </is>
+      </c>
+      <c r="C86" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D86" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E86" s="2" t="inlineStr">
+        <is>
+          <t>1. You are signed in to the ShopView App on a desktop browser.
+2. You are on the Parts area of the app with some sample data present.</t>
+        </is>
+      </c>
+      <c r="F86" s="2" t="inlineStr">
+        <is>
+          <t>1. Open a Parts list page that has a filter button (for example Inventory).
+2. Open a filter button and choose one value.
+3. Watch the table below.</t>
+        </is>
+      </c>
+      <c r="G86" s="2" t="inlineStr">
+        <is>
+          <t>1. The table updates to show only the rows that match the chosen filter value.
+2. The chosen value is shown on the filter button so you can see what is applied.
+3. Behaviour to confirm — pending Branko's product write-up; to be checked live once the feature is available. (exactly which filters apply on which Parts page, the full option lists, and whether results update immediately).</t>
+        </is>
+      </c>
+      <c r="H86" s="2" t="inlineStr">
+        <is>
+          <t>Filters (Epic key TBD); Figma 11884-16885 (Parts filters); design-notes.md §B.5</t>
+        </is>
+      </c>
+      <c r="I86" s="2" t="inlineStr"/>
+      <c r="J86" s="2" t="inlineStr"/>
+    </row>
+    <row r="87">
+      <c r="A87" s="2" t="inlineStr">
+        <is>
+          <t>Parts filters support multiple choices and can be cleared</t>
+        </is>
+      </c>
+      <c r="B87" s="2" t="inlineStr">
+        <is>
+          <t>Parts Page Filters</t>
+        </is>
+      </c>
+      <c r="C87" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D87" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E87" s="2" t="inlineStr">
+        <is>
+          <t>1. You are signed in to the ShopView App on a desktop browser.
+2. You are on the Parts area of the app with some sample data present.</t>
+        </is>
+      </c>
+      <c r="F87" s="2" t="inlineStr">
+        <is>
+          <t>1. Open a Parts filter button that shows a list of choices.
+2. Try selecting more than one choice.
+3. Use the Clear selection action, then look at the filter bar for a way to clear all filters.</t>
+        </is>
+      </c>
+      <c r="G87" s="2" t="inlineStr">
+        <is>
+          <t>1. More than one value can be chosen inside a filter (to be checked live once available).
+2. Clear selection removes the choices for that one filter.
+3. Behaviour to confirm — pending Branko's product write-up; to be checked live once the feature is available. (whether multi-select, per-filter Clear selection, and an overall Clear filters action all work the same as on the Work Orders page).</t>
+        </is>
+      </c>
+      <c r="H87" s="2" t="inlineStr">
+        <is>
+          <t>Filters (Epic key TBD); Figma 11884-16885 (Parts filters); design-notes.md §B.5</t>
+        </is>
+      </c>
+      <c r="I87" s="2" t="inlineStr"/>
+      <c r="J87" s="2" t="inlineStr"/>
+    </row>
+    <row r="88">
+      <c r="A88" s="2" t="inlineStr">
+        <is>
+          <t>Timesheet Activities report shows Staff, Date, Status, Modified by filters</t>
+        </is>
+      </c>
+      <c r="B88" s="2" t="inlineStr">
+        <is>
+          <t>Reports Page Filters</t>
+        </is>
+      </c>
+      <c r="C88" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D88" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E88" s="2" t="inlineStr">
+        <is>
+          <t>1. You are signed in to the ShopView App on a desktop browser.
+2. You are on the Reports area of the app with some sample data present.</t>
+        </is>
+      </c>
+      <c r="F88" s="2" t="inlineStr">
+        <is>
+          <t>1. Open the Reports area and go to the Timesheet Activities report.
+2. Look at the filter buttons shown above the report table.</t>
+        </is>
+      </c>
+      <c r="G88" s="2" t="inlineStr">
+        <is>
+          <t>1. The Timesheet Activities report shows four filter buttons: Staff, Date, Status and Modified by.
+2. The table shows columns including Date, Employee, Work Order, Clock In Activity, Clock In, Clock Out, Total Hours, WO Hours, Internal Hours, Modified By and Modified Date/Time.</t>
+        </is>
+      </c>
+      <c r="H88" s="2" t="inlineStr">
+        <is>
+          <t>Filters (Epic key TBD); Figma 11903-10573 (Reports filters); design-notes.md §B.6 #1</t>
+        </is>
+      </c>
+      <c r="I88" s="2" t="inlineStr"/>
+      <c r="J88" s="2" t="inlineStr"/>
+    </row>
+    <row r="89">
+      <c r="A89" s="2" t="inlineStr">
+        <is>
+          <t>Payroll Timesheet report shows Employee and Date filters</t>
+        </is>
+      </c>
+      <c r="B89" s="2" t="inlineStr">
+        <is>
+          <t>Reports Page Filters</t>
+        </is>
+      </c>
+      <c r="C89" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D89" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E89" s="2" t="inlineStr">
+        <is>
+          <t>1. You are signed in to the ShopView App on a desktop browser.
+2. You are on the Reports area of the app with some sample data present.</t>
+        </is>
+      </c>
+      <c r="F89" s="2" t="inlineStr">
+        <is>
+          <t>1. Open the Reports area and go to the Timesheets (Payroll Timesheet) report.
+2. Look at the filter buttons shown above the report table.</t>
+        </is>
+      </c>
+      <c r="G89" s="2" t="inlineStr">
+        <is>
+          <t>1. The Payroll Timesheet report shows two filter buttons: Employee and Date.
+2. The table shows columns: Employee Name, Date, Clock In Time, Lunch, Clock Out Time and Hours.</t>
+        </is>
+      </c>
+      <c r="H89" s="2" t="inlineStr">
+        <is>
+          <t>Filters (Epic key TBD); Figma 11903-10573 (Reports filters); design-notes.md §B.6 #2</t>
+        </is>
+      </c>
+      <c r="I89" s="2" t="inlineStr"/>
+      <c r="J89" s="2" t="inlineStr"/>
+    </row>
+    <row r="90">
+      <c r="A90" s="2" t="inlineStr">
+        <is>
+          <t>Sales report shows Customer and Date filters</t>
+        </is>
+      </c>
+      <c r="B90" s="2" t="inlineStr">
+        <is>
+          <t>Reports Page Filters</t>
+        </is>
+      </c>
+      <c r="C90" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D90" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E90" s="2" t="inlineStr">
+        <is>
+          <t>1. You are signed in to the ShopView App on a desktop browser.
+2. You are on the Reports area of the app with some sample data present.</t>
+        </is>
+      </c>
+      <c r="F90" s="2" t="inlineStr">
+        <is>
+          <t>1. Open the Reports area and go to the Sales report.
+2. Look at the filter buttons shown above the report table.</t>
+        </is>
+      </c>
+      <c r="G90" s="2" t="inlineStr">
+        <is>
+          <t>1. The Sales report shows two filter buttons: Customer and Date.
+2. The table shows columns including Invoice Date, Invoice, Customer, Inv. Hrs, Billing Efficiency, Labor Invoiced, Labor Margin, Parts Invoiced, Parts Cost, Parts Margin, Profit and Subtotal.</t>
+        </is>
+      </c>
+      <c r="H90" s="2" t="inlineStr">
+        <is>
+          <t>Filters (Epic key TBD); Figma 11903-10573 (Reports filters); design-notes.md §B.6 #3</t>
+        </is>
+      </c>
+      <c r="I90" s="2" t="inlineStr"/>
+      <c r="J90" s="2" t="inlineStr"/>
+    </row>
+    <row r="91">
+      <c r="A91" s="2" t="inlineStr">
+        <is>
+          <t>Technician Efficiency report shows Customer, Technician and Date filters</t>
+        </is>
+      </c>
+      <c r="B91" s="2" t="inlineStr">
+        <is>
+          <t>Reports Page Filters</t>
+        </is>
+      </c>
+      <c r="C91" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D91" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E91" s="2" t="inlineStr">
+        <is>
+          <t>1. You are signed in to the ShopView App on a desktop browser.
+2. You are on the Reports area of the app with some sample data present.</t>
+        </is>
+      </c>
+      <c r="F91" s="2" t="inlineStr">
+        <is>
+          <t>1. Open the Reports area and go to the Technician Efficiency report.
+2. Look at the filter buttons shown above the report table.</t>
+        </is>
+      </c>
+      <c r="G91" s="2" t="inlineStr">
+        <is>
+          <t>1. The Technician Efficiency report shows three filter buttons: Customer, Technician and Date, on both the Invoiced and Completed tabs.
+2. The report has two view tabs: Invoiced and Completed; the same three filter buttons appear on each.
+3. 'Technician' is spelled correctly here (unlike the Work Orders list, see the spelling note).</t>
+        </is>
+      </c>
+      <c r="H91" s="2" t="inlineStr">
+        <is>
+          <t>Filters (Epic key TBD); Figma 11903-10573 (Reports filters); design-notes.md §B.6 #4 and #5</t>
+        </is>
+      </c>
+      <c r="I91" s="2" t="inlineStr"/>
+      <c r="J91" s="2" t="inlineStr"/>
+    </row>
+    <row r="92">
+      <c r="A92" s="2" t="inlineStr">
+        <is>
+          <t>Advisor Analysis report shows Customer, Date and Advisor filters</t>
+        </is>
+      </c>
+      <c r="B92" s="2" t="inlineStr">
+        <is>
+          <t>Reports Page Filters</t>
+        </is>
+      </c>
+      <c r="C92" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D92" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E92" s="2" t="inlineStr">
+        <is>
+          <t>1. You are signed in to the ShopView App on a desktop browser.
+2. You are on the Reports area of the app with some sample data present.</t>
+        </is>
+      </c>
+      <c r="F92" s="2" t="inlineStr">
+        <is>
+          <t>1. Open the Reports area and go to the Advisor Analysis report.
+2. Look at the filter buttons shown above the report table.</t>
+        </is>
+      </c>
+      <c r="G92" s="2" t="inlineStr">
+        <is>
+          <t>1. The Advisor Analysis report shows three filter buttons: Customer, Date and Advisor.
+2. The table shows columns including Date, Invoice, Customer, Advisor, Days Open, Lines, Hrs Worked, Hrs Invoiced, Hrs Profit, Billing Efficiency, ELR, Parts Cost, Parts Invoiced, Parts Margin and Subtotal.</t>
+        </is>
+      </c>
+      <c r="H92" s="2" t="inlineStr">
+        <is>
+          <t>Filters (Epic key TBD); Figma 11903-10573 (Reports filters); design-notes.md §B.6 #6</t>
+        </is>
+      </c>
+      <c r="I92" s="2" t="inlineStr"/>
+      <c r="J92" s="2" t="inlineStr"/>
+    </row>
+    <row r="93">
+      <c r="A93" s="2" t="inlineStr">
+        <is>
+          <t>Shop Efficiency report shows only a Date filter</t>
+        </is>
+      </c>
+      <c r="B93" s="2" t="inlineStr">
+        <is>
+          <t>Reports Page Filters</t>
+        </is>
+      </c>
+      <c r="C93" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D93" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E93" s="2" t="inlineStr">
+        <is>
+          <t>1. You are signed in to the ShopView App on a desktop browser.
+2. You are on the Reports area of the app with some sample data present.</t>
+        </is>
+      </c>
+      <c r="F93" s="2" t="inlineStr">
+        <is>
+          <t>1. Open the Reports area and go to the Shop Efficiency report.
+2. Look at the filter buttons shown above the report table.</t>
+        </is>
+      </c>
+      <c r="G93" s="2" t="inlineStr">
+        <is>
+          <t>1. The Shop Efficiency report shows a single filter button: Date.
+2. The table shows columns: Total Clocked Hours, Total Invoiced Hours, Difference and Efficiency.</t>
+        </is>
+      </c>
+      <c r="H93" s="2" t="inlineStr">
+        <is>
+          <t>Filters (Epic key TBD); Figma 11903-10573 (Reports filters); design-notes.md §B.6 #7</t>
+        </is>
+      </c>
+      <c r="I93" s="2" t="inlineStr"/>
+      <c r="J93" s="2" t="inlineStr"/>
+    </row>
+    <row r="94">
+      <c r="A94" s="2" t="inlineStr">
+        <is>
+          <t>Work in Progress report shows Status, Date and Customer filters</t>
+        </is>
+      </c>
+      <c r="B94" s="2" t="inlineStr">
+        <is>
+          <t>Reports Page Filters</t>
+        </is>
+      </c>
+      <c r="C94" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D94" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E94" s="2" t="inlineStr">
+        <is>
+          <t>1. You are signed in to the ShopView App on a desktop browser.
+2. You are on the Reports area of the app with some sample data present.</t>
+        </is>
+      </c>
+      <c r="F94" s="2" t="inlineStr">
+        <is>
+          <t>1. Open the Reports area and go to the Work in Progress report.
+2. Look at the filter buttons shown above the report table.</t>
+        </is>
+      </c>
+      <c r="G94" s="2" t="inlineStr">
+        <is>
+          <t>1. The Work in Progress report shows three filter buttons: Status, Date and Customer.
+2. The table groups rows by status (Pending Authorization, In Progress, Ready To Invoice) with columns Sales, Cost, Profit $ and Profit %.</t>
+        </is>
+      </c>
+      <c r="H94" s="2" t="inlineStr">
+        <is>
+          <t>Filters (Epic key TBD); Figma 11903-10573 (Reports filters); design-notes.md §B.6 #8</t>
+        </is>
+      </c>
+      <c r="I94" s="2" t="inlineStr"/>
+      <c r="J94" s="2" t="inlineStr"/>
+    </row>
+    <row r="95">
+      <c r="A95" s="2" t="inlineStr">
+        <is>
+          <t>Sales Follow Up report shows Customer, Date and Contact filters</t>
+        </is>
+      </c>
+      <c r="B95" s="2" t="inlineStr">
+        <is>
+          <t>Reports Page Filters</t>
+        </is>
+      </c>
+      <c r="C95" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D95" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E95" s="2" t="inlineStr">
+        <is>
+          <t>1. You are signed in to the ShopView App on a desktop browser.
+2. You are on the Reports area of the app with some sample data present.</t>
+        </is>
+      </c>
+      <c r="F95" s="2" t="inlineStr">
+        <is>
+          <t>1. Open the Reports area and go to the Sales Follow Up report.
+2. Look at the filter buttons shown above the report table.</t>
+        </is>
+      </c>
+      <c r="G95" s="2" t="inlineStr">
+        <is>
+          <t>1. The Sales Follow Up report shows three filter buttons: Customer, Date and Contact.
+2. The table shows columns: Customer, Sales Representative, Number Of Work Orders, Total Spend and Last Visit.</t>
+        </is>
+      </c>
+      <c r="H95" s="2" t="inlineStr">
+        <is>
+          <t>Filters (Epic key TBD); Figma 11903-10573 (Reports filters); design-notes.md §B.6 #9</t>
+        </is>
+      </c>
+      <c r="I95" s="2" t="inlineStr"/>
+      <c r="J95" s="2" t="inlineStr"/>
+    </row>
+    <row r="96">
+      <c r="A96" s="2" t="inlineStr">
+        <is>
+          <t>Sales Tax Collected tab shows Date, Invoice Status and Customer filters</t>
+        </is>
+      </c>
+      <c r="B96" s="2" t="inlineStr">
+        <is>
+          <t>Reports Page Filters</t>
+        </is>
+      </c>
+      <c r="C96" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D96" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E96" s="2" t="inlineStr">
+        <is>
+          <t>1. You are signed in to the ShopView App on a desktop browser.
+2. You are on the Reports area of the app with some sample data present.</t>
+        </is>
+      </c>
+      <c r="F96" s="2" t="inlineStr">
+        <is>
+          <t>1. Open the Reports area and go to the Sales Tax (Collected tab) report.
+2. Look at the filter buttons shown above the report table.</t>
+        </is>
+      </c>
+      <c r="G96" s="2" t="inlineStr">
+        <is>
+          <t>1. On the Sales Tax report's Collected tab, three filter buttons are shown: Date, Invoice Status and Customer.
+2. The report has two view tabs: Collected and All Tax Rates.
+2. Note: in the design the report body uses a sample placeholder table, so only the title, tabs and filter buttons are design-confirmed here; the real report columns come from Branko's PRD.</t>
+        </is>
+      </c>
+      <c r="H96" s="2" t="inlineStr">
+        <is>
+          <t>Filters (Epic key TBD); Figma 11903-10573 (Reports filters); design-notes.md §B.6 #10</t>
+        </is>
+      </c>
+      <c r="I96" s="2" t="inlineStr"/>
+      <c r="J96" s="2" t="inlineStr"/>
+    </row>
+    <row r="97">
+      <c r="A97" s="2" t="inlineStr">
+        <is>
+          <t>Sales Tax All Tax Rates tab shows only an Invoice Status filter</t>
+        </is>
+      </c>
+      <c r="B97" s="2" t="inlineStr">
+        <is>
+          <t>Reports Page Filters</t>
+        </is>
+      </c>
+      <c r="C97" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D97" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E97" s="2" t="inlineStr">
+        <is>
+          <t>1. You are signed in to the ShopView App on a desktop browser.
+2. You are on the Reports area of the app with some sample data present.</t>
+        </is>
+      </c>
+      <c r="F97" s="2" t="inlineStr">
+        <is>
+          <t>1. Open the Reports area and go to the Sales Tax (All Tax Rates tab) report.
+2. Look at the filter buttons shown above the report table.</t>
+        </is>
+      </c>
+      <c r="G97" s="2" t="inlineStr">
+        <is>
+          <t>1. On the Sales Tax report's All Tax Rates tab, a single filter button is shown: Invoice Status.
+2. Note: in the design the report body uses a sample placeholder table, so only the title, tabs and filter buttons are design-confirmed here; the real report columns come from Branko's PRD.</t>
+        </is>
+      </c>
+      <c r="H97" s="2" t="inlineStr">
+        <is>
+          <t>Filters (Epic key TBD); Figma 11903-10573 (Reports filters); design-notes.md §B.6 #11</t>
+        </is>
+      </c>
+      <c r="I97" s="2" t="inlineStr"/>
+      <c r="J97" s="2" t="inlineStr"/>
+    </row>
+    <row r="98">
+      <c r="A98" s="2" t="inlineStr">
+        <is>
+          <t>A/R Aging Summary report shows Customer and Date filters</t>
+        </is>
+      </c>
+      <c r="B98" s="2" t="inlineStr">
+        <is>
+          <t>Reports Page Filters</t>
+        </is>
+      </c>
+      <c r="C98" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D98" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E98" s="2" t="inlineStr">
+        <is>
+          <t>1. You are signed in to the ShopView App on a desktop browser.
+2. You are on the Reports area of the app with some sample data present.</t>
+        </is>
+      </c>
+      <c r="F98" s="2" t="inlineStr">
+        <is>
+          <t>1. Open the Reports area and go to the A/R Aging Summary report.
+2. Look at the filter buttons shown above the report table.</t>
+        </is>
+      </c>
+      <c r="G98" s="2" t="inlineStr">
+        <is>
+          <t>1. The A/R Aging Summary report shows two filter buttons: Customer and Date.
+2. A print icon is shown in the toolbar.
+2. Note: in the design the report body uses a sample placeholder table, so only the title, tabs and filter buttons are design-confirmed here; the real report columns come from Branko's PRD.</t>
+        </is>
+      </c>
+      <c r="H98" s="2" t="inlineStr">
+        <is>
+          <t>Filters (Epic key TBD); Figma 11903-10573 (Reports filters); design-notes.md §B.6 #12</t>
+        </is>
+      </c>
+      <c r="I98" s="2" t="inlineStr"/>
+      <c r="J98" s="2" t="inlineStr"/>
+    </row>
+    <row r="99">
+      <c r="A99" s="2" t="inlineStr">
+        <is>
+          <t>A/R Aging Detail shows Customer, Date, Location, Transaction Type filters</t>
+        </is>
+      </c>
+      <c r="B99" s="2" t="inlineStr">
+        <is>
+          <t>Reports Page Filters</t>
+        </is>
+      </c>
+      <c r="C99" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D99" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E99" s="2" t="inlineStr">
+        <is>
+          <t>1. You are signed in to the ShopView App on a desktop browser.
+2. You are on the Reports area of the app with some sample data present.</t>
+        </is>
+      </c>
+      <c r="F99" s="2" t="inlineStr">
+        <is>
+          <t>1. Open the Reports area and go to the A/R Aging Detail report.
+2. Look at the filter buttons shown above the report table.</t>
+        </is>
+      </c>
+      <c r="G99" s="2" t="inlineStr">
+        <is>
+          <t>1. The A/R Aging Detail report shows four filter buttons: Customer, Date, Location and Transaction Type.
+2. A print icon is shown in the toolbar.
+3. Location and Transaction Type are new filter types not on the Work Orders page — Behaviour to confirm — pending Branko's product write-up; to be checked live once the feature is available.
+2. Note: in the design the report body uses a sample placeholder table, so only the title, tabs and filter buttons are design-confirmed here; the real report columns come from Branko's PRD.</t>
+        </is>
+      </c>
+      <c r="H99" s="2" t="inlineStr">
+        <is>
+          <t>Filters (Epic key TBD); Figma 11903-10573 (Reports filters); design-notes.md §B.6 #13</t>
+        </is>
+      </c>
+      <c r="I99" s="2" t="inlineStr"/>
+      <c r="J99" s="2" t="inlineStr"/>
+    </row>
+    <row r="100">
+      <c r="A100" s="2" t="inlineStr">
+        <is>
+          <t>A/R Aging Collection shows Customer, Date, Location, Transaction Type</t>
+        </is>
+      </c>
+      <c r="B100" s="2" t="inlineStr">
+        <is>
+          <t>Reports Page Filters</t>
+        </is>
+      </c>
+      <c r="C100" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D100" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E100" s="2" t="inlineStr">
+        <is>
+          <t>1. You are signed in to the ShopView App on a desktop browser.
+2. You are on the Reports area of the app with some sample data present.</t>
+        </is>
+      </c>
+      <c r="F100" s="2" t="inlineStr">
+        <is>
+          <t>1. Open the Reports area and go to the A/R Aging Collection report.
+2. Look at the filter buttons shown above the report table.</t>
+        </is>
+      </c>
+      <c r="G100" s="2" t="inlineStr">
+        <is>
+          <t>1. The A/R Aging Collection report shows four filter buttons: Customer, Date, Location and Transaction Type.
+2. A print icon is shown in the toolbar.
+2. Note: in the design the report body uses a sample placeholder table, so only the title, tabs and filter buttons are design-confirmed here; the real report columns come from Branko's PRD.</t>
+        </is>
+      </c>
+      <c r="H100" s="2" t="inlineStr">
+        <is>
+          <t>Filters (Epic key TBD); Figma 11903-10573 (Reports filters); design-notes.md §B.6 #14</t>
+        </is>
+      </c>
+      <c r="I100" s="2" t="inlineStr"/>
+      <c r="J100" s="2" t="inlineStr"/>
+    </row>
+    <row r="101">
+      <c r="A101" s="2" t="inlineStr">
+        <is>
+          <t>A/P Aging Summary report shows Vendor and Date filters</t>
+        </is>
+      </c>
+      <c r="B101" s="2" t="inlineStr">
+        <is>
+          <t>Reports Page Filters</t>
+        </is>
+      </c>
+      <c r="C101" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D101" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E101" s="2" t="inlineStr">
+        <is>
+          <t>1. You are signed in to the ShopView App on a desktop browser.
+2. You are on the Reports area of the app with some sample data present.</t>
+        </is>
+      </c>
+      <c r="F101" s="2" t="inlineStr">
+        <is>
+          <t>1. Open the Reports area and go to the A/P Aging Summary report.
+2. Look at the filter buttons shown above the report table.</t>
+        </is>
+      </c>
+      <c r="G101" s="2" t="inlineStr">
+        <is>
+          <t>1. The A/P Aging Summary report shows two filter buttons: Vendor and Date.
+2. A print icon is shown in the toolbar.
+2. Note: in the design the report body uses a sample placeholder table, so only the title, tabs and filter buttons are design-confirmed here; the real report columns come from Branko's PRD.</t>
+        </is>
+      </c>
+      <c r="H101" s="2" t="inlineStr">
+        <is>
+          <t>Filters (Epic key TBD); Figma 11903-10573 (Reports filters); design-notes.md §B.6 #15</t>
+        </is>
+      </c>
+      <c r="I101" s="2" t="inlineStr"/>
+      <c r="J101" s="2" t="inlineStr"/>
+    </row>
+    <row r="102">
+      <c r="A102" s="2" t="inlineStr">
+        <is>
+          <t>A/P Aging Detail shows Vendor, Date, Location, Transaction Type filters</t>
+        </is>
+      </c>
+      <c r="B102" s="2" t="inlineStr">
+        <is>
+          <t>Reports Page Filters</t>
+        </is>
+      </c>
+      <c r="C102" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D102" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E102" s="2" t="inlineStr">
+        <is>
+          <t>1. You are signed in to the ShopView App on a desktop browser.
+2. You are on the Reports area of the app with some sample data present.</t>
+        </is>
+      </c>
+      <c r="F102" s="2" t="inlineStr">
+        <is>
+          <t>1. Open the Reports area and go to the A/P Aging Detail report.
+2. Look at the filter buttons shown above the report table.</t>
+        </is>
+      </c>
+      <c r="G102" s="2" t="inlineStr">
+        <is>
+          <t>1. The A/P Aging Detail report shows four filter buttons: Vendor, Date, Location and Transaction Type.
+2. A print icon is shown in the toolbar.
+2. Note: in the design the report body uses a sample placeholder table, so only the title, tabs and filter buttons are design-confirmed here; the real report columns come from Branko's PRD.</t>
+        </is>
+      </c>
+      <c r="H102" s="2" t="inlineStr">
+        <is>
+          <t>Filters (Epic key TBD); Figma 11903-10573 (Reports filters); design-notes.md §B.6 #16</t>
+        </is>
+      </c>
+      <c r="I102" s="2" t="inlineStr"/>
+      <c r="J102" s="2" t="inlineStr"/>
+    </row>
+    <row r="103">
+      <c r="A103" s="2" t="inlineStr">
+        <is>
+          <t>A/P Unpaid Invoices shows Vendor, Date, Location, Transaction Type filters</t>
+        </is>
+      </c>
+      <c r="B103" s="2" t="inlineStr">
+        <is>
+          <t>Reports Page Filters</t>
+        </is>
+      </c>
+      <c r="C103" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D103" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E103" s="2" t="inlineStr">
+        <is>
+          <t>1. You are signed in to the ShopView App on a desktop browser.
+2. You are on the Reports area of the app with some sample data present.</t>
+        </is>
+      </c>
+      <c r="F103" s="2" t="inlineStr">
+        <is>
+          <t>1. Open the Reports area and go to the A/P Unpaid Invoices report.
+2. Look at the filter buttons shown above the report table.</t>
+        </is>
+      </c>
+      <c r="G103" s="2" t="inlineStr">
+        <is>
+          <t>1. The A/P Unpaid Invoices report shows four filter buttons: Vendor, Date, Location and Transaction Type.
+2. A print icon is shown in the toolbar.
+2. Note: in the design the report body uses a sample placeholder table, so only the title, tabs and filter buttons are design-confirmed here; the real report columns come from Branko's PRD.</t>
+        </is>
+      </c>
+      <c r="H103" s="2" t="inlineStr">
+        <is>
+          <t>Filters (Epic key TBD); Figma 11903-10573 (Reports filters); design-notes.md §B.6 #17</t>
+        </is>
+      </c>
+      <c r="I103" s="2" t="inlineStr"/>
+      <c r="J103" s="2" t="inlineStr"/>
+    </row>
+    <row r="104">
+      <c r="A104" s="2" t="inlineStr">
+        <is>
+          <t>Notes report shows Author, Date and Mention filters</t>
+        </is>
+      </c>
+      <c r="B104" s="2" t="inlineStr">
+        <is>
+          <t>Reports Page Filters</t>
+        </is>
+      </c>
+      <c r="C104" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D104" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E104" s="2" t="inlineStr">
+        <is>
+          <t>1. You are signed in to the ShopView App on a desktop browser.
+2. You are on the Reports area of the app with some sample data present.</t>
+        </is>
+      </c>
+      <c r="F104" s="2" t="inlineStr">
+        <is>
+          <t>1. Open the Reports area and go to the Notes report.
+2. Look at the filter buttons shown above the report table.</t>
+        </is>
+      </c>
+      <c r="G104" s="2" t="inlineStr">
+        <is>
+          <t>1. The Notes report shows three filter buttons: Author, Date and Mention (the Mention button uses an @ icon).
+2. The toolbar also shows a search icon, a filter icon and a sort icon.
+3. Mention is a new filter type not on the Work Orders page — Behaviour to confirm — pending Branko's product write-up; to be checked live once the feature is available.</t>
+        </is>
+      </c>
+      <c r="H104" s="2" t="inlineStr">
+        <is>
+          <t>Filters (Epic key TBD); Figma 11903-10573 (Reports filters); design-notes.md §B.6 #18</t>
+        </is>
+      </c>
+      <c r="I104" s="2" t="inlineStr"/>
+      <c r="J104" s="2" t="inlineStr"/>
+    </row>
+    <row r="105">
+      <c r="A105" s="2" t="inlineStr">
+        <is>
+          <t>Reminders report shows only a Date filter</t>
+        </is>
+      </c>
+      <c r="B105" s="2" t="inlineStr">
+        <is>
+          <t>Reports Page Filters</t>
+        </is>
+      </c>
+      <c r="C105" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D105" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E105" s="2" t="inlineStr">
+        <is>
+          <t>1. You are signed in to the ShopView App on a desktop browser.
+2. You are on the Reports area of the app with some sample data present.</t>
+        </is>
+      </c>
+      <c r="F105" s="2" t="inlineStr">
+        <is>
+          <t>1. Open the Reports area and go to the Reminders report.
+2. Look at the filter buttons shown above the report table.</t>
+        </is>
+      </c>
+      <c r="G105" s="2" t="inlineStr">
+        <is>
+          <t>1. The Reminders report shows a single filter button: Date.
+2. When no reminders match, the report shows the message 'There are no reminders for selected date range'.</t>
+        </is>
+      </c>
+      <c r="H105" s="2" t="inlineStr">
+        <is>
+          <t>Filters (Epic key TBD); Figma 11903-10573 (Reports filters); design-notes.md §B.6 #19</t>
+        </is>
+      </c>
+      <c r="I105" s="2" t="inlineStr"/>
+      <c r="J105" s="2" t="inlineStr"/>
+    </row>
+    <row r="106">
+      <c r="A106" s="2" t="inlineStr">
+        <is>
+          <t>IBS Batch Transactions report shows Customer, Date and Status filters</t>
+        </is>
+      </c>
+      <c r="B106" s="2" t="inlineStr">
+        <is>
+          <t>Reports Page Filters</t>
+        </is>
+      </c>
+      <c r="C106" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D106" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E106" s="2" t="inlineStr">
+        <is>
+          <t>1. You are signed in to the ShopView App on a desktop browser.
+2. You are on the Reports area of the app with some sample data present.</t>
+        </is>
+      </c>
+      <c r="F106" s="2" t="inlineStr">
+        <is>
+          <t>1. Open the Reports area and go to the IBS Batch Transactions report.
+2. Look at the filter buttons shown above the report table.</t>
+        </is>
+      </c>
+      <c r="G106" s="2" t="inlineStr">
+        <is>
+          <t>1. The IBS Batch Transactions report shows three filter buttons: Customer, Date and Status.
+2. The report has three view tabs: Ready To Send, Sent and Payments.
+3. The table shows columns: (checkbox), Date, Type, No., Customer, Total, Balance and Status.</t>
+        </is>
+      </c>
+      <c r="H106" s="2" t="inlineStr">
+        <is>
+          <t>Filters (Epic key TBD); Figma 11903-10573 (Reports filters); design-notes.md §B.6 #20</t>
+        </is>
+      </c>
+      <c r="I106" s="2" t="inlineStr"/>
+      <c r="J106" s="2" t="inlineStr"/>
+    </row>
+    <row r="107">
+      <c r="A107" s="2" t="inlineStr">
+        <is>
+          <t>QB Unexported report filters change per tab (Customer / Vendor / User)</t>
+        </is>
+      </c>
+      <c r="B107" s="2" t="inlineStr">
+        <is>
+          <t>Reports Page Filters</t>
+        </is>
+      </c>
+      <c r="C107" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D107" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E107" s="2" t="inlineStr">
+        <is>
+          <t>1. You are signed in to the ShopView App on a desktop browser.
+2. You are on the Reports area of the app with some sample data present.</t>
+        </is>
+      </c>
+      <c r="F107" s="2" t="inlineStr">
+        <is>
+          <t>1. Open the Reports area and go to the QB Unexported report.
+2. Look at the filter buttons shown above the report table.</t>
+        </is>
+      </c>
+      <c r="G107" s="2" t="inlineStr">
+        <is>
+          <t>1. The QB Unexported report has three view tabs, and the first filter button changes per tab.
+2. On the Customers tab the filter buttons are Customer, Date and Type.
+3. On the Vendors tab they are Vendor, Date and Type.
+4. On the Journal Entries tab they are User, Date and Type.
+5. Behaviour to confirm — pending Branko's product write-up; to be checked live once the feature is available. (option lists behind each button).</t>
+        </is>
+      </c>
+      <c r="H107" s="2" t="inlineStr">
+        <is>
+          <t>Filters (Epic key TBD); Figma 11903-10573 (Reports filters); design-notes.md §B.6 #21, #22, #23</t>
+        </is>
+      </c>
+      <c r="I107" s="2" t="inlineStr"/>
+      <c r="J107" s="2" t="inlineStr"/>
+    </row>
+    <row r="108">
+      <c r="A108" s="2" t="inlineStr">
+        <is>
+          <t>Choosing a Reports filter narrows the report results</t>
+        </is>
+      </c>
+      <c r="B108" s="2" t="inlineStr">
+        <is>
+          <t>Reports Page Filters</t>
+        </is>
+      </c>
+      <c r="C108" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D108" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E108" s="2" t="inlineStr">
+        <is>
+          <t>1. You are signed in to the ShopView App on a desktop browser.
+2. You are on the Reports area of the app with some sample data present.</t>
+        </is>
+      </c>
+      <c r="F108" s="2" t="inlineStr">
+        <is>
+          <t>1. Open the Reports area and go to the any (for example Sales) report.
+2. Look at the filter buttons shown above the report table.</t>
+        </is>
+      </c>
+      <c r="G108" s="2" t="inlineStr">
+        <is>
+          <t>1. The report updates to show only the rows matching the chosen filter value, and the chosen value is shown on the filter button.
+2. Behaviour to confirm — pending Branko's product write-up; to be checked live once the feature is available. (exactly which filters apply on each report, the full option lists, and whether results update immediately).</t>
+        </is>
+      </c>
+      <c r="H108" s="2" t="inlineStr">
+        <is>
+          <t>Filters (Epic key TBD); Figma 11903-10573 (Reports filters); design-notes.md §B.6</t>
+        </is>
+      </c>
+      <c r="I108" s="2" t="inlineStr"/>
+      <c r="J108" s="2" t="inlineStr"/>
+    </row>
+    <row r="109">
+      <c r="A109" s="2" t="inlineStr">
+        <is>
+          <t>New Reports filter types behave correctly (Location, Transaction Type, etc.)</t>
+        </is>
+      </c>
+      <c r="B109" s="2" t="inlineStr">
+        <is>
+          <t>Reports Page Filters</t>
+        </is>
+      </c>
+      <c r="C109" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D109" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E109" s="2" t="inlineStr">
+        <is>
+          <t>1. You are signed in to the ShopView App on a desktop browser.
+2. You are on the Reports area of the app with some sample data present.</t>
+        </is>
+      </c>
+      <c r="F109" s="2" t="inlineStr">
+        <is>
+          <t>1. Open the Reports area and go to the reports that use them (for example A/R Aging Detail, Notes) report.
+2. Look at the filter buttons shown above the report table.</t>
+        </is>
+      </c>
+      <c r="G109" s="2" t="inlineStr">
+        <is>
+          <t>1. Each new filter type (Location, Transaction Type, Invoice Status, Type, User, Mention) opens a list of choices and filters the report by the choice.
+2. Behaviour to confirm — pending Branko's product write-up; to be checked live once the feature is available. (the exact choices, single- vs multi-select, and how each new filter type filters the report).</t>
+        </is>
+      </c>
+      <c r="H109" s="2" t="inlineStr">
+        <is>
+          <t>Filters (Epic key TBD); Figma 11903-10573 (Reports filters); design-notes.md §B.6</t>
+        </is>
+      </c>
+      <c r="I109" s="2" t="inlineStr"/>
+      <c r="J109" s="2" t="inlineStr"/>
+    </row>
+    <row r="110">
+      <c r="A110" s="2" t="inlineStr">
+        <is>
+          <t>Page search opens with the 'Search or ask a question' box</t>
+        </is>
+      </c>
+      <c r="B110" s="2" t="inlineStr">
+        <is>
+          <t>Page Search (Command-K)</t>
+        </is>
+      </c>
+      <c r="C110" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D110" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E110" s="2" t="inlineStr">
+        <is>
+          <t>1. You are signed in to the ShopView App on a desktop browser.
+2. Some sample work orders, customers, assets, parts and vendors exist.</t>
+        </is>
+      </c>
+      <c r="F110" s="2" t="inlineStr">
+        <is>
+          <t>1. From anywhere in the app, open the page search (the Search box in the top bar, or press Command-K / Ctrl-K).
+2. Look at the search panel that opens.</t>
+        </is>
+      </c>
+      <c r="G110" s="2" t="inlineStr">
+        <is>
+          <t>1. A search panel opens with an empty search box at the top.
+2. The box shows the placeholder text 'Search or ask a question' with a magnifier icon on the left and a clear (X) button on the right.
+3. Behaviour to confirm — pending Branko's product write-up; to be checked live once the feature is available. (whether 'ask a question' means an AI search — this is out of scope for now).</t>
+        </is>
+      </c>
+      <c r="H110" s="2" t="inlineStr">
+        <is>
+          <t>Filters (Epic key TBD); Figma 11829-8908 (page-search component); design-2026-07-27/DESIGN-INGEST-2026-07-27.md §1/§3.D</t>
+        </is>
+      </c>
+      <c r="I110" s="2" t="inlineStr"/>
+      <c r="J110" s="2" t="inlineStr"/>
+    </row>
+    <row r="111">
+      <c r="A111" s="2" t="inlineStr">
+        <is>
+          <t>Page search shows entity tabs All, Work Orders, Customers, Assets, Parts...</t>
+        </is>
+      </c>
+      <c r="B111" s="2" t="inlineStr">
+        <is>
+          <t>Page Search (Command-K)</t>
+        </is>
+      </c>
+      <c r="C111" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D111" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E111" s="2" t="inlineStr">
+        <is>
+          <t>1. You are signed in to the ShopView App on a desktop browser.
+2. Some sample work orders, customers, assets, parts and vendors exist.</t>
+        </is>
+      </c>
+      <c r="F111" s="2" t="inlineStr">
+        <is>
+          <t>1. Open the page search panel.
+2. Look at the row of tabs under the search box.</t>
+        </is>
+      </c>
+      <c r="G111" s="2" t="inlineStr">
+        <is>
+          <t>1. A row of tabs is shown: All, Work Orders, Customers, Assets, Parts, Vendors and Part Sales.
+2. The All tab is selected by default.
+3. Behaviour to confirm — pending Branko's product write-up; to be checked live once the feature is available. (whether choosing a tab limits results to that type only).</t>
+        </is>
+      </c>
+      <c r="H111" s="2" t="inlineStr">
+        <is>
+          <t>Filters (Epic key TBD); Figma 11829-8908 (page-search component); design-2026-07-27/DESIGN-INGEST-2026-07-27.md §1/§3.D</t>
+        </is>
+      </c>
+      <c r="I111" s="2" t="inlineStr"/>
+      <c r="J111" s="2" t="inlineStr"/>
+    </row>
+    <row r="112">
+      <c r="A112" s="2" t="inlineStr">
+        <is>
+          <t>Typing a term shows grouped results with counts and highlighting</t>
+        </is>
+      </c>
+      <c r="B112" s="2" t="inlineStr">
+        <is>
+          <t>Page Search (Command-K)</t>
+        </is>
+      </c>
+      <c r="C112" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D112" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E112" s="2" t="inlineStr">
+        <is>
+          <t>1. You are signed in to the ShopView App on a desktop browser.
+2. Some sample work orders, customers, assets, parts and vendors exist.</t>
+        </is>
+      </c>
+      <c r="F112" s="2" t="inlineStr">
+        <is>
+          <t>1. Open the page search panel.
+2. Type a few letters (for example 'Fib') into the search box.
+3. Look at the results.</t>
+        </is>
+      </c>
+      <c r="G112" s="2" t="inlineStr">
+        <is>
+          <t>1. Results are grouped by type with a count next to each group heading, for example 'Work orders (2)', 'Customers (2)', 'Vendors (1)', 'Assets (2)', 'Parts (1)'.
+2. The matching part of each result is highlighted in yellow.
+3. Each work order row shows its number, name, a status pill (for example Approved or Estimate), the person and a date.
+4. Behaviour to confirm — pending Branko's product write-up; to be checked live once the feature is available. (how matching works — exact vs fuzzy — and the ranking order).</t>
+        </is>
+      </c>
+      <c r="H112" s="2" t="inlineStr">
+        <is>
+          <t>Filters (Epic key TBD); Figma 11829-8908 (page-search component); design-2026-07-27/DESIGN-INGEST-2026-07-27.md §1/§3.D</t>
+        </is>
+      </c>
+      <c r="I112" s="2" t="inlineStr"/>
+      <c r="J112" s="2" t="inlineStr"/>
+    </row>
+    <row r="113">
+      <c r="A113" s="2" t="inlineStr">
+        <is>
+          <t>Recent searches are shown grouped by Today, Yesterday, Past week...</t>
+        </is>
+      </c>
+      <c r="B113" s="2" t="inlineStr">
+        <is>
+          <t>Page Search (Command-K)</t>
+        </is>
+      </c>
+      <c r="C113" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D113" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E113" s="2" t="inlineStr">
+        <is>
+          <t>1. You are signed in to the ShopView App on a desktop browser.
+2. Some sample work orders, customers, assets, parts and vendors exist.</t>
+        </is>
+      </c>
+      <c r="F113" s="2" t="inlineStr">
+        <is>
+          <t>1. Open the page search panel without typing anything.
+2. Look at the list shown under the tabs.</t>
+        </is>
+      </c>
+      <c r="G113" s="2" t="inlineStr">
+        <is>
+          <t>1. A list of recent items is shown, grouped under headings: Today, Yesterday, Past week and Past 30 days.
+2. Each item shows a type icon, its name and a short detail line (for example a customer address or a date).
+3. Behaviour to confirm — pending Branko's product write-up; to be checked live once the feature is available. (how many recent items are kept and how long they persist).</t>
+        </is>
+      </c>
+      <c r="H113" s="2" t="inlineStr">
+        <is>
+          <t>Filters (Epic key TBD); Figma 11829-8908 (page-search component); design-2026-07-27/DESIGN-INGEST-2026-07-27.md §1/§3.D</t>
+        </is>
+      </c>
+      <c r="I113" s="2" t="inlineStr"/>
+      <c r="J113" s="2" t="inlineStr"/>
+    </row>
+    <row r="114">
+      <c r="A114" s="2" t="inlineStr">
+        <is>
+          <t>Re-opening page search keeps the last typed text and its results</t>
+        </is>
+      </c>
+      <c r="B114" s="2" t="inlineStr">
+        <is>
+          <t>Page Search (Command-K)</t>
+        </is>
+      </c>
+      <c r="C114" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D114" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E114" s="2" t="inlineStr">
+        <is>
+          <t>1. You are signed in to the ShopView App on a desktop browser.
+2. Some sample work orders, customers, assets, parts and vendors exist.</t>
+        </is>
+      </c>
+      <c r="F114" s="2" t="inlineStr">
+        <is>
+          <t>1. Open the page search and type a term (for example 'Fibridge').
+2. Close the panel, then open it again.
+3. Look at the search box and the results.</t>
+        </is>
+      </c>
+      <c r="G114" s="2" t="inlineStr">
+        <is>
+          <t>1. The previous search text is still in the box (shown selected/highlighted) and its results are shown.
+2. Behaviour to confirm — pending Branko's product write-up; to be checked live once the feature is available. (whether the last search is remembered per person and for how long — this is the 'persisting search' state).</t>
+        </is>
+      </c>
+      <c r="H114" s="2" t="inlineStr">
+        <is>
+          <t>Filters (Epic key TBD); Figma 11829-8908 (page-search component); design-2026-07-27/DESIGN-INGEST-2026-07-27.md §1/§3.D</t>
+        </is>
+      </c>
+      <c r="I114" s="2" t="inlineStr"/>
+      <c r="J114" s="2" t="inlineStr"/>
+    </row>
+    <row r="115">
+      <c r="A115" s="2" t="inlineStr">
+        <is>
+          <t>Hovering a search result shows quick-action buttons</t>
+        </is>
+      </c>
+      <c r="B115" s="2" t="inlineStr">
+        <is>
+          <t>Page Search (Command-K)</t>
+        </is>
+      </c>
+      <c r="C115" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D115" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E115" s="2" t="inlineStr">
+        <is>
+          <t>1. You are signed in to the ShopView App on a desktop browser.
+2. Some sample work orders, customers, assets, parts and vendors exist.</t>
+        </is>
+      </c>
+      <c r="F115" s="2" t="inlineStr">
+        <is>
+          <t>1. Open the page search panel (recent items or results shown).
+2. Move the mouse over a result row.
+3. Look at the right side of that row.</t>
+        </is>
+      </c>
+      <c r="G115" s="2" t="inlineStr">
+        <is>
+          <t>1. Quick-action buttons appear on the row, depending on the result type — for example 'Add new line' on a work order, 'New work order' on an asset or customer, 'Add part' on a part sale, 'Add contact' on a vendor and 'Add to work order' on a part.
+2. Behaviour to confirm — pending Branko's product write-up; to be checked live once the feature is available. (exactly which quick actions show for which result type, and what each one does).</t>
+        </is>
+      </c>
+      <c r="H115" s="2" t="inlineStr">
+        <is>
+          <t>Filters (Epic key TBD); Figma 11829-8908 (page-search component); design-2026-07-27/DESIGN-INGEST-2026-07-27.md §1/§3.D</t>
+        </is>
+      </c>
+      <c r="I115" s="2" t="inlineStr"/>
+      <c r="J115" s="2" t="inlineStr"/>
+    </row>
+    <row r="116">
+      <c r="A116" s="2" t="inlineStr">
+        <is>
+          <t>Page search shows keyboard hints and supports keyboard navigation</t>
+        </is>
+      </c>
+      <c r="B116" s="2" t="inlineStr">
+        <is>
+          <t>Page Search (Command-K)</t>
+        </is>
+      </c>
+      <c r="C116" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D116" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E116" s="2" t="inlineStr">
+        <is>
+          <t>1. You are signed in to the ShopView App on a desktop browser.
+2. Some sample work orders, customers, assets, parts and vendors exist.</t>
+        </is>
+      </c>
+      <c r="F116" s="2" t="inlineStr">
+        <is>
+          <t>1. Open the page search panel.
+2. Look at the bar along the bottom of the panel.
+3. Use the up/down arrow keys, Enter and Esc.</t>
+        </is>
+      </c>
+      <c r="G116" s="2" t="inlineStr">
+        <is>
+          <t>1. The bottom bar shows keyboard hints: up/down arrows labelled 'Navigate', the Enter key labelled 'Select', and 'Close esc'.
+2. Arrow keys move the highlight between results, Enter opens the highlighted result, and Esc closes the panel (to be checked live once available).
+3. Behaviour to confirm — pending Branko's product write-up; to be checked live once the feature is available. (exact keyboard behaviour).</t>
+        </is>
+      </c>
+      <c r="H116" s="2" t="inlineStr">
+        <is>
+          <t>Filters (Epic key TBD); Figma 11829-8908 (page-search component); design-2026-07-27/DESIGN-INGEST-2026-07-27.md §1/§3.D</t>
+        </is>
+      </c>
+      <c r="I116" s="2" t="inlineStr"/>
+      <c r="J116" s="2" t="inlineStr"/>
+    </row>
+    <row r="117">
+      <c r="A117" s="2" t="inlineStr">
+        <is>
+          <t>Page search results include a Refresh action</t>
+        </is>
+      </c>
+      <c r="B117" s="2" t="inlineStr">
+        <is>
+          <t>Page Search (Command-K)</t>
+        </is>
+      </c>
+      <c r="C117" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D117" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E117" s="2" t="inlineStr">
+        <is>
+          <t>1. You are signed in to the ShopView App on a desktop browser.
+2. Some sample work orders, customers, assets, parts and vendors exist.</t>
+        </is>
+      </c>
+      <c r="F117" s="2" t="inlineStr">
+        <is>
+          <t>1. Open the page search and type a term so grouped results appear.
+2. Look at the top right of the results area.</t>
+        </is>
+      </c>
+      <c r="G117" s="2" t="inlineStr">
+        <is>
+          <t>1. A 'Refresh' link is shown at the top right of the results.
+2. Behaviour to confirm — pending Branko's product write-up; to be checked live once the feature is available. (what Refresh reloads and when it is shown).</t>
+        </is>
+      </c>
+      <c r="H117" s="2" t="inlineStr">
+        <is>
+          <t>Filters (Epic key TBD); Figma 11829-8908 (page-search component); design-2026-07-27/DESIGN-INGEST-2026-07-27.md §1/§3.D</t>
+        </is>
+      </c>
+      <c r="I117" s="2" t="inlineStr"/>
+      <c r="J117" s="2" t="inlineStr"/>
+    </row>
+    <row r="118">
+      <c r="A118" s="2" t="inlineStr">
+        <is>
+          <t>Page search scope belongs to Filters or Global Search (to decide)</t>
+        </is>
+      </c>
+      <c r="B118" s="2" t="inlineStr">
+        <is>
+          <t>Page Search (Command-K)</t>
+        </is>
+      </c>
+      <c r="C118" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D118" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E118" s="2" t="inlineStr">
+        <is>
+          <t>1. You are signed in to the ShopView App on a desktop browser.
+2. Some sample work orders, customers, assets, parts and vendors exist.</t>
+        </is>
+      </c>
+      <c r="F118" s="2" t="inlineStr">
+        <is>
+          <t>1. Review where the page search / Command-K component is owned for testing.
+2. Compare against the Global Search project's existing cases.</t>
+        </is>
+      </c>
+      <c r="G118" s="2" t="inlineStr">
+        <is>
+          <t>1. The page-search component is agreed to belong to either the Filters test suite or the Global Search test suite, not both.
+2. Behaviour to confirm — pending Branko's product write-up; to be checked live once the feature is available. (product/QA decision on which project owns page search).</t>
+        </is>
+      </c>
+      <c r="H118" s="2" t="inlineStr">
+        <is>
+          <t>Filters (Epic key TBD); Figma 11829-8908 (page-search component); design-2026-07-27/DESIGN-INGEST-2026-07-27.md §1/§3.D</t>
+        </is>
+      </c>
+      <c r="I118" s="2" t="inlineStr"/>
+      <c r="J118" s="2" t="inlineStr"/>
+    </row>
+    <row r="119">
+      <c r="A119" s="2" t="inlineStr">
+        <is>
           <t>The work order list request carries the active filter selections</t>
         </is>
       </c>
-      <c r="B76" s="2" t="inlineStr">
+      <c r="B119" s="2" t="inlineStr">
         <is>
           <t>API — Work Orders List Filtering</t>
         </is>
       </c>
-      <c r="C76" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D76" s="2" t="inlineStr">
+      <c r="C119" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D119" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E76" s="2" t="inlineStr">
+      <c r="E119" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in to the ShopView App on a desktop browser with developer tools open on the Network tab.
 2. You are on the Work Orders page with no filters applied.</t>
         </is>
       </c>
-      <c r="F76" s="2" t="inlineStr">
+      <c r="F119" s="2" t="inlineStr">
         <is>
           <t>1. Apply a Status selection and a Customer selection in the filter bar.
 2. In the Network tab, find the work order list request the page sends after the change.
 3. Inspect the request's parameters.</t>
         </is>
       </c>
-      <c r="G76" s="2" t="inlineStr">
+      <c r="G119" s="2" t="inlineStr">
         <is>
           <t>1. The list request includes the active filter selections as request parameters (status values and customer identifiers).
 2. The request succeeds (HTTP 200).
 3. The response contains only work orders matching the filters - the filtering is done by the backend, not just hidden client-side.</t>
         </is>
       </c>
-      <c r="H76" s="2" t="inlineStr">
+      <c r="H119" s="2" t="inlineStr">
         <is>
           <t>requirements.md Story 2 S2-R2; Story 3 S3-R6 (backend view)</t>
         </is>
       </c>
-      <c r="I76" s="2" t="inlineStr"/>
-      <c r="J76" s="2" t="inlineStr"/>
-    </row>
-    <row r="77">
-      <c r="A77" s="2" t="inlineStr">
+      <c r="I119" s="2" t="inlineStr"/>
+      <c r="J119" s="2" t="inlineStr"/>
+    </row>
+    <row r="120">
+      <c r="A120" s="2" t="inlineStr">
         <is>
           <t>A combined multi-filter request returns only work orders matching all filters, any value within each filter</t>
         </is>
       </c>
-      <c r="B77" s="2" t="inlineStr">
+      <c r="B120" s="2" t="inlineStr">
         <is>
           <t>API — Work Orders List Filtering</t>
         </is>
       </c>
-      <c r="C77" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D77" s="2" t="inlineStr">
+      <c r="C120" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D120" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E77" s="2" t="inlineStr">
+      <c r="E120" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in with developer tools open on the Network tab.
 2. Seeded ZZAUTOTEST work orders exist: customer A with an Estimate and an Approved work order, customer B with an Estimate work order.</t>
         </is>
       </c>
-      <c r="F77" s="2" t="inlineStr">
+      <c r="F120" s="2" t="inlineStr">
         <is>
           <t>1. On the Work Orders page apply Status = Estimate + Approved and Customer = customer A.
 2. Capture the resulting list request and response.</t>
         </is>
       </c>
-      <c r="G77" s="2" t="inlineStr">
+      <c r="G120" s="2" t="inlineStr">
         <is>
           <t>1. One request carries both filters together (both statuses and the customer).
 2. The response returns customer A's Estimate and Approved work orders only.
 3. Customer B's work orders are absent - the customer filter and status filter both restrict the result, while the two statuses combine as either-or.</t>
         </is>
       </c>
-      <c r="H77" s="2" t="inlineStr">
+      <c r="H120" s="2" t="inlineStr">
         <is>
           <t>requirements.md Story 2 S2-R2; Story 3 S3-R6; Story 8 S8-R3 (backend view)</t>
         </is>
       </c>
-      <c r="I77" s="2" t="inlineStr"/>
-      <c r="J77" s="2" t="inlineStr"/>
-    </row>
-    <row r="78">
-      <c r="A78" s="2" t="inlineStr">
+      <c r="I120" s="2" t="inlineStr"/>
+      <c r="J120" s="2" t="inlineStr"/>
+    </row>
+    <row r="121">
+      <c r="A121" s="2" t="inlineStr">
         <is>
           <t>A list request with a deleted or unknown filter value is handled without a server error</t>
         </is>
       </c>
-      <c r="B78" s="2" t="inlineStr">
+      <c r="B121" s="2" t="inlineStr">
         <is>
           <t>API — Work Orders List Filtering</t>
         </is>
       </c>
-      <c r="C78" s="2" t="inlineStr">
+      <c r="C121" s="2" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="D78" s="2" t="inlineStr">
+      <c r="D121" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E78" s="2" t="inlineStr">
+      <c r="E121" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in and can replay/edit the work order list request (developer tools or an API client).
 2. You have a captured filtered list request, and one of its filter values has since been deleted (for example a removed ZZAUTOTEST customer) or is a made-up identifier.</t>
         </is>
       </c>
-      <c r="F78" s="2" t="inlineStr">
+      <c r="F121" s="2" t="inlineStr">
         <is>
           <t>1. Send the list request containing the no-longer-existing (or made-up) filter value.
 2. Inspect the HTTP status and the response body.</t>
         </is>
       </c>
-      <c r="G78" s="2" t="inlineStr">
+      <c r="G121" s="2" t="inlineStr">
         <is>
           <t>1. The backend does not fail with a server error (no HTTP 5xx).
 2. The response is a normal, successful list response - the invalid value is ignored or simply matches nothing.
 3. Any still-valid filter values in the same request are applied normally.</t>
         </is>
       </c>
-      <c r="H78" s="2" t="inlineStr">
+      <c r="H121" s="2" t="inlineStr">
         <is>
           <t>requirements.md Story 10 S10-N1; Story 11 S11-R3</t>
         </is>
       </c>
-      <c r="I78" s="2" t="inlineStr"/>
-      <c r="J78" s="2" t="inlineStr"/>
-    </row>
-    <row r="79">
-      <c r="A79" s="2" t="inlineStr">
+      <c r="I121" s="2" t="inlineStr"/>
+      <c r="J121" s="2" t="inlineStr"/>
+    </row>
+    <row r="122">
+      <c r="A122" s="2" t="inlineStr">
         <is>
           <t>A list request with malformed filter parameters does not produce a server error</t>
         </is>
       </c>
-      <c r="B79" s="2" t="inlineStr">
+      <c r="B122" s="2" t="inlineStr">
         <is>
           <t>API — Work Orders List Filtering</t>
         </is>
       </c>
-      <c r="C79" s="2" t="inlineStr">
+      <c r="C122" s="2" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="D79" s="2" t="inlineStr">
+      <c r="D122" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E79" s="2" t="inlineStr">
+      <c r="E122" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in and can replay/edit the work order list request.
 2. You have a captured filtered list request to tamper with.</t>
         </is>
       </c>
-      <c r="F79" s="2" t="inlineStr">
+      <c r="F122" s="2" t="inlineStr">
         <is>
           <t>1. Corrupt the filter parameters (wrong types, scrambled values, nonsense text) and send the request.
 2. Inspect the HTTP status and the response body.
 3. Also open the equally malformed page URL in the browser and watch the page.</t>
         </is>
       </c>
-      <c r="G79" s="2" t="inlineStr">
+      <c r="G122" s="2" t="inlineStr">
         <is>
           <t>1. The backend responds gracefully - no HTTP 5xx / crash; either a normal (unfiltered or empty) list or a clean validation response.
 2. In the browser the page still loads without filters and without an error message, matching the malformed-URL requirement.</t>
         </is>
       </c>
-      <c r="H79" s="2" t="inlineStr">
+      <c r="H122" s="2" t="inlineStr">
         <is>
           <t>requirements.md Story 11 S11-N1</t>
         </is>
       </c>
-      <c r="I79" s="2" t="inlineStr"/>
-      <c r="J79" s="2" t="inlineStr"/>
-    </row>
-    <row r="80">
-      <c r="A80" s="2" t="inlineStr">
+      <c r="I122" s="2" t="inlineStr"/>
+      <c r="J122" s="2" t="inlineStr"/>
+    </row>
+    <row r="123">
+      <c r="A123" s="2" t="inlineStr">
         <is>
           <t>A filter combination matching nothing returns a successful empty list, not an error</t>
         </is>
       </c>
-      <c r="B80" s="2" t="inlineStr">
+      <c r="B123" s="2" t="inlineStr">
         <is>
           <t>API — Work Orders List Filtering</t>
         </is>
       </c>
-      <c r="C80" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D80" s="2" t="inlineStr">
+      <c r="C123" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D123" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E80" s="2" t="inlineStr">
+      <c r="E123" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in with developer tools open on the Network tab.
 2. A filter combination is known to match no work orders (for example a seeded customer plus a status they never have).</t>
         </is>
       </c>
-      <c r="F80" s="2" t="inlineStr">
+      <c r="F123" s="2" t="inlineStr">
         <is>
           <t>1. Apply that filter combination on the Work Orders page.
 2. Capture the list request and response.</t>
         </is>
       </c>
-      <c r="G80" s="2" t="inlineStr">
+      <c r="G123" s="2" t="inlineStr">
         <is>
           <t>1. The request succeeds (HTTP 200).
 2. The response contains an empty result set (zero work orders) - an empty match is a normal outcome, not an error.
 3. The page renders the no-results empty state from this response.</t>
         </is>
       </c>
-      <c r="H80" s="2" t="inlineStr">
+      <c r="H123" s="2" t="inlineStr">
         <is>
           <t>requirements.md Story 8 S8-R3; Story 2 S2-N3</t>
         </is>
       </c>
-      <c r="I80" s="2" t="inlineStr"/>
-      <c r="J80" s="2" t="inlineStr"/>
+      <c r="I123" s="2" t="inlineStr"/>
+      <c r="J123" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Rule 54: Filters 110/110 pushed; local source, id-maps and imports synced
Filters 110/110 written and byte-verified (custom_expected + refs).
Local case source mirrored for both projects; Filters id-map gained a refs
column mirroring the Schedule schema (110/110 populated, Rule 20).
Imports regenerated: 165 and 110 records, provenance line on 100%, header
sha256 identical to all four peer projects, 0 VIU/flag words, 0 duplicate
titles, 0 internal-ID or C-id leaks, 0 Rule-4 misplacements.
id-maps restored after gen_import blanked the C-id column (known behaviour).
Runs 357 and 352 verified unchanged: tests set-equal both ways, every prior
result present by id (429 and 395).
</commit_message>
<xml_diff>
--- a/testrail-import/filters-v1-testrail-import.xlsx
+++ b/testrail-import/filters-v1-testrail-import.xlsx
@@ -523,12 +523,14 @@
       <c r="G2" s="2" t="inlineStr">
         <is>
           <t>1. A filter bar is visible directly below the tab row and above the work order table.
-2. The filter bar is shown by default (expanded) without having to turn anything on.</t>
+2. The filter bar is shown by default (expanded) without having to turn anything on.
+---
+This is the expected behaviour as per epic SV-8785 and the Filters specification version 1.6 (S1-R1).</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>Filters (no Jira epic) (S1-R1) [spec v1.6 2026-07-28]</t>
+          <t>SV-8786 (S1-R1) [spec v1.6 2026-07-28]</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr"/>
@@ -572,12 +574,14 @@
         <is>
           <t>1. Exactly five filter chips appear, in this order: Status, Customer, Lead Technician, Service Advisor, Asset on site.
 2. Each chip shows a small icon, the filter name and a down arrow (chevron) indicating it opens a dropdown.
-3. In the design the icons are: a spinner for Status, a person for Customer, a wrench for Lead Technician, a headset for Service Advisor and a truck for Asset on site.</t>
+3. In the design the icons are: a spinner for Status, a person for Customer, a wrench for Lead Technician, a headset for Service Advisor and a truck for Asset on site.
+---
+This is the expected behaviour as per epic SV-8785 and the Filters specification version 1.6 (S1-R2, S1-R3).</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>Filters (no Jira epic) (S1-R2; S1-R3) [spec v1.6 2026-07-28]</t>
+          <t>SV-8786 (S1-R2; S1-R3) [spec v1.6 2026-07-28]</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr"/>
@@ -620,12 +624,14 @@
         <is>
           <t>1. The filter bar is still shown - it does not disappear on this tab.
 2. The Customer, Lead Technician, Service Advisor and Asset on site chips are all displayed and usable.
-3. The Status chip is not usable on this tab: it is shown greyed out and already filled in with the tab's own status, and cannot be clicked.</t>
+3. The Status chip is not usable on this tab: it is shown greyed out and already filled in with the tab's own status, and cannot be clicked.
+---
+This is the expected behaviour as per epic SV-8785 and the Filters specification version 1.6 (S1-N1, S9-R2). The current behaviour follows a later product owner decision dated 2026-07-17.</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>Filters (no Jira epic) (S1-N1; S9-R2; §4 Key Decisions - PRD text says "hidden"; behaviour per Branko Q4=B 2026-07-17 + QA-lead ruling 2026-07-30 = shown greyed-out/disabled) [spec v1.6 2026-07-28]</t>
+          <t>SV-8785 [epic] (S1-N1; S9-R2; §4 Key Decisions - PRD text says "hidden"; behaviour per Branko Q4=B 2026-07-17 + QA-lead ruling 2026-07-30 = shown greyed-out/disabled) [spec v1.6 2026-07-28]</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr"/>
@@ -671,12 +677,14 @@
           <t>1. A dropdown panel opens under the Status chip.
 2. It lists all nine statuses as checkboxes, in this order: Estimate, Approved, In progress, Review, Complete, Invoiced, Paid, Declined, Imported.
 3. All checkboxes are unticked (nothing selected yet).
-4. A 'Clear selection' action is shown at the bottom of the dropdown.</t>
+4. A 'Clear selection' action is shown at the bottom of the dropdown.
+---
+This is the expected behaviour as per epic SV-8785 and the Filters specification version 1.6 (S2-R1, S2-R4).</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>Filters (no Jira epic) (S2-R1; S2-R4) [spec v1.6 2026-07-28]</t>
+          <t>SV-8787 (S2-R1; S2-R4) [spec v1.6 2026-07-28]</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr"/>
@@ -721,12 +729,14 @@
         <is>
           <t>1. The ticked checkbox appears filled (checked).
 2. The table updates immediately to show only work orders in the selected status - there is no confirm or apply button on desktop.
-3. Work orders in other statuses are no longer listed.</t>
+3. Work orders in other statuses are no longer listed.
+---
+This is the expected behaviour as per epic SV-8785 and the Filters specification version 1.6 (S2-R2, S2-R3, S2-R6).</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>Filters (no Jira epic) (S2-R2; S2-R3; S2-R6) [spec v1.6 2026-07-28]</t>
+          <t>SV-8787 (S2-R2; S2-R3; S2-R6) [spec v1.6 2026-07-28]</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr"/>
@@ -772,12 +782,14 @@
           <t>1. Every ticked status shows a filled checkbox.
 2. The table shows work orders whose status matches ANY of the ticked statuses (both Estimate and Approved rows appear).
 3. Work orders in statuses that are not ticked are hidden.
-4. There is no limit on how many statuses you can tick.</t>
+4. There is no limit on how many statuses you can tick.
+---
+This is the expected behaviour as per epic SV-8785 and the Filters specification version 1.6 (S2-R2).</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>Filters (no Jira epic) (S2-R2; §4 Key Decisions (no selection limit)) [spec v1.6 2026-07-28]</t>
+          <t>SV-8787 (S2-R2; §4 Key Decisions (no selection limit)) [spec v1.6 2026-07-28]</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr"/>
@@ -822,12 +834,14 @@
         <is>
           <t>1. All status checkboxes become unticked.
 2. The Status filter is removed and the table returns to showing work orders of every status.
-3. Only the Status filter is affected - any other active filters stay applied.</t>
+3. Only the Status filter is affected - any other active filters stay applied.
+---
+This is the expected behaviour as per epic SV-8785 and the Filters specification version 1.6 (S2-R4, S8-R2).</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>Filters (no Jira epic) (S2-R4; S8-R2) [spec v1.6 2026-07-28]</t>
+          <t>SV-8785 [epic] (S2-R4; S8-R2) [spec v1.6 2026-07-28]</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr"/>
@@ -871,12 +885,14 @@
         <is>
           <t>1. The dropdown closes.
 2. The ticked statuses stay selected - the Status chip stays in its active state showing the selection.
-3. The table stays filtered by the selected statuses.</t>
+3. The table stays filtered by the selected statuses.
+---
+This is the expected behaviour as per epic SV-8785 and the Filters specification version 1.6 (S2-R5).</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>Filters (no Jira epic) (S2-R5) [spec v1.6 2026-07-28]</t>
+          <t>SV-8787 (S2-R5) [spec v1.6 2026-07-28]</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr"/>
@@ -921,12 +937,14 @@
         <is>
           <t>1. The table shows no rows.
 2. An empty state is displayed saying no results were found for the current filters (see the Empty State cases for its full content).
-3. The app does not show an error.</t>
+3. The app does not show an error.
+---
+This is the expected behaviour as per epic SV-8785 and the Filters specification version 1.6 (S2-N3, S8-R3).</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>Filters (no Jira epic) (S2-N3; S8-R3) [spec v1.6 2026-07-28]</t>
+          <t>SV-8785 [epic] (S2-N3; S8-R3) [spec v1.6 2026-07-28]</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr"/>
@@ -973,12 +991,14 @@
           <t>1. The table switches to showing imported work orders only.
 2. While Imported is ticked, the other filter chips are greyed out and cannot be used.
 3. Imported cannot be combined with other statuses - selecting it works alone.
-4. Unticking Imported re-enables the other chips and the normal list returns.</t>
+4. Unticking Imported re-enables the other chips and the normal list returns.
+---
+This is the expected behaviour as per epic SV-8785 and the Filters specification version 1.6 (S2-R7, S2-N4).</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>Filters (no Jira epic) (S2-R7 (Imported cannot be combined with anything else; other filter chips disabled while it is active); S2-N4 (the combination is prevented rather than returning an empty result)) [spec v1.6 2026-07-28]</t>
+          <t>SV-8787 (S2-R7 (Imported cannot be combined with anything else; other filter chips disabled while it is active); S2-N4 (the combination is prevented rather than returning an empty result)) [spec v1.6 2026-07-28]</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr"/>
@@ -1024,12 +1044,14 @@
           <t>1. A dropdown panel opens under the Customer chip.
 2. A search input with the placeholder 'Search customer' is at the top, already focused so you can type right away.
 3. Below it is a scrollable list of customer names.
-4. A 'Clear selection' action is shown at the bottom of the panel.</t>
+4. A 'Clear selection' action is shown at the bottom of the panel.
+---
+This is the expected behaviour as per epic SV-8785 and the Filters specification version 1.6 (S3-R1).</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>Filters (no Jira epic) (S3-R1) [spec v1.6 2026-07-28]</t>
+          <t>SV-8788 (S3-R1) [spec v1.6 2026-07-28]</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr"/>
@@ -1073,12 +1095,14 @@
         <is>
           <t>1. The customer list narrows as you type, showing only names that match what you entered.
 2. Customers that do not match are removed from the list.
-3. Deleting the text brings the full list back.</t>
+3. Deleting the text brings the full list back.
+---
+This is the expected behaviour as per epic SV-8785 and the Filters specification version 1.6 (S3-R2).</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>Filters (no Jira epic) (S3-R2) [spec v1.6 2026-07-28]</t>
+          <t>SV-8788 (S3-R2) [spec v1.6 2026-07-28]</t>
         </is>
       </c>
       <c r="I13" s="2" t="inlineStr"/>
@@ -1124,12 +1148,14 @@
           <t>1. Each selected customer appears as a tag (small chip) with an x in the input area at the top of the dropdown.
 2. Each selected customer's row in the list shows a checkmark on the right.
 3. Long customer names on tags are shortened with an ellipsis (for example 'Texas Truck And Aut...').
-4. You can keep selecting as many customers as needed - there is no selection limit.</t>
+4. You can keep selecting as many customers as needed - there is no selection limit.
+---
+This is the expected behaviour as per epic SV-8785 and the Filters specification version 1.6 (S3-R3, S3-R4).</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>Filters (no Jira epic) (S3-R3; S3-R4; §4 Key Decisions (no selection limit)) [spec v1.6 2026-07-28]</t>
+          <t>SV-8788 (S3-R3; S3-R4; §4 Key Decisions (no selection limit)) [spec v1.6 2026-07-28]</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr"/>
@@ -1174,12 +1200,14 @@
           <t>1. That customer's tag disappears from the input area.
 2. The checkmark next to that customer in the list is removed.
 3. The other selected customers keep their tags and checkmarks.
-4. The table updates to no longer include that customer's work orders.</t>
+4. The table updates to no longer include that customer's work orders.
+---
+This is the expected behaviour as per epic SV-8785 and the Filters specification version 1.6 (S3-R5).</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>Filters (no Jira epic) (S3-R5) [spec v1.6 2026-07-28]</t>
+          <t>SV-8788 (S3-R5) [spec v1.6 2026-07-28]</t>
         </is>
       </c>
       <c r="I15" s="2" t="inlineStr"/>
@@ -1223,12 +1251,14 @@
         <is>
           <t>1. The table shows only work orders whose customer is one of the two selected customers.
 2. Work orders belonging to any other customer are hidden.
-3. The table updates in real time as you make the selections (no apply button on desktop).</t>
+3. The table updates in real time as you make the selections (no apply button on desktop).
+---
+This is the expected behaviour as per epic SV-8785 and the Filters specification version 1.6 (S3-R6, S2-R6).</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>Filters (no Jira epic) (S3-R6; S2-R6 (real-time pattern)) [spec v1.6 2026-07-28]</t>
+          <t>SV-8785 [epic] (S3-R6; S2-R6 (real-time pattern)) [spec v1.6 2026-07-28]</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr"/>
@@ -1274,12 +1304,14 @@
           <t>1. All customer tags are removed from the input area.
 2. All checkmarks in the list are removed.
 3. The Customer filter is removed and the table shows work orders of all customers again.
-4. Other active filters (if any) are not affected.</t>
+4. Other active filters (if any) are not affected.
+---
+This is the expected behaviour as per epic SV-8785 and the Filters specification version 1.6 (S3-R7, S8-R2).</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>Filters (no Jira epic) (S3-R7; S8-R2) [spec v1.6 2026-07-28]</t>
+          <t>SV-8785 [epic] (S3-R7; S8-R2) [spec v1.6 2026-07-28]</t>
         </is>
       </c>
       <c r="I17" s="2" t="inlineStr"/>
@@ -1323,12 +1355,14 @@
         <is>
           <t>1. The dropdown closes when you click outside it.
 2. The Customer chip stays in the active (blue) state showing the selection and the table stays filtered.
-3. When reopened, the selected customers' tags are still visible in the input area.</t>
+3. When reopened, the selected customers' tags are still visible in the input area.
+---
+This is the expected behaviour as per epic SV-8785 and the Filters specification version 1.6 (S3-R8).</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>Filters (no Jira epic) (S3-R8) [spec v1.6 2026-07-28]</t>
+          <t>SV-8788 (S3-R8) [spec v1.6 2026-07-28]</t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr"/>
@@ -1371,12 +1405,14 @@
         <is>
           <t>1. The list shows a message saying there are no results (instead of an empty gap).
 2. The app does not show an error.
-3. Clearing the search text brings the customer list back.</t>
+3. Clearing the search text brings the customer list back.
+---
+This is the expected behaviour as per epic SV-8785 and the Filters specification version 1.6 (S3-N1).</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>Filters (no Jira epic) (S3-N1) [spec v1.6 2026-07-28]</t>
+          <t>SV-8788 (S3-N1) [spec v1.6 2026-07-28]</t>
         </is>
       </c>
       <c r="I19" s="2" t="inlineStr"/>
@@ -1421,12 +1457,14 @@
         <is>
           <t>1. The customer with no work orders IS shown in the filter list (they are not hidden).
 2. After selecting only that customer, the table shows no rows and the filtered empty state is displayed.
-3. No error is shown.</t>
+3. No error is shown.
+---
+This is the expected behaviour as per epic SV-8785 and the Filters specification version 1.6 (S3-E1, S3-N2, S8-R3).</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>Filters (no Jira epic) (S3-E1; S3-N2; S8-R3) [spec v1.6 2026-07-28]</t>
+          <t>SV-8785 [epic] (S3-E1; S3-N2; S8-R3) [spec v1.6 2026-07-28]</t>
         </is>
       </c>
       <c r="I20" s="2" t="inlineStr"/>
@@ -1471,12 +1509,14 @@
           <t>1. A dropdown panel opens under the Lead Technician chip.
 2. A search input with the placeholder 'Search technician' is at the top.
 3. Below it is a scrollable list of technician names.
-4. A 'Clear selection' action is shown at the bottom.</t>
+4. A 'Clear selection' action is shown at the bottom.
+---
+This is the expected behaviour as per epic SV-8785 and the Filters specification version 1.6 (S4-R1).</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>Filters (no Jira epic) (S4-R1) [spec v1.6 2026-07-28]</t>
+          <t>SV-8789 (S4-R1) [spec v1.6 2026-07-28]</t>
         </is>
       </c>
       <c r="I21" s="2" t="inlineStr"/>
@@ -1518,12 +1558,14 @@
       <c r="G22" s="2" t="inlineStr">
         <is>
           <t>1. The technician list narrows to only the names matching what you typed.
-2. Deleting the text brings the full list back.</t>
+2. Deleting the text brings the full list back.
+---
+This is the expected behaviour as per epic SV-8785 and the Filters specification version 1.6 (S4-R2).</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>Filters (no Jira epic) (S4-R2) [spec v1.6 2026-07-28]</t>
+          <t>SV-8789 (S4-R2) [spec v1.6 2026-07-28]</t>
         </is>
       </c>
       <c r="I22" s="2" t="inlineStr"/>
@@ -1568,12 +1610,14 @@
           <t>1. Selected technicians show a filled checkbox in the list.
 2. The table shows only work orders where one of the selected technicians is assigned as the LEAD technician.
 3. A work order where the technician is assigned only in a non-lead role does not appear.
-4. The table updates in real time as you select.</t>
+4. The table updates in real time as you select.
+---
+This is the expected behaviour as per epic SV-8785 and the Filters specification version 1.6 (S4-R3, S4-R4).</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>Filters (no Jira epic) (S4-R3; S4-R4) [spec v1.6 2026-07-28]</t>
+          <t>SV-8789 (S4-R3; S4-R4) [spec v1.6 2026-07-28]</t>
         </is>
       </c>
       <c r="I23" s="2" t="inlineStr"/>
@@ -1617,12 +1661,14 @@
         <is>
           <t>1. All technician selections are removed (checkboxes unticked).
 2. The Lead Technician filter no longer restricts the table.
-3. Other active filters are not affected.</t>
+3. Other active filters are not affected.
+---
+This is the expected behaviour as per epic SV-8785 and the Filters specification version 1.6 (S4-R5, S8-R2).</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>Filters (no Jira epic) (S4-R5; S8-R2) [spec v1.6 2026-07-28]</t>
+          <t>SV-8785 [epic] (S4-R5; S8-R2) [spec v1.6 2026-07-28]</t>
         </is>
       </c>
       <c r="I24" s="2" t="inlineStr"/>
@@ -1664,12 +1710,14 @@
       <c r="G25" s="2" t="inlineStr">
         <is>
           <t>1. The dropdown closes.
-2. The selection stays applied - the chip stays active and the table stays filtered.</t>
+2. The selection stays applied - the chip stays active and the table stays filtered.
+---
+This is the expected behaviour as per epic SV-8785 and the Filters specification version 1.6 (S4-R6).</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>Filters (no Jira epic) (S4-R6) [spec v1.6 2026-07-28]</t>
+          <t>SV-8789 (S4-R6) [spec v1.6 2026-07-28]</t>
         </is>
       </c>
       <c r="I25" s="2" t="inlineStr"/>
@@ -1712,12 +1760,14 @@
       <c r="G26" s="2" t="inlineStr">
         <is>
           <t>1. The table shows no rows and the filtered empty state is displayed.
-2. No error is shown.</t>
+2. No error is shown.
+---
+This is the expected behaviour as per epic SV-8785 and the Filters specification version 1.6 (S4-N1, S8-R3).</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>Filters (no Jira epic) (S4-N1; S8-R3) [spec v1.6 2026-07-28]</t>
+          <t>SV-8785 [epic] (S4-N1; S8-R3) [spec v1.6 2026-07-28]</t>
         </is>
       </c>
       <c r="I26" s="2" t="inlineStr"/>
@@ -1761,12 +1811,14 @@
       <c r="G27" s="2" t="inlineStr">
         <is>
           <t>1. The deactivated technician is NOT shown in the filter list.
-2. Active technicians are still listed normally.</t>
+2. Active technicians are still listed normally.
+---
+This is the expected behaviour as per epic SV-8785 and the Filters specification version 1.6 (S4-E1).</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr">
         <is>
-          <t>Filters (no Jira epic) (S4-E1) [spec v1.6 2026-07-28]</t>
+          <t>SV-8789 (S4-E1) [spec v1.6 2026-07-28]</t>
         </is>
       </c>
       <c r="I27" s="2" t="inlineStr"/>
@@ -1811,12 +1863,14 @@
           <t>1. A dropdown panel opens under the Service Advisor chip.
 2. A search input with the placeholder 'Search advisor' is at the top.
 3. Below it is a scrollable list of advisor names.
-4. A 'Clear selection' action is shown at the bottom.</t>
+4. A 'Clear selection' action is shown at the bottom.
+---
+This is the expected behaviour as per epic SV-8785 and the Filters specification version 1.6 (S5-R1).</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>Filters (no Jira epic) (S5-R1) [spec v1.6 2026-07-28]</t>
+          <t>SV-8790 (S5-R1) [spec v1.6 2026-07-28]</t>
         </is>
       </c>
       <c r="I28" s="2" t="inlineStr"/>
@@ -1858,12 +1912,14 @@
       <c r="G29" s="2" t="inlineStr">
         <is>
           <t>1. The advisor list narrows to only the names matching what you typed.
-2. Deleting the text brings the full list back.</t>
+2. Deleting the text brings the full list back.
+---
+This is the expected behaviour as per epic SV-8785 and the Filters specification version 1.6 (S5-R2).</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>Filters (no Jira epic) (S5-R2) [spec v1.6 2026-07-28]</t>
+          <t>SV-8790 (S5-R2) [spec v1.6 2026-07-28]</t>
         </is>
       </c>
       <c r="I29" s="2" t="inlineStr"/>
@@ -1907,12 +1963,14 @@
         <is>
           <t>1. Selected advisors show a filled checkbox in the list.
 2. The table shows only work orders assigned to any of the selected advisors.
-3. The table updates in real time as you select.</t>
+3. The table updates in real time as you select.
+---
+This is the expected behaviour as per epic SV-8785 and the Filters specification version 1.6 (S5-R3, S5-R4).</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>Filters (no Jira epic) (S5-R3; S5-R4) [spec v1.6 2026-07-28]</t>
+          <t>SV-8790 (S5-R3; S5-R4) [spec v1.6 2026-07-28]</t>
         </is>
       </c>
       <c r="I30" s="2" t="inlineStr"/>
@@ -1956,12 +2014,14 @@
         <is>
           <t>1. All advisor selections are removed.
 2. The Service Advisor filter no longer restricts the table.
-3. Other active filters are not affected.</t>
+3. Other active filters are not affected.
+---
+This is the expected behaviour as per epic SV-8785 and the Filters specification version 1.6 (S5-R5, S8-R2).</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr">
         <is>
-          <t>Filters (no Jira epic) (S5-R5; S8-R2) [spec v1.6 2026-07-28]</t>
+          <t>SV-8785 [epic] (S5-R5; S8-R2) [spec v1.6 2026-07-28]</t>
         </is>
       </c>
       <c r="I31" s="2" t="inlineStr"/>
@@ -2003,12 +2063,14 @@
       <c r="G32" s="2" t="inlineStr">
         <is>
           <t>1. The dropdown closes.
-2. The selection stays applied - the chip stays active and the table stays filtered.</t>
+2. The selection stays applied - the chip stays active and the table stays filtered.
+---
+This is the expected behaviour as per epic SV-8785 and the Filters specification version 1.6 (S5-R6).</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
-          <t>Filters (no Jira epic) (S5-R6) [spec v1.6 2026-07-28]</t>
+          <t>SV-8790 (S5-R6) [spec v1.6 2026-07-28]</t>
         </is>
       </c>
       <c r="I32" s="2" t="inlineStr"/>
@@ -2051,12 +2113,14 @@
       <c r="G33" s="2" t="inlineStr">
         <is>
           <t>1. The table shows no rows and the filtered empty state is displayed.
-2. No error is shown.</t>
+2. No error is shown.
+---
+This is the expected behaviour as per epic SV-8785 and the Filters specification version 1.6 (S5-N1, S8-R3).</t>
         </is>
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
-          <t>Filters (no Jira epic) (S5-N1; S8-R3) [spec v1.6 2026-07-28]</t>
+          <t>SV-8785 [epic] (S5-N1; S8-R3) [spec v1.6 2026-07-28]</t>
         </is>
       </c>
       <c r="I33" s="2" t="inlineStr"/>
@@ -2100,12 +2164,14 @@
       <c r="G34" s="2" t="inlineStr">
         <is>
           <t>1. The deactivated advisor is NOT shown in the filter list.
-2. Active advisors are still listed normally.</t>
+2. Active advisors are still listed normally.
+---
+This is the expected behaviour as per epic SV-8785 and the Filters specification version 1.6 (S5-E1).</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>Filters (no Jira epic) (S5-E1) [spec v1.6 2026-07-28]</t>
+          <t>SV-8790 (S5-E1) [spec v1.6 2026-07-28]</t>
         </is>
       </c>
       <c r="I34" s="2" t="inlineStr"/>
@@ -2149,12 +2215,14 @@
           <t>1. A small dropdown panel opens under the Asset on site chip.
 2. It contains exactly two options: Yes and No.
 3. A 'Clear selection' action is shown at the bottom.
-4. It is a dropdown (like the other filters), not an on/off toggle.</t>
+4. It is a dropdown (like the other filters), not an on/off toggle.
+---
+This is the expected behaviour as per epic SV-8785 and the Filters specification version 1.6 (S6-R1).</t>
         </is>
       </c>
       <c r="H35" s="2" t="inlineStr">
         <is>
-          <t>Filters (no Jira epic) (S6-R1; §4 Key Decisions (dropdown - not toggle)) [spec v1.6 2026-07-28]</t>
+          <t>SV-8791 (S6-R1; §4 Key Decisions (dropdown - not toggle)) [spec v1.6 2026-07-28]</t>
         </is>
       </c>
       <c r="I35" s="2" t="inlineStr"/>
@@ -2197,12 +2265,14 @@
       <c r="G36" s="2" t="inlineStr">
         <is>
           <t>1. The table shows only work orders whose asset is currently on site.
-2. Work orders whose asset is not on site are hidden.</t>
+2. Work orders whose asset is not on site are hidden.
+---
+This is the expected behaviour as per epic SV-8785 and the Filters specification version 1.6 (S6-R2).</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr">
         <is>
-          <t>Filters (no Jira epic) (S6-R2) [spec v1.6 2026-07-28]</t>
+          <t>SV-8791 (S6-R2) [spec v1.6 2026-07-28]</t>
         </is>
       </c>
       <c r="I36" s="2" t="inlineStr"/>
@@ -2246,12 +2316,14 @@
         <is>
           <t>1. No becomes the selected option and Yes is deselected automatically - only one option can be selected at a time.
 2. The table switches to showing only the not-on-site work orders.
-3. The chip shows the currently selected value.</t>
+3. The chip shows the currently selected value.
+---
+This is the expected behaviour as per epic SV-8785 and the Filters specification version 1.6 (S6-R3).</t>
         </is>
       </c>
       <c r="H37" s="2" t="inlineStr">
         <is>
-          <t>Filters (no Jira epic) (S6-R3) [spec v1.6 2026-07-28]</t>
+          <t>SV-8791 (S6-R3) [spec v1.6 2026-07-28]</t>
         </is>
       </c>
       <c r="I37" s="2" t="inlineStr"/>
@@ -2294,12 +2366,14 @@
         <is>
           <t>1. The selection is removed and the chip returns to its default (inactive) state.
 2. The table shows work orders regardless of on-site status again.
-3. Other active filters are not affected.</t>
+3. Other active filters are not affected.
+---
+This is the expected behaviour as per epic SV-8785 and the Filters specification version 1.6 (S6-R4, S8-R2).</t>
         </is>
       </c>
       <c r="H38" s="2" t="inlineStr">
         <is>
-          <t>Filters (no Jira epic) (S6-R4; S8-R2) [spec v1.6 2026-07-28]</t>
+          <t>SV-8785 [epic] (S6-R4; S8-R2) [spec v1.6 2026-07-28]</t>
         </is>
       </c>
       <c r="I38" s="2" t="inlineStr"/>
@@ -2341,12 +2415,14 @@
       <c r="G39" s="2" t="inlineStr">
         <is>
           <t>1. The dropdown closes.
-2. The Yes selection stays applied - the chip stays active and the table stays filtered.</t>
+2. The Yes selection stays applied - the chip stays active and the table stays filtered.
+---
+This is the expected behaviour as per epic SV-8785 and the Filters specification version 1.6 (S6-R5).</t>
         </is>
       </c>
       <c r="H39" s="2" t="inlineStr">
         <is>
-          <t>Filters (no Jira epic) (S6-R5) [spec v1.6 2026-07-28]</t>
+          <t>SV-8791 (S6-R5) [spec v1.6 2026-07-28]</t>
         </is>
       </c>
       <c r="I39" s="2" t="inlineStr"/>
@@ -2389,12 +2465,14 @@
       <c r="G40" s="2" t="inlineStr">
         <is>
           <t>1. The table shows no rows and the filtered empty state is displayed.
-2. No error is shown.</t>
+2. No error is shown.
+---
+This is the expected behaviour as per epic SV-8785 and the Filters specification version 1.6 (S6-N1, S8-R3).</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr">
         <is>
-          <t>Filters (no Jira epic) (S6-N1; S8-R3) [spec v1.6 2026-07-28]</t>
+          <t>SV-8785 [epic] (S6-N1; S8-R3) [spec v1.6 2026-07-28]</t>
         </is>
       </c>
       <c r="I40" s="2" t="inlineStr"/>
@@ -2439,12 +2517,14 @@
         <is>
           <t>1. Only work orders whose asset is NOT on site remain in the list.
 2. Every work order with the asset on site is excluded.
-3. The chip shows the active No selection.</t>
+3. The chip shows the active No selection.
+---
+This is the expected behaviour as per epic SV-8785 and the Filters specification version 1.6 (S6-R2).</t>
         </is>
       </c>
       <c r="H41" s="2" t="inlineStr">
         <is>
-          <t>Filters (no Jira epic) (S6-R2; tech plan 2026-07-29 G4 (filtering No is new capability)) [spec v1.6 2026-07-28]</t>
+          <t>SV-8791 (S6-R2; tech plan 2026-07-29 G4 (filtering No is new capability)) [spec v1.6 2026-07-28]</t>
         </is>
       </c>
       <c r="I41" s="2" t="inlineStr"/>
@@ -2487,12 +2567,14 @@
         <is>
           <t>1. The Status chip changes to an active/highlighted look (blue pill).
 2. The chip displays the selected value (for example 'Status: Estimate').
-3. The other chips stay in their default state.</t>
+3. The other chips stay in their default state.
+---
+This is the expected behaviour as per epic SV-8785 and the Filters specification version 1.6 (S7-R1).</t>
         </is>
       </c>
       <c r="H42" s="2" t="inlineStr">
         <is>
-          <t>Filters (no Jira epic) (S7-R1) [spec v1.6 2026-07-28]</t>
+          <t>SV-8792 (S7-R1) [spec v1.6 2026-07-28]</t>
         </is>
       </c>
       <c r="I42" s="2" t="inlineStr"/>
@@ -2534,12 +2616,14 @@
       <c r="G43" s="2" t="inlineStr">
         <is>
           <t>1. The chip lists the selected values starting with the first one and shortens the label when it gets too long (the design shows 'Status: Estimate, In progress, Approved...').
-2. The chip stays a single compact pill - it does not grow to show every value in full.</t>
+2. The chip stays a single compact pill - it does not grow to show every value in full.
+---
+This is the expected behaviour as per epic SV-8785 and the Filters specification version 1.6 (S7-R2).</t>
         </is>
       </c>
       <c r="H43" s="2" t="inlineStr">
         <is>
-          <t>Filters (no Jira epic) (S7-R2) [spec v1.6 2026-07-28]</t>
+          <t>SV-8792 (S7-R2) [spec v1.6 2026-07-28]</t>
         </is>
       </c>
       <c r="I43" s="2" t="inlineStr"/>
@@ -2584,12 +2668,14 @@
         <is>
           <t>1. With no filters active, no 'Clear filters' button/link is shown (there is nothing to click).
 2. As soon as one filter is active, a blue 'Clear filters' link appears at the right end of the chip row.
-3. When the last active filter is removed, 'Clear filters' disappears again.</t>
+3. When the last active filter is removed, 'Clear filters' disappears again.
+---
+This is the expected behaviour as per epic SV-8785 and the Filters specification version 1.6 (S7-R3, S7-N1, S8-N1).</t>
         </is>
       </c>
       <c r="H44" s="2" t="inlineStr">
         <is>
-          <t>Filters (no Jira epic) (S7-R3; S7-N1; S8-N1) [spec v1.6 2026-07-28]</t>
+          <t>SV-8785 [epic] (S7-R3; S7-N1; S8-N1) [spec v1.6 2026-07-28]</t>
         </is>
       </c>
       <c r="I44" s="2" t="inlineStr"/>
@@ -2635,12 +2721,14 @@
           <t>1. Every active filter is cleared in one click.
 2. All chips return to their default (inactive) look with no values shown.
 3. The table shows the full unfiltered list again (no text is in the page Search box, so nothing else is narrowing it).
-4. The 'Clear filters' link disappears.</t>
+4. The 'Clear filters' link disappears.
+---
+This is the expected behaviour as per epic SV-8785 and the Filters specification version 1.6 (S8-R1, S13-R13).</t>
         </is>
       </c>
       <c r="H45" s="2" t="inlineStr">
         <is>
-          <t>Filters (no Jira epic) (S8-R1; §4 Key Decisions; S13-R13 (clearing filters does not clear a typed search)) [spec v1.6 2026-07-28]</t>
+          <t>SV-8785 [epic] (S8-R1; §4 Key Decisions; S13-R13 (clearing filters does not clear a typed search)) [spec v1.6 2026-07-28]</t>
         </is>
       </c>
       <c r="I45" s="2" t="inlineStr"/>
@@ -2684,12 +2772,14 @@
         <is>
           <t>1. Only the Status filter is cleared - its chip returns to default.
 2. The Customer filter stays selected and active (blue) and keeps filtering the table.
-3. 'Clear filters' remains visible because a filter is still active.</t>
+3. 'Clear filters' remains visible because a filter is still active.
+---
+This is the expected behaviour as per epic SV-8785 and the Filters specification version 1.6 (S8-R2).</t>
         </is>
       </c>
       <c r="H46" s="2" t="inlineStr">
         <is>
-          <t>Filters (no Jira epic) (S8-R2; §4 Key Decisions) [spec v1.6 2026-07-28]</t>
+          <t>SV-8793 (S8-R2; §4 Key Decisions) [spec v1.6 2026-07-28]</t>
         </is>
       </c>
       <c r="I46" s="2" t="inlineStr"/>
@@ -2734,12 +2824,14 @@
         <is>
           <t>1. Only customer A's Estimate work order is shown.
 2. Customer A's Approved work order is hidden (wrong status) and customer B's Estimate work order is hidden (wrong customer) - each additional filter narrows the result further.
-3. Both chips are in the active state and 'Clear filters' is visible.</t>
+3. Both chips are in the active state and 'Clear filters' is visible.
+---
+This is the expected behaviour as per epic SV-8785 and the Filters specification version 1.6 (S8-R3).</t>
         </is>
       </c>
       <c r="H47" s="2" t="inlineStr">
         <is>
-          <t>Filters (no Jira epic) (§2 Feature Overview (multi-criteria); S8-R3 ('combination of active filters')) [spec v1.6 2026-07-28]</t>
+          <t>SV-8793 (§2 Feature Overview (multi-criteria); S8-R3 ('combination of active filters')) [spec v1.6 2026-07-28]</t>
         </is>
       </c>
       <c r="I47" s="2" t="inlineStr"/>
@@ -2783,12 +2875,14 @@
         <is>
           <t>1. The filter bar row is hidden.
 2. The work order table moves up and uses the reclaimed vertical space.
-3. The filter icon shows a pressed/active look while the bar is collapsed.</t>
+3. The filter icon shows a pressed/active look while the bar is collapsed.
+---
+This is the expected behaviour as per epic SV-8785 and the Filters specification version 1.6 (S1-R4, S1-R5).</t>
         </is>
       </c>
       <c r="H48" s="2" t="inlineStr">
         <is>
-          <t>Filters (no Jira epic) (S1-R4; S1-R5) [spec v1.6 2026-07-28]</t>
+          <t>SV-8786 (S1-R4; S1-R5) [spec v1.6 2026-07-28]</t>
         </is>
       </c>
       <c r="I48" s="2" t="inlineStr"/>
@@ -2832,12 +2926,14 @@
         <is>
           <t>1. The filter bar reappears below the tab row.
 2. The previously selected filters are still shown on their chips in the active (blue) state - nothing was lost while collapsed.
-3. The 'Clear filters' link is still shown at the right end of the chip row.</t>
+3. The 'Clear filters' link is still shown at the right end of the chip row.
+---
+This is the expected behaviour as per epic SV-8785 and the Filters specification version 1.6 (S1-R6).</t>
         </is>
       </c>
       <c r="H49" s="2" t="inlineStr">
         <is>
-          <t>Filters (no Jira epic) (S1-R6) [spec v1.6 2026-07-28]</t>
+          <t>SV-8786 (S1-R6) [spec v1.6 2026-07-28]</t>
         </is>
       </c>
       <c r="I49" s="2" t="inlineStr"/>
@@ -2881,12 +2977,14 @@
       <c r="G50" s="2" t="inlineStr">
         <is>
           <t>1. After step 2 the filter bar is still collapsed (your choice was remembered).
-2. After step 4 the filter bar is expanded again when you return - whichever state you left it in is restored.</t>
+2. After step 4 the filter bar is expanded again when you return - whichever state you left it in is restored.
+---
+This is the expected behaviour as per epic SV-8785 and the Filters specification version 1.6 (S1-R7, S10-R1).</t>
         </is>
       </c>
       <c r="H50" s="2" t="inlineStr">
         <is>
-          <t>Filters (no Jira epic) (S1-R7; S10-R1) [spec v1.6 2026-07-28]</t>
+          <t>SV-8785 [epic] (S1-R7; S10-R1) [spec v1.6 2026-07-28]</t>
         </is>
       </c>
       <c r="I50" s="2" t="inlineStr"/>
@@ -2929,12 +3027,14 @@
       <c r="G51" s="2" t="inlineStr">
         <is>
           <t>1. After step 1 the filter icon shows no special indicator (only its normal pressed look).
-2. After step 3 the filter icon shows a visual indicator (filters icon in primary blue) signalling that active filters are in effect while the bar is hidden.</t>
+2. After step 3 the filter icon shows a visual indicator (filters icon in primary blue) signalling that active filters are in effect while the bar is hidden.
+---
+This is the expected behaviour as per epic SV-8785 and the Filters specification version 1.6 (S7-R4, S7-N2).</t>
         </is>
       </c>
       <c r="H51" s="2" t="inlineStr">
         <is>
-          <t>Filters (no Jira epic) (S7-R4; S7-N2) [spec v1.6 2026-07-28]</t>
+          <t>SV-8792 (S7-R4; S7-N2) [spec v1.6 2026-07-28]</t>
         </is>
       </c>
       <c r="I51" s="2" t="inlineStr"/>
@@ -2977,12 +3077,14 @@
       <c r="G52" s="2" t="inlineStr">
         <is>
           <t>1. The table content does not change when the bar collapses - it still shows only the work orders matching the active filters.
-2. Hiding the bar only hides the chips; it does not remove or pause the filtering.</t>
+2. Hiding the bar only hides the chips; it does not remove or pause the filtering.
+---
+This is the expected behaviour as per epic SV-8785 and the Filters specification version 1.6 (S7-R5).</t>
         </is>
       </c>
       <c r="H52" s="2" t="inlineStr">
         <is>
-          <t>Filters (no Jira epic) (S7-R5) [spec v1.6 2026-07-28]</t>
+          <t>SV-8792 (S7-R5) [spec v1.6 2026-07-28]</t>
         </is>
       </c>
       <c r="I52" s="2" t="inlineStr"/>
@@ -3026,12 +3128,14 @@
         <is>
           <t>1. The table body is replaced by an empty state (not just a bare empty grid).
 2. The empty state shows a message indicating no results were found for the current filters.
-3. No error message or broken layout appears.</t>
+3. No error message or broken layout appears.
+---
+This is the expected behaviour as per epic SV-8785 and the Filters specification version 1.6 (S8-R3).</t>
         </is>
       </c>
       <c r="H53" s="2" t="inlineStr">
         <is>
-          <t>Filters (no Jira epic) (S8-R3) [spec v1.6 2026-07-28]</t>
+          <t>SV-8793 (S8-R3) [spec v1.6 2026-07-28]</t>
         </is>
       </c>
       <c r="I53" s="2" t="inlineStr"/>
@@ -3076,12 +3180,14 @@
         <is>
           <t>1. The empty state includes a prompt or link to clear the filters.
 2. Clicking it removes the active filters and the full work order list is shown again (with no text in the Search box, nothing else is narrowing the list).
-3. The chips return to their default state.</t>
+3. The chips return to their default state.
+---
+This is the expected behaviour as per epic SV-8785 and the Filters specification version 1.6 (S8-R4, S8-R5).</t>
         </is>
       </c>
       <c r="H54" s="2" t="inlineStr">
         <is>
-          <t>Filters (no Jira epic) (S8-R4 (the empty state includes a prompt or link to clear filters); S8-R5 (where a query is also active each is cleared independently)) [spec v1.6 2026-07-28]</t>
+          <t>SV-8793 (S8-R4 (the empty state includes a prompt or link to clear filters); S8-R5 (where a query is also active each is cleared independently)) [spec v1.6 2026-07-28]</t>
         </is>
       </c>
       <c r="I54" s="2" t="inlineStr"/>
@@ -3128,12 +3234,14 @@
           <t>1. The table is replaced by a no-results message that mentions BOTH the current filters and the search - not the filters alone.
 2. The message offers a way to clear the filters and, because a search is active, a separate way to clear the search.
 3. Clearing the search brings back the list as narrowed by the filter only - the filter is still on.
-4. Clearing the filters leaves your typed word in the box and still applied - each is cleared on its own without wiping the other.</t>
+4. Clearing the filters leaves your typed word in the box and still applied - each is cleared on its own without wiping the other.
+---
+This is the expected behaviour as per epic SV-8785 and the Filters specification version 1.6 (S8-R3, S8-R4, S8-R5, S13-N1, S13-N2).</t>
         </is>
       </c>
       <c r="H55" s="2" t="inlineStr">
         <is>
-          <t>Filters (no Jira epic) (S8-R3 (empty state covers filters AND any active query); S8-R4 (prompt to clear filters and the query where active); S8-R5 (each cleared independently from the empty state); S13-N1; S13-N2) [spec v1.6 2026-07-28]</t>
+          <t>SV-8785 [epic] (S8-R3 (empty state covers filters AND any active query); S8-R4 (prompt to clear filters and the query where active); S8-R5 (each cleared independently from the empty state); S13-N1; S13-N2) [spec v1.6 2026-07-28]</t>
         </is>
       </c>
       <c r="I55" s="2" t="inlineStr"/>
@@ -3175,12 +3283,14 @@
       <c r="G56" s="2" t="inlineStr">
         <is>
           <t>1. All five chips are shown: Status, Customer, Lead Technician, Service Advisor, Asset on site.
-2. Each chip opens its dropdown and can be used.</t>
+2. Each chip opens its dropdown and can be used.
+---
+This is the expected behaviour as per epic SV-8785 and the Filters specification version 1.6 (S9-R1).</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
         <is>
-          <t>Filters (no Jira epic) (S9-R1) [spec v1.6 2026-07-28]</t>
+          <t>SV-8794 (S9-R1) [spec v1.6 2026-07-28]</t>
         </is>
       </c>
       <c r="I56" s="2" t="inlineStr"/>
@@ -3227,12 +3337,14 @@
         <is>
           <t>1. The Status chip is shown but greyed out, already filled in as 'Status: Estimate', and cannot be clicked or changed - the tab already pre-filters the list to Estimate.
 2. Customer, Lead Technician, Service Advisor and Asset on site chips are shown and usable.
-3. After step 4 the table shows only that customer's ESTIMATE work orders - the customer filter narrows the pre-filtered Estimates list.</t>
+3. After step 4 the table shows only that customer's ESTIMATE work orders - the customer filter narrows the pre-filtered Estimates list.
+---
+This is the expected behaviour as per epic SV-8785 and the Filters specification version 1.6 (S9-R2, S2-N1). The current behaviour follows a later product owner decision dated 2026-07-17.</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
         <is>
-          <t>Filters (no Jira epic) (S9-R2; S2-N1; §4 Key Decisions - PRD text says "hidden"; behaviour per Branko Q4=B 2026-07-17 + QA-lead ruling 2026-07-30 = shown greyed-out/disabled; PRD alignment is Branko's open item) [spec v1.6 2026-07-28]</t>
+          <t>SV-8785 [epic] (S9-R2; S2-N1; §4 Key Decisions - PRD text says "hidden"; behaviour per Branko Q4=B 2026-07-17 + QA-lead ruling 2026-07-30 = shown greyed-out/disabled; PRD alignment is Branko's open item) [spec v1.6 2026-07-28]</t>
         </is>
       </c>
       <c r="I57" s="2" t="inlineStr"/>
@@ -3279,12 +3391,14 @@
         <is>
           <t>1. The Status chip is shown but greyed out, already filled in with this tab's status, and cannot be clicked or changed - the tab already pre-filters the list to Complete.
 2. Customer, Lead Technician, Service Advisor and Asset on site chips are shown and usable.
-3. After step 4 the table shows only that customer's COMPLETE work orders.</t>
+3. After step 4 the table shows only that customer's COMPLETE work orders.
+---
+This is the expected behaviour as per epic SV-8785 and the Filters specification version 1.6 (S9-R3, S2-N2). The current behaviour follows a later product owner decision dated 2026-07-17.</t>
         </is>
       </c>
       <c r="H58" s="2" t="inlineStr">
         <is>
-          <t>Filters (no Jira epic) (S9-R3; S2-N2; §4 Key Decisions - PRD text says "hidden"; behaviour per Branko Q4=B 2026-07-17 + QA-lead ruling 2026-07-30 = shown greyed-out/disabled; PRD alignment is Branko's open item) [spec v1.6 2026-07-28]</t>
+          <t>SV-8785 [epic] (S9-R3; S2-N2; §4 Key Decisions - PRD text says "hidden"; behaviour per Branko Q4=B 2026-07-17 + QA-lead ruling 2026-07-30 = shown greyed-out/disabled; PRD alignment is Branko's open item) [spec v1.6 2026-07-28]</t>
         </is>
       </c>
       <c r="I58" s="2" t="inlineStr"/>
@@ -3329,12 +3443,14 @@
         <is>
           <t>1. All five filter chips are shown on the My Work Orders tab.
 2. The table only ever shows work orders assigned to you (the tab's own scope stays).
-3. After step 2 it shows only YOUR work orders in the ticked status - the filters narrow the user-scoped list, they do not widen it to other users' work orders.</t>
+3. After step 2 it shows only YOUR work orders in the ticked status - the filters narrow the user-scoped list, they do not widen it to other users' work orders.
+---
+This is the expected behaviour as per epic SV-8785 and the Filters specification version 1.6 (S9-R4).</t>
         </is>
       </c>
       <c r="H59" s="2" t="inlineStr">
         <is>
-          <t>Filters (no Jira epic) (S9-R4; §4 Key Decisions (My Work Orders tab does not remove filters)) [spec v1.6 2026-07-28]</t>
+          <t>SV-8794 (S9-R4; §4 Key Decisions (My Work Orders tab does not remove filters)) [spec v1.6 2026-07-28]</t>
         </is>
       </c>
       <c r="I59" s="2" t="inlineStr"/>
@@ -3378,12 +3494,14 @@
         <is>
           <t>1. On the Estimates tab your Status choice is not applied and cannot be changed - the Status chip is greyed out and pre-filled with the tab's own status. The Customer selection is still shown and still filters the list.
 2. Back on the All tab the Status chip reappears with the SAME selection (Approved) still applied - the selection was retained in memory, not lost.
-3. The Customer selection is unchanged throughout.</t>
+3. The Customer selection is unchanged throughout.
+---
+This is the expected behaviour as per epic SV-8785 and the Filters specification version 1.6 (S9-R5, S9-N1, S9-R2). The current behaviour follows a later product owner decision dated 2026-07-17.</t>
         </is>
       </c>
       <c r="H60" s="2" t="inlineStr">
         <is>
-          <t>Filters (no Jira epic) (S9-R5; S9-N1; S9-R2 - behaviour per Branko Q4=B 2026-07-17 + QA-lead ruling 2026-07-30) [spec v1.6 2026-07-28]</t>
+          <t>SV-8794 (S9-R5; S9-N1; S9-R2 - behaviour per Branko Q4=B 2026-07-17 + QA-lead ruling 2026-07-30) [spec v1.6 2026-07-28]</t>
         </is>
       </c>
       <c r="I60" s="2" t="inlineStr"/>
@@ -3426,12 +3544,14 @@
       <c r="G61" s="2" t="inlineStr">
         <is>
           <t>1. On the very first visit the Estimates tab is the selected one, even though All is the FIRST tab in the row (order and default are different on purpose).
-2. After switching to All and returning, the All tab is selected - the app remembers your last-used tab per account.</t>
+2. After switching to All and returning, the All tab is selected - the app remembers your last-used tab per account.
+---
+This is the expected behaviour as per epic SV-8785 and the engineering technical plan. No numbered requirement in the Filters specification version 1.6 covers this point yet.</t>
         </is>
       </c>
       <c r="H61" s="2" t="inlineStr">
         <is>
-          <t>Filters (no Jira epic) (no requirement in the ratified spec v1.6 - default/last-used tab is engineering-plan-only - confirmation requested); tech plan 2026-07-29 D10 (default tab = Estimates; last-used tab persists) [spec v1.6 2026-07-28]</t>
+          <t>SV-8785 [epic] (no requirement in the ratified spec v1.6 - default/last-used tab is engineering-plan-only - confirmation requested); tech plan 2026-07-29 D10 (default tab = Estimates; last-used tab persists) [spec v1.6 2026-07-28]</t>
         </is>
       </c>
       <c r="I61" s="2" t="inlineStr"/>
@@ -3476,12 +3596,14 @@
         <is>
           <t>1. After step 2 the same Status and Customer selections are still applied - chips active with the same values, table filtered the same way.
 2. The filter bar is still expanded (as you left it).
-3. After step 4 the filter bar comes back collapsed - the collapsed/expanded state is restored too.</t>
+3. After step 4 the filter bar comes back collapsed - the collapsed/expanded state is restored too.
+---
+This is the expected behaviour as per epic SV-8785 and the Filters specification version 1.6 (S10-R1, S1-R7).</t>
         </is>
       </c>
       <c r="H62" s="2" t="inlineStr">
         <is>
-          <t>Filters (no Jira epic) (S10-R1; S1-R7) [spec v1.6 2026-07-28]</t>
+          <t>SV-8785 [epic] (S10-R1; S1-R7) [spec v1.6 2026-07-28]</t>
         </is>
       </c>
       <c r="I62" s="2" t="inlineStr"/>
@@ -3528,12 +3650,14 @@
         <is>
           <t>1. After moving around the app (step 2) the filter selections are still applied - you do not have to re-apply them.
 2. After closing the browser completely and signing back in (step 5) the same filter selections are still applied - the app remembers your filters for you permanently, not just for one browser session.
-3. The same filter selections are applied on the other computer too - the filters are saved to your account, not to one computer or browser (to confirm live once built).</t>
+3. The same filter selections are applied on the other computer too - the filters are saved to your account, not to one computer or browser (to confirm live once built).
+---
+This is the expected behaviour as per epic SV-8785 and the Filters specification version 1.6 (S10-R2, S10-R3, S10-R1).</t>
         </is>
       </c>
       <c r="H63" s="2" t="inlineStr">
         <is>
-          <t>Filters (no Jira epic) (S10-R2 (stored server-side against the account; survives logout; syncs across devices); S10-R3 (saved per user); S10-R1 (restored after navigating away)) + Branko Q2 2026-07-17 - now matched by the PRD [spec v1.6 2026-07-28]</t>
+          <t>SV-8795 (S10-R2 (stored server-side against the account; survives logout; syncs across devices); S10-R3 (saved per user); S10-R1 (restored after navigating away)) + Branko Q2 2026-07-17 - now matched by the PRD [spec v1.6 2026-07-28]</t>
         </is>
       </c>
       <c r="I63" s="2" t="inlineStr"/>
@@ -3576,12 +3700,14 @@
       <c r="G64" s="2" t="inlineStr">
         <is>
           <t>1. User B does not see user A's filters - user B's page opens with user B's own (or no) filters.
-2. User B's new filter does not change what user A sees; each user keeps their own saved filter state.</t>
+2. User B's new filter does not change what user A sees; each user keeps their own saved filter state.
+---
+This is the expected behaviour as per epic SV-8785 and the Filters specification version 1.6 (S10-R3).</t>
         </is>
       </c>
       <c r="H64" s="2" t="inlineStr">
         <is>
-          <t>Filters (no Jira epic) (S10-R3; §4 Key Decisions (saved per user)) [spec v1.6 2026-07-28]</t>
+          <t>SV-8795 (S10-R3; §4 Key Decisions (saved per user)) [spec v1.6 2026-07-28]</t>
         </is>
       </c>
       <c r="I64" s="2" t="inlineStr"/>
@@ -3625,12 +3751,14 @@
         <is>
           <t>1. The deleted customer is silently ignored - no error or warning appears.
 2. The Customer filter now reflects only the still-valid selection (the real customer).
-3. The table is filtered by the remaining valid selection only.</t>
+3. The table is filtered by the remaining valid selection only.
+---
+This is the expected behaviour as per epic SV-8785 and the Filters specification version 1.6 (S10-N1).</t>
         </is>
       </c>
       <c r="H65" s="2" t="inlineStr">
         <is>
-          <t>Filters (no Jira epic) (S10-N1) [spec v1.6 2026-07-28]</t>
+          <t>SV-8795 (S10-N1) [spec v1.6 2026-07-28]</t>
         </is>
       </c>
       <c r="I65" s="2" t="inlineStr"/>
@@ -3675,12 +3803,14 @@
         <is>
           <t>1. The second Parts view does NOT show the first view's selections - each view keeps its own.
 2. Returning to the first view restores that view's own selections.
-3. Report tabs likewise keep separate filter choices, each remembered and restored on its own tab.</t>
+3. Report tabs likewise keep separate filter choices, each remembered and restored on its own tab.
+---
+This is the expected behaviour as per epic SV-8785 and the Filters specification version 1.6 (S10-R4).</t>
         </is>
       </c>
       <c r="H66" s="2" t="inlineStr">
         <is>
-          <t>Filters (no Jira epic) (spec v1.6 S10-R4; §4 "Parts and Reports selections are scoped to their view/tab and persist there"); Branko answers 2026-07-31 Q5 exception 1; tech plan 2026-07-29 D20</t>
+          <t>SV-8795 (spec v1.6 S10-R4; §4 "Parts and Reports selections are scoped to their view/tab and persist there"); Branko answers 2026-07-31 Q5 exception 1; tech plan 2026-07-29 D20</t>
         </is>
       </c>
       <c r="I66" s="2" t="inlineStr"/>
@@ -3722,12 +3852,14 @@
       <c r="G67" s="2" t="inlineStr">
         <is>
           <t>1. The old saved choices appear in the new filter bar on the first visit - the update does not lose them (old status choices show in the Status chip, the old asset-here choice shows as Asset on site: Yes, the old My-Work-Orders toggle maps to the My Work Orders tab, columns and sorting stay).
-2. Those carried-over choices are now saved to the account: the other computer shows them too.</t>
+2. Those carried-over choices are now saved to the account: the other computer shows them too.
+---
+This is the expected behaviour as per epic SV-8785 and the engineering technical plan. No numbered requirement in the Filters specification version 1.6 covers this point yet.</t>
         </is>
       </c>
       <c r="H67" s="2" t="inlineStr">
         <is>
-          <t>Filters (no Jira epic) (no numbered v1.6 requirement covers the one-off migration - context S10-R2 server-side model); tech plan 2026-07-29 s4-3.3 (browser-storage to account-preference migration) - confirmation requested [spec v1.6 2026-07-28]</t>
+          <t>SV-8795 (no numbered v1.6 requirement covers the one-off migration - context S10-R2 server-side model); tech plan 2026-07-29 s4-3.3 (browser-storage to account-preference migration) - confirmation requested [spec v1.6 2026-07-28]</t>
         </is>
       </c>
       <c r="I67" s="2" t="inlineStr"/>
@@ -3770,12 +3902,14 @@
       <c r="G68" s="2" t="inlineStr">
         <is>
           <t>1. After step 1 the URL changes to include the active filter state.
-2. After step 3 the filter part of the URL is removed again.</t>
+2. After step 3 the filter part of the URL is removed again.
+---
+This is the expected behaviour as per epic SV-8785 and the Filters specification version 1.6 (S11-R1).</t>
         </is>
       </c>
       <c r="H68" s="2" t="inlineStr">
         <is>
-          <t>Filters (no Jira epic) (S11-R1) [spec v1.6 2026-07-28]</t>
+          <t>SV-8796 (S11-R1) [spec v1.6 2026-07-28]</t>
         </is>
       </c>
       <c r="I68" s="2" t="inlineStr"/>
@@ -3818,12 +3952,14 @@
         <is>
           <t>1. The page opens with the same filters already applied - chips active with the same values.
 2. The table is already filtered accordingly on load (no need to re-apply anything).
-3. The same works from a saved bookmark.</t>
+3. The same works from a saved bookmark.
+---
+This is the expected behaviour as per epic SV-8785 and the Filters specification version 1.6 (S11-R2).</t>
         </is>
       </c>
       <c r="H69" s="2" t="inlineStr">
         <is>
-          <t>Filters (no Jira epic) (S11-R2; §2 Feature Overview (share or bookmark)) [spec v1.6 2026-07-28]</t>
+          <t>SV-8796 (S11-R2; §2 Feature Overview (share or bookmark)) [spec v1.6 2026-07-28]</t>
         </is>
       </c>
       <c r="I69" s="2" t="inlineStr"/>
@@ -3867,12 +4003,14 @@
         <is>
           <t>1. The page loads normally - no error.
 2. The deleted value is ignored; only the still-valid filter value is applied and shown on the chips.
-3. The table reflects only the valid filter.</t>
+3. The table reflects only the valid filter.
+---
+This is the expected behaviour as per epic SV-8785 and the Filters specification version 1.6 (S11-R3).</t>
         </is>
       </c>
       <c r="H70" s="2" t="inlineStr">
         <is>
-          <t>Filters (no Jira epic) (S11-R3) [spec v1.6 2026-07-28]</t>
+          <t>SV-8796 (S11-R3) [spec v1.6 2026-07-28]</t>
         </is>
       </c>
       <c r="I70" s="2" t="inlineStr"/>
@@ -3916,12 +4054,14 @@
         <is>
           <t>1. The Work Orders page loads normally.
 2. No filters are applied (chips in default state, full list shown) - the unrecognizable state is discarded.
-3. No error message or broken page appears.</t>
+3. No error message or broken page appears.
+---
+This is the expected behaviour as per epic SV-8785 and the Filters specification version 1.6 (S11-N1).</t>
         </is>
       </c>
       <c r="H71" s="2" t="inlineStr">
         <is>
-          <t>Filters (no Jira epic) (S11-N1) [spec v1.6 2026-07-28]</t>
+          <t>SV-8796 (S11-N1) [spec v1.6 2026-07-28]</t>
         </is>
       </c>
       <c r="I71" s="2" t="inlineStr"/>
@@ -3972,12 +4112,14 @@
 3. A 'Back to my view' option is shown while you are looking at the shared link. (If the wording on screen is slightly different, note what it says and carry on.)
 4. Clicking 'Back to my view' brings back your own saved filters and removes the filter part from the web address.
 5. It also empties the Search box and removes your typed text - the search is not something that gets saved, so there is nothing to bring back.
-6. Returning normally later still shows your own saved filters, untouched by the link visit.</t>
+6. Returning normally later still shows your own saved filters, untouched by the link visit.
+---
+This is the expected behaviour as per epic SV-8785 and the Filters specification version 1.6 (S11-R6, S11-R7, S11-R8).</t>
         </is>
       </c>
       <c r="H72" s="2" t="inlineStr">
         <is>
-          <t>Filters (no Jira epic) (S11-R6 (URL state runtime-only with no write-back); S11-R7 (Back to my view - also clears the query); S11-R8 (rationale: the query is never saved)) [spec v1.6 2026-07-28]</t>
+          <t>SV-8796 (S11-R6 (URL state runtime-only with no write-back); S11-R7 (Back to my view - also clears the query); S11-R8 (rationale: the query is never saved)) [spec v1.6 2026-07-28]</t>
         </is>
       </c>
       <c r="I72" s="2" t="inlineStr"/>
@@ -4025,12 +4167,14 @@
           <t>1. On your own view there is no 'Back to my view' option anywhere - it only belongs to a shared-link visit.
 2. Changing your own filters does not make it appear.
 3. When you open the shared link, 'Back to my view' does appear.
-4. After you click it and you are back on your own view, the option disappears again.</t>
+4. After you click it and you are back on your own view, the option disappears again.
+---
+This is the expected behaviour as per epic SV-8785 and the Filters specification version 1.6 (S11-N3, S11-R7).</t>
         </is>
       </c>
       <c r="H73" s="2" t="inlineStr">
         <is>
-          <t>Filters (no Jira epic) (S11-N3; S11-R7) [spec v1.6 2026-07-28]</t>
+          <t>SV-8796 (S11-N3; S11-R7) [spec v1.6 2026-07-28]</t>
         </is>
       </c>
       <c r="I73" s="2" t="inlineStr"/>
@@ -4073,12 +4217,14 @@
         <is>
           <t>1. A filter chip row is shown below the tabs, starting with an 'All Filters' chip (with a filter icon) followed by the individual filter chips (Status, Customer, Lead Technician, ...).
 2. The row scrolls horizontally - chips that do not fit are reachable by swiping.
-3. An arrow at the right-hand edge shows that the row can be scrolled. (This is what the design shows - if your screen looks different, write down what you actually see and carry on.)</t>
+3. An arrow at the right-hand edge shows that the row can be scrolled. (This is what the design shows - if your screen looks different, write down what you actually see and carry on.)
+---
+This is the expected behaviour as per epic SV-8785 and the Filters specification version 1.6 (S12-R1). The screen described above comes from the agreed design rather than that specification, and a product owner decision is still awaited.</t>
         </is>
       </c>
       <c r="H74" s="2" t="inlineStr">
         <is>
-          <t>Filters (no Jira epic) (S12-R1) [spec v1.6 2026-07-28]</t>
+          <t>SV-8797 (S12-R1) [spec v1.6 2026-07-28]</t>
         </is>
       </c>
       <c r="I74" s="2" t="inlineStr"/>
@@ -4121,12 +4267,14 @@
         <is>
           <t>1. A bottom sheet slides up with a drag handle at the top, the centered title 'All Filters' and a close (x) button.
 2. It lists the five filters as expandable accordion rows, each with its icon, name and a down arrow: Status, Customer, Lead Technician, Service Advisor, Asset on site.
-3. A sticky blue 'Apply filters' button sits at the bottom of the sheet.</t>
+3. A sticky blue 'Apply filters' button sits at the bottom of the sheet.
+---
+This is the expected behaviour as per epic SV-8785 and the Filters specification version 1.6 (S12-R3). The screen described above comes from the agreed design rather than that specification, and a product owner decision is still awaited.</t>
         </is>
       </c>
       <c r="H75" s="2" t="inlineStr">
         <is>
-          <t>Filters (no Jira epic) (S12-R3) [spec v1.6 2026-07-28]</t>
+          <t>SV-8797 (S12-R3) [spec v1.6 2026-07-28]</t>
         </is>
       </c>
       <c r="I75" s="2" t="inlineStr"/>
@@ -4172,12 +4320,14 @@
         <is>
           <t>1. Expanding Status reveals the same nine status checkboxes as desktop (Estimate, Approved, In progress, Review, Complete, Invoiced, Paid, Declined, Imported) plus 'Clear selection'.
 2. After 'Apply filters' the sheet closes and the work order list shows only the ticked statuses.
-3. The reopened sheet's title shows the applied-filter count, for example 'All Filters (1)', and the Status accordion header is highlighted with the selected values ticked.</t>
+3. The reopened sheet's title shows the applied-filter count, for example 'All Filters (1)', and the Status accordion header is highlighted with the selected values ticked.
+---
+This is the expected behaviour as per epic SV-8785 and the Filters specification version 1.6 (S12-R2, S12-R3, S2-R1). The screen described above comes from the agreed design rather than that specification, and a product owner decision is still awaited.</t>
         </is>
       </c>
       <c r="H76" s="2" t="inlineStr">
         <is>
-          <t>Filters (no Jira epic) (S12-R2; S12-R3; S2-R1) [spec v1.6 2026-07-28]</t>
+          <t>SV-8785 [epic] (S12-R2; S12-R3; S2-R1) [spec v1.6 2026-07-28]</t>
         </is>
       </c>
       <c r="I76" s="2" t="inlineStr"/>
@@ -4221,12 +4371,14 @@
         <is>
           <t>1. A bottom sheet opens for that single filter: its title row shows the filter's icon and name (for example 'Status') with a close (x) button - no accordion list of the other filters.
 2. The sheet shows only that filter's options (the nine status checkboxes plus 'Clear selection').
-3. The bottom button reads 'Apply filter' (singular); tapping it applies the selection and filters the list.</t>
+3. The bottom button reads 'Apply filter' (singular); tapping it applies the selection and filters the list.
+---
+This is the expected behaviour as per epic SV-8785 and the Filters specification version 1.6 (S12-R2, S12-R3). The screen described above comes from the agreed design rather than that specification, and a product owner decision is still awaited.</t>
         </is>
       </c>
       <c r="H77" s="2" t="inlineStr">
         <is>
-          <t>Filters (no Jira epic) (S12-R2; S12-R3) [spec v1.6 2026-07-28]</t>
+          <t>SV-8797 (S12-R2; S12-R3) [spec v1.6 2026-07-28] ; individual-chip real-time per S12-R2 + tech-plan 2026-07-29; only the combined All Filters sheet is batch</t>
         </is>
       </c>
       <c r="I77" s="2" t="inlineStr"/>
@@ -4273,12 +4425,14 @@
           <t>1. The list narrows to matching names as you type.
 2. Each selected customer appears as a tag with an x in the input area, and its list row shows a checkmark.
 3. Removing a tag deselects just that customer.
-4. After 'Apply filters' the list shows only work orders of the remaining selected customers, and the sheet title counts the applied filters (for example 'All Filters (2)').</t>
+4. After 'Apply filters' the list shows only work orders of the remaining selected customers, and the sheet title counts the applied filters (for example 'All Filters (2)').
+---
+This is the expected behaviour as per epic SV-8785 and the Filters specification version 1.6 (S12-R2, S3-R2/R3/R5). The screen described above comes from the agreed design rather than that specification, and a product owner decision is still awaited.</t>
         </is>
       </c>
       <c r="H78" s="2" t="inlineStr">
         <is>
-          <t>Filters (no Jira epic) (S12-R2; S3-R2/R3/R5) [spec v1.6 2026-07-28]</t>
+          <t>SV-8785 [epic] (S12-R2; S3-R2/R3/R5) [spec v1.6 2026-07-28]</t>
         </is>
       </c>
       <c r="I78" s="2" t="inlineStr"/>
@@ -4323,12 +4477,14 @@
         <is>
           <t>1. The Lead Technician row opens with a 'Search technician' field and the technician list.
 2. The Service Advisor row opens with a 'Search advisor' field and the advisor list.
-3. Applying a selection filters the work order list just like on desktop.</t>
+3. Applying a selection filters the work order list just like on desktop.
+---
+This is the expected behaviour as per epic SV-8785 and the Filters specification version 1.6 (S12-R2, S4-R1, S5-R1). The screen described above comes from the agreed design rather than that specification, and a product owner decision is still awaited.</t>
         </is>
       </c>
       <c r="H79" s="2" t="inlineStr">
         <is>
-          <t>Filters (no Jira epic) (S12-R2; S4-R1; S5-R1) [spec v1.6 2026-07-28]</t>
+          <t>SV-8785 [epic] (S12-R2; S4-R1; S5-R1) [spec v1.6 2026-07-28]</t>
         </is>
       </c>
       <c r="I79" s="2" t="inlineStr"/>
@@ -4373,12 +4529,14 @@
         <is>
           <t>1. The Asset on site row opens showing the two options Yes and No plus 'Clear selection'.
 2. Only one option can be selected at a time.
-3. After applying, the list shows only work orders matching the chosen on-site state.</t>
+3. After applying, the list shows only work orders matching the chosen on-site state.
+---
+This is the expected behaviour as per epic SV-8785 and the Filters specification version 1.6 (S12-R2, S6-R1/R2/R3). The screen described above comes from the agreed design rather than that specification, and a product owner decision is still awaited.</t>
         </is>
       </c>
       <c r="H80" s="2" t="inlineStr">
         <is>
-          <t>Filters (no Jira epic) (S12-R2; S6-R1/R2/R3) [spec v1.6 2026-07-28]</t>
+          <t>SV-8785 [epic] (S12-R2; S6-R1/R2/R3) [spec v1.6 2026-07-28]</t>
         </is>
       </c>
       <c r="I80" s="2" t="inlineStr"/>
@@ -4422,12 +4580,14 @@
         <is>
           <t>1. The chip for the applied filter shows the active state with the selected value(s), like on desktop.
 2. A 'Clear filters' control appears while at least one filter is active.
-3. Using it removes all active filters, the chips return to default and the full list comes back.</t>
+3. Using it removes all active filters, the chips return to default and the full list comes back.
+---
+This is the expected behaviour as per epic SV-8785 and the Filters specification version 1.6 (S12-R2, S7-R1/R3, S8-R1).</t>
         </is>
       </c>
       <c r="H81" s="2" t="inlineStr">
         <is>
-          <t>Filters (no Jira epic) (S12-R2; S7-R1/R3; S8-R1) [spec v1.6 2026-07-28]</t>
+          <t>SV-8785 [epic] (S12-R2; S7-R1/R3; S8-R1) [spec v1.6 2026-07-28]</t>
         </is>
       </c>
       <c r="I81" s="2" t="inlineStr"/>
@@ -4469,12 +4629,14 @@
       <c r="G82" s="2" t="inlineStr">
         <is>
           <t>1. There is no filter-bar collapse/expand (filter icon) toggle on mobile.
-2. The filter chip row is always visible on the mobile Work Orders page.</t>
+2. The filter chip row is always visible on the mobile Work Orders page.
+---
+This is the expected behaviour as per epic SV-8785 and the Filters specification version 1.6 (S12-R4).</t>
         </is>
       </c>
       <c r="H82" s="2" t="inlineStr">
         <is>
-          <t>Filters (no Jira epic) (S12-R4) [spec v1.6 2026-07-28]</t>
+          <t>SV-8797 (S12-R4) [spec v1.6 2026-07-28]</t>
         </is>
       </c>
       <c r="I82" s="2" t="inlineStr"/>
@@ -4517,12 +4679,14 @@
         <is>
           <t>1. The list shows the same no-results empty state as desktop, saying no results were found for the current filters.
 2. The empty state includes the prompt to clear filters.
-3. No error appears.</t>
+3. No error appears.
+---
+This is the expected behaviour as per epic SV-8785 and the Filters specification version 1.6 (S12-N1, S8-R3/R4).</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
         <is>
-          <t>Filters (no Jira epic) (S12-N1; S8-R3/R4) [spec v1.6 2026-07-28]</t>
+          <t>SV-8785 [epic] (S12-N1; S8-R3/R4) [spec v1.6 2026-07-28]</t>
         </is>
       </c>
       <c r="I83" s="2" t="inlineStr"/>
@@ -4583,12 +4747,14 @@
 10. Every Parts list page also shows a Search (magnifier) icon and a filter icon in the toolbar; some pages (for example Inventory) also show a column/layout toggle icon.
 11. Every filter button shown above is a working filter on that page - none of them is display-only.
 12. The choices inside each filter come from your own shop's data (for example your real vendors or categories), so there is no fixed list to compare against - check that the choices you see match the data in your shop.
-13. Still to check on the live build: what the filter icon and the column/layout icon do (the written description does not cover the toolbar icons).</t>
+13. Still to check on the live build: what the filter icon and the column/layout icon do (the written description does not cover the toolbar icons).
+---
+This is the expected behaviour as per epic SV-8785 and the Filters specification version 1.6 (§2, §4), which covers this area in its overview and key decisions only. The detailed behaviour above follows a later product owner decision dated 2026-07-31.</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr">
         <is>
-          <t>Filters (no Jira epic) (spec v1.6 §2 Feature Overview -&gt; Parts Filters; §4 Key Decisions -&gt; "Context-specific filter sets on Parts and Reports" + "Multi-select where it makes sense"); Branko answers 2026-07-31 Q2/Q3/Q5/Q7; Figma 11884-16885</t>
+          <t>SV-8785 [epic] (spec v1.6 §2 Feature Overview -&gt; Parts Filters; §4 Key Decisions -&gt; "Context-specific filter sets on Parts and Reports" + "Multi-select where it makes sense"); Branko answers 2026-07-31 Q2/Q3/Q5/Q7; Figma 11884-16885</t>
         </is>
       </c>
       <c r="I84" s="2" t="inlineStr"/>
@@ -4634,12 +4800,14 @@
           <t>1. A small menu opens with two options: Core and Non Core.
 2. A Clear selection action is shown at the bottom of the menu.
 3. You can tick both Core and Non Core at the same time - this filter allows more than one choice.
-4. As soon as you tick a choice the list below narrows to matching parts straight away, with no Apply button to press; Clear selection puts the list back.</t>
+4. As soon as you tick a choice the list below narrows to matching parts straight away, with no Apply button to press; Clear selection puts the list back.
+---
+This is the expected behaviour as per epic SV-8785 and the Filters specification version 1.6 (§2, §4), which covers this area in its overview and key decisions only. The detailed behaviour above follows a later product owner decision dated 2026-07-31.</t>
         </is>
       </c>
       <c r="H85" s="2" t="inlineStr">
         <is>
-          <t>Filters (no Jira epic) (spec v1.6 §2 Feature Overview -&gt; Parts Filters; §4 Key Decisions -&gt; "Context-specific filter sets on Parts and Reports" + "Multi-select where it makes sense"); Branko answers 2026-07-31 Q2/Q3/Q5/Q7; Figma 11884-16885</t>
+          <t>SV-8785 [epic] (spec v1.6 §2 Feature Overview -&gt; Parts Filters; §4 Key Decisions -&gt; "Context-specific filter sets on Parts and Reports" + "Multi-select where it makes sense"); Branko answers 2026-07-31 Q2/Q3/Q5/Q7; Figma 11884-16885</t>
         </is>
       </c>
       <c r="I85" s="2" t="inlineStr"/>
@@ -4683,12 +4851,14 @@
         <is>
           <t>1. The table updates to show only the rows that match the chosen filter value.
 2. The chosen value is shown on the filter button so you can see what is applied.
-3. The list narrows as soon as you pick the value - there is no Apply or Search button to press. Every filter button on every Parts page works this way.</t>
+3. The list narrows as soon as you pick the value - there is no Apply or Search button to press. Every filter button on every Parts page works this way.
+---
+This is the expected behaviour as per epic SV-8785 and the Filters specification version 1.6 (§2, §4), which covers this area in its overview and key decisions only. The detailed behaviour above follows a later product owner decision dated 2026-07-31.</t>
         </is>
       </c>
       <c r="H86" s="2" t="inlineStr">
         <is>
-          <t>Filters (no Jira epic) (spec v1.6 §2 Feature Overview -&gt; Parts Filters; §4 Key Decisions -&gt; "Context-specific filter sets on Parts and Reports" + "Multi-select where it makes sense"); Branko answers 2026-07-31 Q2/Q3/Q5/Q7; Figma 11884-16885</t>
+          <t>SV-8785 [epic] (spec v1.6 §2 Feature Overview -&gt; Parts Filters; §4 Key Decisions -&gt; "Context-specific filter sets on Parts and Reports" + "Multi-select where it makes sense"); Branko answers 2026-07-31 Q2/Q3/Q5/Q7; Figma 11884-16885</t>
         </is>
       </c>
       <c r="I86" s="2" t="inlineStr"/>
@@ -4732,12 +4902,14 @@
         <is>
           <t>1. More than one value can be chosen inside the filter, and the button shows what you picked.
 2. Clear selection removes the choices for that one filter.
-3. A Clear filters button appears in the filter bar while any filter is set, and using it clears them all at once - exactly as it works on the Work Orders page.</t>
+3. A Clear filters button appears in the filter bar while any filter is set, and using it clears them all at once - exactly as it works on the Work Orders page.
+---
+This is the expected behaviour as per epic SV-8785 and the Filters specification version 1.6 (§2, §4), which covers this area in its overview and key decisions only. The detailed behaviour above follows a later product owner decision dated 2026-07-31.</t>
         </is>
       </c>
       <c r="H87" s="2" t="inlineStr">
         <is>
-          <t>Filters (no Jira epic) (spec v1.6 §2 Feature Overview -&gt; Parts Filters; §4 Key Decisions -&gt; "Context-specific filter sets on Parts and Reports" + "Multi-select where it makes sense"); Branko answers 2026-07-31 Q2/Q3/Q5/Q7; Figma 11884-16885</t>
+          <t>SV-8785 [epic] (spec v1.6 §2 Feature Overview -&gt; Parts Filters; §4 Key Decisions -&gt; "Context-specific filter sets on Parts and Reports" + "Multi-select where it makes sense"); Branko answers 2026-07-31 Q2/Q3/Q5/Q7; Figma 11884-16885</t>
         </is>
       </c>
       <c r="I87" s="2" t="inlineStr"/>
@@ -4784,12 +4956,14 @@
         <is>
           <t>1. Every filter the page offered before is still offered - nothing has been taken away.
 2. Every choice each of those filters offered before is still available inside the new button.
-3. If any filter or choice is missing, write down exactly which page, which filter and which choice - that is a bug worth reporting.</t>
+3. If any filter or choice is missing, write down exactly which page, which filter and which choice - that is a bug worth reporting.
+---
+This is the expected behaviour as per epic SV-8785 and the Filters specification version 1.6 (§2), which covers this area in its overview and key decisions only. The detailed behaviour above follows a later product owner decision dated 2026-07-31.</t>
         </is>
       </c>
       <c r="H88" s="2" t="inlineStr">
         <is>
-          <t>Filters (no Jira epic) (spec v1.6 §2 Parts Filters + Reports Filters); Branko answers 2026-07-31 Q3 ("support all the filters we have right now in the app as well as all choices per filter"); tech plan 2026-07-29 rollout rule</t>
+          <t>SV-8785 [epic] (spec v1.6 §2 Parts Filters + Reports Filters); Branko answers 2026-07-31 Q3 ("support all the filters we have right now in the app as well as all choices per filter"); tech plan 2026-07-29 rollout rule</t>
         </is>
       </c>
       <c r="I88" s="2" t="inlineStr"/>
@@ -4867,12 +5041,14 @@
 21. On every report above, each filter button shows its name and a down arrow.
 22. Every filter button shown above is a working filter on that report - none of them is display-only.
 23. The choices inside each filter come from your own shop's data (for example your real vendors or categories), so there is no fixed list to compare against - check that the choices you see match the data in your shop.
-24. Still to check on the live build: the real columns of the Sales Tax report and of the six A/R and A/P aging reports. The design uses sample placeholder tables for those, and the written description does not list their columns.</t>
+24. Still to check on the live build: the real columns of the Sales Tax report and of the six A/R and A/P aging reports. The design uses sample placeholder tables for those, and the written description does not list their columns.
+---
+This is the expected behaviour as per epic SV-8785 and the Filters specification version 1.6 (§2, §4), which covers this area in its overview and key decisions only. The detailed behaviour above follows a later product owner decision dated 2026-07-31.</t>
         </is>
       </c>
       <c r="H89" s="2" t="inlineStr">
         <is>
-          <t>Filters (no Jira epic) (spec v1.6 §2 Reports Filters; §4 Key Decisions "New date-range filter type" + "Multi-select where it makes sense"); Branko answers 2026-07-31 Q2/Q3/Q5/Q7; Figma 11903-10573</t>
+          <t>SV-8785 [epic] (spec v1.6 §2 Reports Filters; §4 Key Decisions "New date-range filter type" + "Multi-select where it makes sense"); Branko answers 2026-07-31 Q2/Q3/Q5/Q7; Figma 11903-10573</t>
         </is>
       </c>
       <c r="I89" s="2" t="inlineStr"/>
@@ -4915,12 +5091,14 @@
       <c r="G90" s="2" t="inlineStr">
         <is>
           <t>1. The report updates to show only the rows matching the chosen filter value, and the chosen value is shown on the filter button.
-2. The report narrows as soon as you pick the value - there is no Apply or Run button to press. Every filter button on every report works this way.</t>
+2. The report narrows as soon as you pick the value - there is no Apply or Run button to press. Every filter button on every report works this way.
+---
+This is the expected behaviour as per epic SV-8785 and the Filters specification version 1.6 (§2, §4), which covers this area in its overview and key decisions only. The detailed behaviour above follows a later product owner decision dated 2026-07-31.</t>
         </is>
       </c>
       <c r="H90" s="2" t="inlineStr">
         <is>
-          <t>Filters (no Jira epic) (spec v1.6 §2 Reports Filters; §4 Key Decisions "New date-range filter type" + "Multi-select where it makes sense"); Branko answers 2026-07-31 Q2/Q3/Q5/Q7; Figma 11903-10573</t>
+          <t>SV-8785 [epic] (spec v1.6 §2 Reports Filters; §4 Key Decisions "New date-range filter type" + "Multi-select where it makes sense"); Branko answers 2026-07-31 Q2/Q3/Q5/Q7; Figma 11903-10573</t>
         </is>
       </c>
       <c r="I90" s="2" t="inlineStr"/>
@@ -4964,12 +5142,14 @@
         <is>
           <t>1. Each of these filter buttons - Location, Transaction Type, Invoice Status, Type, User and Mention - opens a list of choices, lets you tick more than one, and narrows the report straight away with no Apply button.
 2. The choices inside each filter come from your own shop's data (for example your real vendors or categories), so there is no fixed list to compare against - check that the choices you see match the data in your shop.
-3. Write down the choices you actually see behind each of these six buttons. They have not been written down anywhere yet, so your list becomes the record.</t>
+3. Write down the choices you actually see behind each of these six buttons. They have not been written down anywhere yet, so your list becomes the record.
+---
+This is the expected behaviour as per epic SV-8785 and the Filters specification version 1.6 (§2, §4), which covers this area in its overview and key decisions only. The detailed behaviour above follows a later product owner decision dated 2026-07-31.</t>
         </is>
       </c>
       <c r="H91" s="2" t="inlineStr">
         <is>
-          <t>Filters (no Jira epic) (spec v1.6 §2 Reports Filters; §4 "Multi-select where it makes sense"); Branko answers 2026-07-31 Q3/Q5 + Q4 (pointer only - the 6 new types are not enumerated in v1.6; see DELTAS.md F1); Figma 11903-10573</t>
+          <t>SV-8785 [epic] (spec v1.6 §2 Reports Filters; §4 "Multi-select where it makes sense"); Branko answers 2026-07-31 Q3/Q5 + Q4 (pointer only - the 6 new types are not enumerated in v1.6; see DELTAS.md F1); Figma 11903-10573</t>
         </is>
       </c>
       <c r="I91" s="2" t="inlineStr"/>
@@ -5017,12 +5197,14 @@
           <t>1. A start/end date picker opens - there are NO preset ranges (no 'Last 30 days' shortcuts) and NO pre-filled default range.
 2. After only the start date, the results do not change yet.
 3. As soon as the second date is picked, the results update immediately to show only records inside the range.
-4. Only one date range can be active at a time on that chip, and the chip shows the active range.</t>
+4. Only one date range can be active at a time on that chip, and the chip shows the active range.
+---
+This is the expected behaviour as per epic SV-8785 and the Filters specification version 1.6 (§4, §2), which covers this area in its overview and key decisions only. The detailed behaviour above follows a later product owner decision dated 2026-07-31.</t>
         </is>
       </c>
       <c r="H92" s="2" t="inlineStr">
         <is>
-          <t>Filters (no Jira epic) (spec v1.6 §4 "New date-range filter type"; §2 Reports Filters - start/end picker; no presets; no default; applies on the second date); Branko answers 2026-07-31 Q5; tech plan 2026-07-29 D19</t>
+          <t>SV-8785 [epic] (spec v1.6 §4 "New date-range filter type"; §2 Reports Filters - start/end picker; no presets; no default; applies on the second date); Branko answers 2026-07-31 Q5; tech plan 2026-07-29 D19</t>
         </is>
       </c>
       <c r="I92" s="2" t="inlineStr"/>
@@ -5070,12 +5252,14 @@
           <t>1. The control expands in place into a small search box showing the placeholder 'Type to search'.
 2. The list narrows as you type, after a brief pause - and ONLY this page's list changes, nothing else in the app.
 3. The round x clears the text and the full list returns.
-4. Clicking away with an empty box collapses it back to the Search button; with text in it, the box stays open.</t>
+4. Clicking away with an empty box collapses it back to the Search button; with text in it, the box stays open.
+---
+This is the expected behaviour as per epic SV-8785 and the Filters specification version 1.6 (S13-R1, S13-R9, S13-R12, S13-R15).</t>
         </is>
       </c>
       <c r="H93" s="2" t="inlineStr">
         <is>
-          <t>Filters (no Jira epic) (S13-R1 (placement in the toolbar action group); S13-R9 (scoped to this table only); S13-R12; S13-R15 (blur rules)) [spec v1.6 2026-07-28]</t>
+          <t>SV-8798 (S13-R1 (placement in the toolbar action group); S13-R9 (scoped to this table only); S13-R12; S13-R15 (blur rules)) [spec v1.6 2026-07-28]</t>
         </is>
       </c>
       <c r="I93" s="2" t="inlineStr"/>
@@ -5120,12 +5304,14 @@
         <is>
           <t>1. With both active, the results match the filter AND the search together (both narrow the list at once).
 2. Clearing the search keeps the filter applied.
-3. Clearing the filter keeps the search applied - each is cleared by its own control without wiping the other.</t>
+3. Clearing the filter keeps the search applied - each is cleared by its own control without wiping the other.
+---
+This is the expected behaviour as per epic SV-8785 and the Filters specification version 1.6 (S13-R10, S13-R13, S8-R5).</t>
         </is>
       </c>
       <c r="H94" s="2" t="inlineStr">
         <is>
-          <t>Filters (no Jira epic) (S13-R10 (search and filters are additive); S13-R13 (each cleared independently); S8-R5) [spec v1.6 2026-07-28]</t>
+          <t>SV-8785 [epic] (S13-R10 (search and filters are additive); S13-R13 (each cleared independently); S8-R5) [spec v1.6 2026-07-28]</t>
         </is>
       </c>
       <c r="I94" s="2" t="inlineStr"/>
@@ -5173,12 +5359,14 @@
           <t>1. Sorting and paging keep your search applied - your text stays in the box and the list stays narrowed.
 2. Leaving the page and coming back also keeps your text in the box and the list still narrowed.
 3. The second browser tab starts clean: its Search box is empty and it shows the full list. Each tab keeps its own search.
-4. After closing the browser and coming back, the Search box is empty and the list is unsearched - a typed search is never remembered for next time (your filters, unlike the search, ARE remembered).</t>
+4. After closing the browser and coming back, the Search box is empty and the list is unsearched - a typed search is never remembered for next time (your filters, unlike the search, ARE remembered).
+---
+This is the expected behaviour as per epic SV-8785 and the Filters specification version 1.6 (S13-R14, S13-R25, S13-N4, S10-R5).</t>
         </is>
       </c>
       <c r="H95" s="2" t="inlineStr">
         <is>
-          <t>Filters (no Jira epic) (S13-R14 (retained for the browser tab session); S13-R25 (never stored against the account; each tab independent); S13-N4 (not restored on a later visit); S10-R5) [spec v1.6 2026-07-28]</t>
+          <t>SV-8785 [epic] (S13-R14 (retained for the browser tab session); S13-R25 (never stored against the account; each tab independent); S13-N4 (not restored on a later visit); S10-R5) [spec v1.6 2026-07-28]</t>
         </is>
       </c>
       <c r="I95" s="2" t="inlineStr"/>
@@ -5223,12 +5411,14 @@
           <t>1. The address contains the search term after step 1.
 2. The fresh tab opens with the search box filled and the list already narrowed.
 3. The malformed part is ignored - the page loads cleanly without an error.
-4. A search arriving via a link is view-only, the same as filters from a link - it does not overwrite your own remembered search.</t>
+4. A search arriving via a link is view-only, the same as filters from a link - it does not overwrite your own remembered search.
+---
+This is the expected behaviour as per epic SV-8785 and the Filters specification version 1.6 (S11-R4, S11-R5, S11-N2, S11-R8).</t>
         </is>
       </c>
       <c r="H96" s="2" t="inlineStr">
         <is>
-          <t>Filters (no Jira epic) (S11-R4 (query reflected in the URL); S11-R5 (URL query pre-applied with the control filled); S11-N2 (malformed query ignored with no error); S11-R8 (rationale: no saved value to overwrite)) [spec v1.6 2026-07-28]</t>
+          <t>SV-8796 (S11-R4 (query reflected in the URL); S11-R5 (URL query pre-applied with the control filled); S11-N2 (malformed query ignored with no error); S11-R8 (rationale: no saved value to overwrite)) [spec v1.6 2026-07-28]</t>
         </is>
       </c>
       <c r="I96" s="2" t="inlineStr"/>
@@ -5275,12 +5465,14 @@
 2. The list narrows as you type, same as desktop.
 3. To make room, the page's main button no longer stretches full-width, and pages with two or more small icon buttons collapse them into a single 'more' menu.
 4. The box stretches to fill the space left in the action row instead of staying the narrow desktop size, and every other toolbar button stays visible and in the same place while you search.
-5. There is no extra 'search is on' badge on mobile: with text in it the box simply stays open showing your text, and an empty box closes back to the Search button when you tap elsewhere - exactly as on desktop.</t>
+5. There is no extra 'search is on' badge on mobile: with text in it the box simply stays open showing your text, and an empty box closes back to the Search button when you tap elsewhere - exactly as on desktop.
+---
+This is the expected behaviour as per epic SV-8785 and the Filters specification version 1.6 (S13-R16, S13-R17, S13-R18, S13-R19, S13-R20, S12-R5).</t>
         </is>
       </c>
       <c r="H97" s="2" t="inlineStr">
         <is>
-          <t>Filters (no Jira epic) (S13-R16 (inline expansion with no modal); S13-R17 (field fills the remaining width); S13-R18 (CTA hug width); S13-R19 (2+ icon actions -&gt; "more" kebab); S13-R20 (no active-query indicator); S12-R5) [spec v1.6 2026-07-28]</t>
+          <t>SV-8785 [epic] (S13-R16 (inline expansion with no modal); S13-R17 (field fills the remaining width); S13-R18 (CTA hug width); S13-R19 (2+ icon actions -&gt; "more" kebab); S13-R20 (no active-query indicator); S12-R5) [spec v1.6 2026-07-28]</t>
         </is>
       </c>
       <c r="I97" s="2" t="inlineStr"/>
@@ -5329,12 +5521,14 @@
           <t>1. Every table listed above has its own Search box - no table lost the ability to narrow by text.
 2. Each Search box narrows only its own table; nothing else in the app changes.
 3. Where the table sits inside a dialog (the Work Order Log, the Line Log, the audit log dialog), the Search box is inside that dialog and works there.
-4. The work order Parts tab keeps the local search input it already had - it was deliberately left as it is.</t>
+4. The work order Parts tab keeps the local search input it already had - it was deliberately left as it is.
+---
+This is the expected behaviour as per epic SV-8785 and the Filters specification version 1.6 (S14-R6, S14-R5, S13-R22, S14-N1).</t>
         </is>
       </c>
       <c r="H98" s="2" t="inlineStr">
         <is>
-          <t>Filters (no Jira epic) (S14-R6 (audit: 42 surfaces across 39 components; Work Order Parts excluded); S14-R5 (app-wide sweep); S13-R22 (every table carries a search control); S14-N1 (verify once at the end)) [spec v1.6 2026-07-28]</t>
+          <t>SV-8785 [epic] (S14-R6 (audit: 42 surfaces across 39 components; Work Order Parts excluded); S14-R5 (app-wide sweep); S13-R22 (every table carries a search control); S14-N1 (verify once at the end)) [spec v1.6 2026-07-28]</t>
         </is>
       </c>
       <c r="I98" s="2" t="inlineStr"/>
@@ -5379,12 +5573,14 @@
         <is>
           <t>1. The page list does NOT narrow while you type in the navigation search - only its dropdown of matching records appears.
 2. The same holds on the other pages checked.
-3. Picking a dropdown result still takes you to that record - the navigation search keeps its find-and-open role.</t>
+3. Picking a dropdown result still takes you to that record - the navigation search keeps its find-and-open role.
+---
+This is the expected behaviour as per epic SV-8785 and the Filters specification version 1.6 (S14-R1, S14-R2, S14-R4, S14-R5).</t>
         </is>
       </c>
       <c r="H99" s="2" t="inlineStr">
         <is>
-          <t>Filters (no Jira epic) (S14-R1 (navigational results only); S14-R2 (the page-filtering code path is removed rather than dormant); S14-R4 (the list is left untouched); S14-R5) [spec v1.6 2026-07-28]</t>
+          <t>SV-8799 (S14-R1 (navigational results only); S14-R2 (the page-filtering code path is removed rather than dormant); S14-R4 (the list is left untouched); S14-R5) [spec v1.6 2026-07-28]</t>
         </is>
       </c>
       <c r="I99" s="2" t="inlineStr"/>
@@ -5433,12 +5629,14 @@
 3. Clicking it turns the button into a small text box in the same spot (the design sets it at 180 pixels wide), the typing cursor is already inside it, and the box grows towards the left so the other toolbar buttons do not move.
 4. While the box is empty it shows the magnifier icon and the grey placeholder text 'Type to search'.
 5. As soon as you type, your text shows in a dark grey and a small round x appears at the right-hand end of the box.
-6. A very long sentence does not make the box grow and does not cut the text off - the text scrolls sideways inside the box and the cursor stays where you are typing.</t>
+6. A very long sentence does not make the box grow and does not cut the text off - the text scrolls sideways inside the box and the cursor stays where you are typing.
+---
+This is the expected behaviour as per epic SV-8785 and the Filters specification version 1.6 (S13-R2, S13-R3, S13-R4, S13-R5, S13-R6, S13-R8).</t>
         </is>
       </c>
       <c r="H100" s="2" t="inlineStr">
         <is>
-          <t>Filters (no Jira epic) (S13-R2 (default text button); S13-R3 (hover fill); S13-R4 (expands in place at 180px); S13-R5 (placeholder "Type to search"); S13-R6 (typed text + X-circle clear); S13-R8 (long queries scroll)) [spec v1.6 2026-07-28]</t>
+          <t>SV-8798 (S13-R2 (default text button); S13-R3 (hover fill); S13-R4 (expands in place at 180px); S13-R5 (placeholder "Type to search"); S13-R6 (typed text + X-circle clear); S13-R8 (long queries scroll)) [spec v1.6 2026-07-28]</t>
         </is>
       </c>
       <c r="I100" s="2" t="inlineStr"/>
@@ -5487,12 +5685,14 @@
 2. The matching rows appear in the table you were already looking at; no separate results page, results list or pop-up window opens.
 3. There is no Apply or Submit button anywhere next to the Search box.
 4. Pressing Enter changes nothing that has not already happened - the same rows stay listed and no page reload happens.
-5. Parts Inventory behaves the same way, only it waits a fraction longer before reacting; that longer wait is on purpose because that page carries more data.</t>
+5. Parts Inventory behaves the same way, only it waits a fraction longer before reacting; that longer wait is on purpose because that page carries more data.
+---
+This is the expected behaviour as per epic SV-8785 and the Filters specification version 1.6 (S13-R7, S13-R12).</t>
         </is>
       </c>
       <c r="H101" s="2" t="inlineStr">
         <is>
-          <t>Filters (no Jira epic) (S13-R7 (applies as you type; debounced 300ms; no apply/submit; Enter not required; Inventory 350ms); S13-R12 (results replace the table in place)) [spec v1.6 2026-07-28]</t>
+          <t>SV-8798 (S13-R7 (applies as you type; debounced 300ms; no apply/submit; Enter not required; Inventory 350ms); S13-R12 (results replace the table in place)) [spec v1.6 2026-07-28]</t>
         </is>
       </c>
       <c r="I101" s="2" t="inlineStr"/>
@@ -5539,12 +5739,14 @@
           <t>1. On the All tab only the rows matching your word remain.
 2. On the Estimates tab your word is still in the Search box, and the list shows only Estimates rows that match it - no rows from the other tabs appear.
 3. The Completed tab behaves the same way: your word is still there and only that tab's matching rows are listed.
-4. Clearing the search clears it for all the Work Orders tabs - they share one search - and each tab shows its full list again.</t>
+4. Clearing the search clears it for all the Work Orders tabs - they share one search - and each tab shows its full list again.
+---
+This is the expected behaviour as per epic SV-8785 and the Filters specification version 1.6 (S13-R11, S13-R24).</t>
         </is>
       </c>
       <c r="H102" s="2" t="inlineStr">
         <is>
-          <t>Filters (no Jira epic) (S13-R11 (search applies within the active tab only); S13-R24 (the Work Orders tabs share a single query - views of one dataset)) [spec v1.6 2026-07-28]</t>
+          <t>SV-8798 (S13-R11 (search applies within the active tab only); S13-R24 (the Work Orders tabs share a single query - views of one dataset)) [spec v1.6 2026-07-28]</t>
         </is>
       </c>
       <c r="I102" s="2" t="inlineStr"/>
@@ -5591,12 +5793,14 @@
           <t>1. The second Parts view opens with an empty Search box and its full list - the word you typed on the first view is not carried over.
 2. Going back to the first view brings its own word back and narrows its list again.
 3. Each report tab behaves the same way: a word typed on one tab stays on that tab only, and each tab remembers its own.
-4. No search is ever applied to a table it was not typed on.</t>
+4. No search is ever applied to a table it was not typed on.
+---
+This is the expected behaviour as per epic SV-8785 and the Filters specification version 1.6 (S13-R24, S13-R11, S10-R4).</t>
         </is>
       </c>
       <c r="H103" s="2" t="inlineStr">
         <is>
-          <t>Filters (no Jira epic) (S13-R24 (Reports sub-tabs and Parts views each keep their own query); S13-R11; S10-R4 (each view/tab keeps its own set)) [spec v1.6 2026-07-28]</t>
+          <t>SV-8785 [epic] (S13-R24 (Reports sub-tabs and Parts views each keep their own query); S13-R11; S10-R4 (each view/tab keeps its own set)) [spec v1.6 2026-07-28]</t>
         </is>
       </c>
       <c r="I103" s="2" t="inlineStr"/>
@@ -5642,12 +5846,14 @@
           <t>1. The page opens with the normal list for your own saved filters - the old search word does NOT narrow the list.
 2. The page's own Search box is empty; nothing was carried into it.
 3. No error is shown - the leftover search part in the address is simply ignored. (Whether it also disappears from the address is not important; note what you see.)
-4. After typing in the top-of-screen search and reloading, the list is still not narrowed and nothing about that word was remembered for the list.</t>
+4. After typing in the top-of-screen search and reloading, the list is still not narrowed and nothing about that word was remembered for the list.
+---
+This is the expected behaviour as per epic SV-8785 and the Filters specification version 1.6 (S14-R3, S14-R2, S14-R1).</t>
         </is>
       </c>
       <c r="H104" s="2" t="inlineStr">
         <is>
-          <t>Filters (no Jira epic) (S14-R3 (state / URL parameters / persisted values carrying a global search term into page filtering are removed with it); S14-R2; S14-R1) [spec v1.6 2026-07-28]</t>
+          <t>SV-8799 (S14-R3 (state / URL parameters / persisted values carrying a global search term into page filtering are removed with it); S14-R2; S14-R1) [spec v1.6 2026-07-28]</t>
         </is>
       </c>
       <c r="I104" s="2" t="inlineStr"/>
@@ -5692,12 +5898,14 @@
         <is>
           <t>1. The list stays narrowed by your word - collapsing the filter bar does not cancel the search.
 2. The Search box stays in the toolbar row with your word still showing; it is not tucked away with the filter bar, because the search sits in the toolbar row and the chips sit in the row below.
-3. Expanding the bar again changes nothing about the search or the narrowed list.</t>
+3. Expanding the bar again changes nothing about the search or the narrowed list.
+---
+This is the expected behaviour as per epic SV-8785 and the Filters specification version 1.6 (S13-E1).</t>
         </is>
       </c>
       <c r="H105" s="2" t="inlineStr">
         <is>
-          <t>Filters (no Jira epic) (S13-E1 (a collapsed filter bar keeps an active query applying and the search control stays in the toolbar); §4 Key Decisions (page search is separate from the filter bar)) [spec v1.6 2026-07-28]</t>
+          <t>SV-8798 (S13-E1 (a collapsed filter bar keeps an active query applying and the search control stays in the toolbar); §4 Key Decisions (page search is separate from the filter bar)) [spec v1.6 2026-07-28]</t>
         </is>
       </c>
       <c r="I105" s="2" t="inlineStr"/>
@@ -5741,12 +5949,14 @@
         <is>
           <t>1. The list request includes the active filter selections as request parameters (status values and customer identifiers).
 2. The request succeeds (HTTP 200).
-3. The response contains only work orders matching the filters - the filtering is done by the backend, not just hidden client-side.</t>
+3. The response contains only work orders matching the filters - the filtering is done by the backend, not just hidden client-side.
+---
+This is the expected behaviour as per epic SV-8785 and the Filters specification version 1.6 (S2-R2, S3-R6).</t>
         </is>
       </c>
       <c r="H106" s="2" t="inlineStr">
         <is>
-          <t>Filters (no Jira epic) (S2-R2; S3-R6 (backend view)) [spec v1.6 2026-07-28]</t>
+          <t>SV-8785 [epic] (S2-R2; S3-R6 (backend view)) [spec v1.6 2026-07-28]</t>
         </is>
       </c>
       <c r="I106" s="2" t="inlineStr"/>
@@ -5789,12 +5999,14 @@
         <is>
           <t>1. One request carries both filters together (both statuses and the customer).
 2. The response returns customer A's Estimate and Approved work orders only.
-3. Customer B's work orders are absent - the customer filter and status filter both restrict the result, while the two statuses combine as either-or.</t>
+3. Customer B's work orders are absent - the customer filter and status filter both restrict the result, while the two statuses combine as either-or.
+---
+This is the expected behaviour as per epic SV-8785 and the Filters specification version 1.6 (S2-R2, S3-R6, S8-R3).</t>
         </is>
       </c>
       <c r="H107" s="2" t="inlineStr">
         <is>
-          <t>Filters (no Jira epic) (S2-R2; S3-R6; S8-R3 (backend view)) [spec v1.6 2026-07-28]</t>
+          <t>SV-8785 [epic] (S2-R2; S3-R6; S8-R3 (backend view)) [spec v1.6 2026-07-28]</t>
         </is>
       </c>
       <c r="I107" s="2" t="inlineStr"/>
@@ -5837,12 +6049,14 @@
         <is>
           <t>1. The backend does not fail with a server error (no HTTP 5xx).
 2. The response is a normal, successful list response - the invalid value is ignored or simply matches nothing.
-3. Any still-valid filter values in the same request are applied normally.</t>
+3. Any still-valid filter values in the same request are applied normally.
+---
+This is the expected behaviour as per epic SV-8785 and the Filters specification version 1.6 (S10-N1, S11-R3).</t>
         </is>
       </c>
       <c r="H108" s="2" t="inlineStr">
         <is>
-          <t>Filters (no Jira epic) (S10-N1; S11-R3) [spec v1.6 2026-07-28]</t>
+          <t>SV-8785 [epic] (S10-N1; S11-R3) [spec v1.6 2026-07-28]</t>
         </is>
       </c>
       <c r="I108" s="2" t="inlineStr"/>
@@ -5885,12 +6099,14 @@
       <c r="G109" s="2" t="inlineStr">
         <is>
           <t>1. The backend responds gracefully - no HTTP 5xx / crash; either a normal (unfiltered or empty) list or a clean validation response.
-2. In the browser the page still loads without filters and without an error message, matching the malformed-URL requirement.</t>
+2. In the browser the page still loads without filters and without an error message, matching the malformed-URL requirement.
+---
+This is the expected behaviour as per epic SV-8785 and the Filters specification version 1.6 (S11-N1).</t>
         </is>
       </c>
       <c r="H109" s="2" t="inlineStr">
         <is>
-          <t>Filters (no Jira epic) (S11-N1) [spec v1.6 2026-07-28]</t>
+          <t>SV-8796 (S11-N1) [spec v1.6 2026-07-28]</t>
         </is>
       </c>
       <c r="I109" s="2" t="inlineStr"/>
@@ -5933,12 +6149,14 @@
         <is>
           <t>1. The request succeeds (HTTP 200).
 2. The response contains an empty result set (zero work orders) - an empty match is a normal outcome, not an error.
-3. The page renders the no-results empty state from this response.</t>
+3. The page renders the no-results empty state from this response.
+---
+This is the expected behaviour as per epic SV-8785 and the Filters specification version 1.6 (S8-R3, S2-N3).</t>
         </is>
       </c>
       <c r="H110" s="2" t="inlineStr">
         <is>
-          <t>Filters (no Jira epic) (S8-R3; S2-N3) [spec v1.6 2026-07-28]</t>
+          <t>SV-8785 [epic] (S8-R3; S2-N3) [spec v1.6 2026-07-28]</t>
         </is>
       </c>
       <c r="I110" s="2" t="inlineStr"/>
@@ -5984,12 +6202,14 @@
           <t>1. Changing a filter sends a save (PUT) to the per-user page-preferences service carrying the page's state, and it succeeds (HTTP 200).
 2. On reload the page requests the saved state back (GET, HTTP 200) and applies it - the filters return without you redoing them.
 3. The second user does NOT receive the first user's saved state - each account's saved filters are isolated.
-4. Asking for a never-saved key returns success with an empty value, not an error page.</t>
+4. Asking for a never-saved key returns success with an empty value, not an error page.
+---
+This is the expected behaviour as per epic SV-8785 and the Filters specification version 1.6 (S10-R2, S10-R3).</t>
         </is>
       </c>
       <c r="H111" s="2" t="inlineStr">
         <is>
-          <t>Filters (no Jira epic) (S10-R2 (filters stored server-side against the user account; last write wins); S10-R3 (saved per user)) + tech plan 2026-07-29 s4-1.3 (GET/PUT per-user page preferences) [spec v1.6 2026-07-28]</t>
+          <t>SV-8795 (S10-R2 (filters stored server-side against the user account; last write wins); S10-R3 (saved per user)) + tech plan 2026-07-29 s4-1.3 (GET/PUT per-user page preferences) [spec v1.6 2026-07-28]</t>
         </is>
       </c>
       <c r="I111" s="2" t="inlineStr"/>

</xml_diff>

<commit_message>
chore(sweeper): checkpoint 10 dirty path(s)
Automatic additive checkpoint so no work is lost (Standing Rule 29).
Paths were hash-stable for 20s and passed the secret scan.
Top-level areas: build, testrail-import

  build/filters/branko-answers-2026-08-04/tools
  build/filters/cases
  build/report-suite/rulings-2026-08-04/evidence/ruling3-iv-export
  testrail-import

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AZ5XzKsK9wv7M41cSPaMyg
</commit_message>
<xml_diff>
--- a/testrail-import/filters-v1-testrail-import.xlsx
+++ b/testrail-import/filters-v1-testrail-import.xlsx
@@ -3546,12 +3546,12 @@
           <t>1. On the very first visit the Estimates tab is the selected one, even though All is the FIRST tab in the row (order and default are different on purpose).
 2. After switching to All and returning, the All tab is selected - the app remembers your last-used tab per account.
 ---
-This is the expected behaviour as per epic SV-8785 and the engineering technical plan. No numbered requirement in the Filters specification version 1.6 covers this point yet.</t>
+This is the expected behaviour as per epic SV-8785 and a product owner decision dated 2026-08-04. No numbered requirement in the Filters specification version 1.6 covers this point. That decision is recorded in Branko's answers, in this file: https://docs.google.com/spreadsheets/d/1fkjdt9hoYSGv2MToXUFJ_4tTMzP7a7X2/edit</t>
         </is>
       </c>
       <c r="H61" s="2" t="inlineStr">
         <is>
-          <t>SV-8785 [epic] (no requirement in the ratified spec v1.6 - default/last-used tab is engineering-plan-only - confirmation requested); tech plan 2026-07-29 D10 (default tab = Estimates; last-used tab persists) [spec v1.6 2026-07-28]</t>
+          <t>SV-8785 [epic] (no requirement in spec v1.6 - default/last-used tab is not in the spec; RULED by Branko answers 2026-08-04 Q2 "A - it's fine"); tech plan 2026-07-29 D10 (default tab = Estimates; last-used tab persists) [spec v1.6 2026-07-28]</t>
         </is>
       </c>
       <c r="I61" s="2" t="inlineStr"/>
@@ -4219,12 +4219,12 @@
 2. The row scrolls horizontally - chips that do not fit are reachable by swiping.
 3. An arrow at the right-hand edge shows that the row can be scrolled. (This is what the design shows - if your screen looks different, write down what you actually see and carry on.)
 ---
-This is the expected behaviour as per epic SV-8785 and the Filters specification version 1.6 (S12-R1). The screen described above comes from the agreed design rather than that specification, and a product owner decision is still awaited.</t>
+This is the expected behaviour as per epic SV-8785 and the Filters specification version 1.6 (S12-R1). The screen described above comes from the agreed design rather than that specification, and the product owner approved it on 2026-08-04. That decision is recorded in Branko's answers, in this file: https://docs.google.com/spreadsheets/d/1fkjdt9hoYSGv2MToXUFJ_4tTMzP7a7X2/edit</t>
         </is>
       </c>
       <c r="H74" s="2" t="inlineStr">
         <is>
-          <t>SV-8797 (S12-R1) [spec v1.6 2026-07-28]</t>
+          <t>SV-8797 (S12-R1) [spec v1.6 2026-07-28]; Branko answers 2026-08-04 Q1 - single-filter sheet applies instantly with no Apply button; the combined All Filters sheet keeps its button</t>
         </is>
       </c>
       <c r="I74" s="2" t="inlineStr"/>
@@ -4269,12 +4269,12 @@
 2. It lists the five filters as expandable accordion rows, each with its icon, name and a down arrow: Status, Customer, Lead Technician, Service Advisor, Asset on site.
 3. A sticky blue 'Apply filters' button sits at the bottom of the sheet.
 ---
-This is the expected behaviour as per epic SV-8785 and the Filters specification version 1.6 (S12-R3). The screen described above comes from the agreed design rather than that specification, and a product owner decision is still awaited.</t>
+This is the expected behaviour as per epic SV-8785 and the Filters specification version 1.6 (S12-R3). The screen described above comes from the agreed design rather than that specification, and the product owner approved it on 2026-08-04. That decision is recorded in Branko's answers, in this file: https://docs.google.com/spreadsheets/d/1fkjdt9hoYSGv2MToXUFJ_4tTMzP7a7X2/edit</t>
         </is>
       </c>
       <c r="H75" s="2" t="inlineStr">
         <is>
-          <t>SV-8797 (S12-R3) [spec v1.6 2026-07-28]</t>
+          <t>SV-8797 (S12-R3) [spec v1.6 2026-07-28]; Branko answers 2026-08-04 Q1 - single-filter sheet applies instantly with no Apply button; the combined All Filters sheet keeps its button</t>
         </is>
       </c>
       <c r="I75" s="2" t="inlineStr"/>
@@ -4322,12 +4322,12 @@
 2. After 'Apply filters' the sheet closes and the work order list shows only the ticked statuses.
 3. The reopened sheet's title shows the applied-filter count, for example 'All Filters (1)', and the Status accordion header is highlighted with the selected values ticked.
 ---
-This is the expected behaviour as per epic SV-8785 and the Filters specification version 1.6 (S12-R2, S12-R3, S2-R1). The screen described above comes from the agreed design rather than that specification, and a product owner decision is still awaited.</t>
+This is the expected behaviour as per epic SV-8785 and the Filters specification version 1.6 (S12-R2, S12-R3, S2-R1). The screen described above comes from the agreed design rather than that specification, and the product owner approved it on 2026-08-04. That decision is recorded in Branko's answers, in this file: https://docs.google.com/spreadsheets/d/1fkjdt9hoYSGv2MToXUFJ_4tTMzP7a7X2/edit</t>
         </is>
       </c>
       <c r="H76" s="2" t="inlineStr">
         <is>
-          <t>SV-8785 [epic] (S12-R2; S12-R3; S2-R1) [spec v1.6 2026-07-28]</t>
+          <t>SV-8785 [epic] (S12-R2; S12-R3; S2-R1) [spec v1.6 2026-07-28]; Branko answers 2026-08-04 Q1 - single-filter sheet applies instantly with no Apply button; the combined All Filters sheet keeps its button</t>
         </is>
       </c>
       <c r="I76" s="2" t="inlineStr"/>
@@ -4336,7 +4336,7 @@
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
         <is>
-          <t>Mobile: tapping one chip opens its own sheet with an 'Apply filter' button</t>
+          <t>Mobile: tapping one chip opens its own sheet and applies in real time</t>
         </is>
       </c>
       <c r="B77" s="2" t="inlineStr">
@@ -4362,23 +4362,25 @@
       </c>
       <c r="F77" s="2" t="inlineStr">
         <is>
-          <t>1. Tap the Status chip (not All Filters).
-2. Read the sheet.
-3. Tick a status and tap the bottom button.</t>
+          <t>1. Tap the Status chip (not the 'All Filters' chip).
+2. Read the sheet that opens.
+3. Tick one status and watch the work order list.
+4. Untick it, then tick a different status, and watch the list again.</t>
         </is>
       </c>
       <c r="G77" s="2" t="inlineStr">
         <is>
-          <t>1. A bottom sheet opens for that single filter: its title row shows the filter's icon and name (for example 'Status') with a close (x) button - no accordion list of the other filters.
+          <t>1. A bottom sheet opens for that single filter: its title row shows the filter's icon and name (for example 'Status') with a close (x) button, and no accordion list of the other filters.
 2. The sheet shows only that filter's options (the nine status checkboxes plus 'Clear selection').
-3. The bottom button reads 'Apply filter' (singular); tapping it applies the selection and filters the list.
----
-This is the expected behaviour as per epic SV-8785 and the Filters specification version 1.6 (S12-R2, S12-R3). The screen described above comes from the agreed design rather than that specification, and a product owner decision is still awaited.</t>
+3. There is no 'Apply filter' button. Ticking or unticking a status filters the work order list immediately, the same as on desktop, with no submit step.
+4. The chip's active state and value update live as the selection changes; closing the sheet with the x just dismisses it and keeps the applied filter.
+---
+This is the expected behaviour as per epic SV-8785 and the Filters specification version 1.6 (S12-R2, S12-R3, S2-R6). Branko confirmed this on 2026-08-04 in his answers in this file: https://docs.google.com/spreadsheets/d/1fkjdt9hoYSGv2MToXUFJ_4tTMzP7a7X2/edit</t>
         </is>
       </c>
       <c r="H77" s="2" t="inlineStr">
         <is>
-          <t>SV-8797 (S12-R2; S12-R3) [spec v1.6 2026-07-28] ; individual-chip real-time per S12-R2 + tech-plan 2026-07-29; only the combined All Filters sheet is batch</t>
+          <t>SV-8797 (S12-R2; S12-R3; S2-R6) [spec v1.6 2026-07-28] ; individual-chip real-time per S12-R2 + S2-R6 + tech-plan 2026-07-29; only the combined All Filters sheet is batch; CONFIRMED by Branko answers 2026-08-04 Q1</t>
         </is>
       </c>
       <c r="I77" s="2" t="inlineStr"/>
@@ -4427,12 +4429,12 @@
 3. Removing a tag deselects just that customer.
 4. After 'Apply filters' the list shows only work orders of the remaining selected customers, and the sheet title counts the applied filters (for example 'All Filters (2)').
 ---
-This is the expected behaviour as per epic SV-8785 and the Filters specification version 1.6 (S12-R2, S3-R2/R3/R5). The screen described above comes from the agreed design rather than that specification, and a product owner decision is still awaited.</t>
+This is the expected behaviour as per epic SV-8785 and the Filters specification version 1.6 (S12-R2, S3-R2/R3/R5). The screen described above comes from the agreed design rather than that specification, and the product owner approved it on 2026-08-04. That decision is recorded in Branko's answers, in this file: https://docs.google.com/spreadsheets/d/1fkjdt9hoYSGv2MToXUFJ_4tTMzP7a7X2/edit</t>
         </is>
       </c>
       <c r="H78" s="2" t="inlineStr">
         <is>
-          <t>SV-8785 [epic] (S12-R2; S3-R2/R3/R5) [spec v1.6 2026-07-28]</t>
+          <t>SV-8785 [epic] (S12-R2; S3-R2/R3/R5) [spec v1.6 2026-07-28]; Branko answers 2026-08-04 Q1 - single-filter sheet applies instantly with no Apply button; the combined All Filters sheet keeps its button</t>
         </is>
       </c>
       <c r="I78" s="2" t="inlineStr"/>
@@ -4479,12 +4481,12 @@
 2. The Service Advisor row opens with a 'Search advisor' field and the advisor list.
 3. Applying a selection filters the work order list just like on desktop.
 ---
-This is the expected behaviour as per epic SV-8785 and the Filters specification version 1.6 (S12-R2, S4-R1, S5-R1). The screen described above comes from the agreed design rather than that specification, and a product owner decision is still awaited.</t>
+This is the expected behaviour as per epic SV-8785 and the Filters specification version 1.6 (S12-R2, S4-R1, S5-R1). The screen described above comes from the agreed design rather than that specification, and the product owner approved it on 2026-08-04. That decision is recorded in Branko's answers, in this file: https://docs.google.com/spreadsheets/d/1fkjdt9hoYSGv2MToXUFJ_4tTMzP7a7X2/edit</t>
         </is>
       </c>
       <c r="H79" s="2" t="inlineStr">
         <is>
-          <t>SV-8785 [epic] (S12-R2; S4-R1; S5-R1) [spec v1.6 2026-07-28]</t>
+          <t>SV-8785 [epic] (S12-R2; S4-R1; S5-R1) [spec v1.6 2026-07-28]; Branko answers 2026-08-04 Q1 - single-filter sheet applies instantly with no Apply button; the combined All Filters sheet keeps its button</t>
         </is>
       </c>
       <c r="I79" s="2" t="inlineStr"/>
@@ -4531,12 +4533,12 @@
 2. Only one option can be selected at a time.
 3. After applying, the list shows only work orders matching the chosen on-site state.
 ---
-This is the expected behaviour as per epic SV-8785 and the Filters specification version 1.6 (S12-R2, S6-R1/R2/R3). The screen described above comes from the agreed design rather than that specification, and a product owner decision is still awaited.</t>
+This is the expected behaviour as per epic SV-8785 and the Filters specification version 1.6 (S12-R2, S6-R1/R2/R3). The screen described above comes from the agreed design rather than that specification, and the product owner approved it on 2026-08-04. That decision is recorded in Branko's answers, in this file: https://docs.google.com/spreadsheets/d/1fkjdt9hoYSGv2MToXUFJ_4tTMzP7a7X2/edit</t>
         </is>
       </c>
       <c r="H80" s="2" t="inlineStr">
         <is>
-          <t>SV-8785 [epic] (S12-R2; S6-R1/R2/R3) [spec v1.6 2026-07-28]</t>
+          <t>SV-8785 [epic] (S12-R2; S6-R1/R2/R3) [spec v1.6 2026-07-28]; Branko answers 2026-08-04 Q1 - single-filter sheet applies instantly with no Apply button; the combined All Filters sheet keeps its button</t>
         </is>
       </c>
       <c r="I80" s="2" t="inlineStr"/>
@@ -4582,12 +4584,12 @@
 2. A 'Clear filters' control appears while at least one filter is active.
 3. Using it removes all active filters, the chips return to default and the full list comes back.
 ---
-This is the expected behaviour as per epic SV-8785 and the Filters specification version 1.6 (S12-R2, S7-R1/R3, S8-R1). The screen described above comes from the agreed design rather than that specification, and a product owner decision is still awaited.</t>
+This is the expected behaviour as per epic SV-8785 and the Filters specification version 1.6 (S12-R2, S7-R1/R3, S8-R1). The screen described above comes from the agreed design rather than that specification, and the product owner approved it on 2026-08-04. That decision is recorded in Branko's answers, in this file: https://docs.google.com/spreadsheets/d/1fkjdt9hoYSGv2MToXUFJ_4tTMzP7a7X2/edit</t>
         </is>
       </c>
       <c r="H81" s="2" t="inlineStr">
         <is>
-          <t>SV-8785 [epic] (S12-R2; S7-R1/R3; S8-R1) [spec v1.6 2026-07-28]</t>
+          <t>SV-8785 [epic] (S12-R2; S7-R1/R3; S8-R1) [spec v1.6 2026-07-28]; Branko answers 2026-08-04 Q1 - single-filter sheet applies instantly with no Apply button; the combined All Filters sheet keeps its button</t>
         </is>
       </c>
       <c r="I81" s="2" t="inlineStr"/>
@@ -4742,19 +4744,19 @@
 5. The Credits tab shows three filter buttons: Vendor, Date and Processed by.
 6. Purchase Orders shows four filter buttons: Vendor, Status, Date and Ordered by.
 7. Vendor Invoices shows four filter buttons: Vendor, Invoice date, Date received and Received by.
-8. The Vendors list page shows two filter buttons: Vendor and State/Province. Note: the developers have not been given a design for the Vendors page filters yet, so this page may not have them — write down what you actually see instead of failing the whole test.
+8. The Vendors list page shows two filter buttons: Vendor and State/Province.
 9. On every page above, each filter button shows a small icon, the filter name and a down arrow.
 10. Every Parts list page also shows a Search (magnifier) icon and a filter icon in the toolbar; some pages (for example Inventory) also show a column/layout toggle icon.
 11. Every filter button shown above is a working filter on that page - none of them is display-only.
 12. The choices inside each filter come from your own shop's data (for example your real vendors or categories), so there is no fixed list to compare against - check that the choices you see match the data in your shop.
 13. Still to check on the live build: what the filter icon and the column/layout icon do (the written description does not cover the toolbar icons).
 ---
-This is the expected behaviour as per epic SV-8785 and the Filters specification version 1.6 (§2, §4), which covers this area in its overview and key decisions only. The detailed behaviour above follows a later product owner decision dated 2026-07-31.</t>
+This is the expected behaviour as per epic SV-8785 and the Filters specification version 1.6 (§2, §4), which covers this area in its overview and key decisions only. The detailed behaviour above follows a later product owner decision dated 2026-08-04. That decision is recorded in Branko's answers, in this file: https://docs.google.com/spreadsheets/d/1fkjdt9hoYSGv2MToXUFJ_4tTMzP7a7X2/edit</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr">
         <is>
-          <t>SV-8785 [epic] (spec v1.6 §2 Feature Overview -&gt; Parts Filters; §4 Key Decisions -&gt; "Context-specific filter sets on Parts and Reports" + "Multi-select where it makes sense"); Branko answers 2026-07-31 Q2/Q3/Q5/Q7; Figma 11884-16885</t>
+          <t>SV-8785 [epic] (spec v1.6 §2 Parts Filters; §4 context-specific filter sets + multi-select); Branko answers 2026-07-31 Q2/Q3/Q5/Q7 + 2026-08-04 Q3 (Vendors design exists Figma 11903-10461) + Q8 (Part Sales chips); Figma 11884-16885</t>
         </is>
       </c>
       <c r="I84" s="2" t="inlineStr"/>
@@ -4958,12 +4960,12 @@
 2. Every choice each of those filters offered before is still available inside the new button.
 3. If any filter or choice is missing, write down exactly which page, which filter and which choice - that is a bug worth reporting.
 ---
-This is the expected behaviour as per epic SV-8785 and the Filters specification version 1.6 (§2), which covers this area in its overview and key decisions only. The detailed behaviour above follows a later product owner decision dated 2026-07-31.</t>
+This is the expected behaviour as per epic SV-8785 and the Filters specification version 1.6 (§2), which covers this area in its overview and key decisions only. The detailed behaviour above follows a later product owner decision dated 2026-08-04. That decision is recorded in Branko's answers, in this file: https://docs.google.com/spreadsheets/d/1fkjdt9hoYSGv2MToXUFJ_4tTMzP7a7X2/edit</t>
         </is>
       </c>
       <c r="H88" s="2" t="inlineStr">
         <is>
-          <t>SV-8785 [epic] (spec v1.6 §2 Parts Filters + Reports Filters); Branko answers 2026-07-31 Q3 ("support all the filters we have right now in the app as well as all choices per filter"); tech plan 2026-07-29 rollout rule</t>
+          <t>SV-8785 [epic] (spec v1.6 §2 Parts Filters + Reports Filters); Branko answers 2026-07-31 Q3 + 2026-08-04 Q8 ("we should have all filters we support now per each page plus we should add new ones"); tech plan 2026-07-29 rollout rule</t>
         </is>
       </c>
       <c r="I88" s="2" t="inlineStr"/>
@@ -5144,12 +5146,12 @@
 2. The choices inside each filter come from your own shop's data (for example your real vendors or categories), so there is no fixed list to compare against - check that the choices you see match the data in your shop.
 3. Write down the choices you actually see behind each of these six buttons. They have not been written down anywhere yet, so your list becomes the record.
 ---
-This is the expected behaviour as per epic SV-8785 and the Filters specification version 1.6 (§2, §4), which covers this area in its overview and key decisions only. The detailed behaviour above follows a later product owner decision dated 2026-07-31.</t>
+This is the expected behaviour as per epic SV-8785 and the Filters specification version 1.6 (§2, §4), which covers this area in its overview and key decisions only. The detailed behaviour above follows a later product owner decision dated 2026-07-31. Branko confirmed this on 2026-08-04 in his answers in this file: https://docs.google.com/spreadsheets/d/1fkjdt9hoYSGv2MToXUFJ_4tTMzP7a7X2/edit</t>
         </is>
       </c>
       <c r="H91" s="2" t="inlineStr">
         <is>
-          <t>SV-8785 [epic] (spec v1.6 §2 Reports Filters; §4 "Multi-select where it makes sense"); Branko answers 2026-07-31 Q3/Q5 + Q4 (pointer only - the 6 new types are not enumerated in v1.6; see DELTAS.md F1); Figma 11903-10573</t>
+          <t>SV-8785 [epic] (spec v1.6 §2 Reports Filters; §4 "Multi-select where it makes sense"); Branko answers 2026-07-31 Q3/Q5 + 2026-08-04 Q8 ("We do not have list of all filter items" - confirms no option list exists); Figma 11903-10573</t>
         </is>
       </c>
       <c r="I91" s="2" t="inlineStr"/>

</xml_diff>

<commit_message>
Filters deliverables regenerated after the marker pass; Schedule halt recorded
Local case source re-synced FROM LIVE first: exactly 102 'expected' fields moved,
matching the 102 writes and nothing else. Shredding guard PASSED. Import differs
from the previous version in one column, 102 rows, only by the appended marker.
All four counts = 110 and set-equal both ways; id-map came back byte-identical
(0 blanks, refs 110/110); import header sha256 matches all 5 peer imports.

Also records why Schedule was not written and why 8 Filters phone cases were left
alone (Branko closed SV-8825 at 05:18 UTC today).

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AZ5XzKsK9wv7M41cSPaMyg
</commit_message>
<xml_diff>
--- a/testrail-import/filters-v1-testrail-import.xlsx
+++ b/testrail-import/filters-v1-testrail-import.xlsx
@@ -528,13 +528,15 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>&lt;ol&gt;
+          <t xml:space="preserve">&lt;ol&gt;
 &lt;li&gt;A filter bar is visible directly below the tab row and above the work order table.&lt;/li&gt;
 &lt;li&gt;The filter bar is shown by default (expanded) without having to turn anything on.&lt;/li&gt;
 &lt;/ol&gt;
 Known and accepted: on the build tested the filter buttons sit on the same row as the tabs instead of on their own row below them. The product behaves this way on purpose for now. Do not raise this as a new problem.
 ---
-This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S1-R1).</t>
+This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S1-R1).
+AUTOMATION: READY - EXPECT FAIL (SV-8843 - closed as accepted, will not be fixed)
+</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -581,11 +583,13 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>1. Exactly five filter chips appear, in this order: Status, Customer, Lead Technician, Service Advisor, Asset on Site.
+          <t xml:space="preserve">1. Exactly five filter chips appear, in this order: Status, Customer, Lead Technician, Service Advisor, Asset on Site.
 2. Each chip shows the filter name and a down arrow (chevron) indicating it opens a dropdown.
 3. Each chip shows only the filter name and the arrow - there is no picture icon in front of the name.
 ---
-This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S1-R2, S1-R3). Note: the design frame also draws a small picture icon in front of each filter name; the specification asks only for the name and the arrow, and the build matches the specification, so this test follows the specification and the build.</t>
+This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S1-R2, S1-R3). Note: the design frame also draws a small picture icon in front of each filter name; the specification asks only for the name and the arrow, and the build matches the specification, so this test follows the specification and the build.
+AUTOMATION: READY
+</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -631,11 +635,13 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>1. The filter bar is still shown - it does not disappear on this tab.
+          <t xml:space="preserve">1. The filter bar is still shown - it does not disappear on this tab.
 2. The Customer, Lead Technician, Service Advisor and Asset on Site chips are all displayed and usable.
 3. The Status chip is not shown on this tab at all - only four chips appear.
 ---
-This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S1-N1, S9-R2). Note: an earlier answer of 2026-07-17 and the design frame both show the Status button greyed out and pre-filled on this tab; the specification and the build both hide it, and the specification is the newer source, so this test follows the specification and the build.</t>
+This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S1-N1, S9-R2). Note: an earlier answer of 2026-07-17 and the design frame both show the Status button greyed out and pre-filled on this tab; the specification and the build both hide it, and the specification is the newer source, so this test follows the specification and the build.
+AUTOMATION: READY
+</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
@@ -689,14 +695,16 @@
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>&lt;ol&gt;
+          <t xml:space="preserve">&lt;ol&gt;
 &lt;li&gt;A dropdown panel opens under the Status chip.&lt;/li&gt;
 &lt;li&gt;It lists all nine statuses as checkboxes, in this order: Estimate, Approved, In progress, Review, Complete, Invoiced, Paid, Declined, Imported.&lt;/li&gt;
 &lt;li&gt;All checkboxes are unticked (nothing selected yet).&lt;/li&gt;
 &lt;li&gt;A 'Clear Selection' action is shown at the bottom of the dropdown.&lt;/li&gt;
 &lt;/ol&gt;
 ---
-This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S2-R1, S2-R4).</t>
+This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S2-R1, S2-R4).
+AUTOMATION: READY
+</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
@@ -744,11 +752,13 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>1. The ticked checkbox appears filled (checked).
+          <t xml:space="preserve">1. The ticked checkbox appears filled (checked).
 2. The table updates immediately to show only work orders in the selected status - there is no confirm or apply button on desktop.
 3. Work orders in other statuses are no longer listed.
 ---
-This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S2-R2, S2-R3, S2-R6).</t>
+This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S2-R2, S2-R3, S2-R6).
+AUTOMATION: READY
+</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
@@ -796,12 +806,14 @@
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>1. Every ticked status shows a filled checkbox.
+          <t xml:space="preserve">1. Every ticked status shows a filled checkbox.
 2. The table shows work orders whose status matches ANY of the ticked statuses (both Estimate and Approved rows appear).
 3. Work orders in statuses that are not ticked are hidden.
 4. There is no limit on how many statuses you can tick.
 ---
-This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S2-R2).</t>
+This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S2-R2).
+AUTOMATION: READY
+</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
@@ -849,11 +861,13 @@
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>1. All status checkboxes become unticked.
+          <t xml:space="preserve">1. All status checkboxes become unticked.
 2. The Status filter is removed and the table returns to showing work orders of every status.
 3. Only the Status filter is affected - any other active filters stay applied.
 ---
-This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S2-R4, S8-R2).</t>
+This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S2-R4, S8-R2).
+AUTOMATION: READY
+</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
@@ -900,11 +914,13 @@
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>1. The dropdown closes.
+          <t xml:space="preserve">1. The dropdown closes.
 2. The ticked statuses stay selected - the Status chip stays in its active state showing the selection.
 3. The table stays filtered by the selected statuses.
 ---
-This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S2-R5).</t>
+This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S2-R5).
+AUTOMATION: READY
+</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
@@ -952,11 +968,13 @@
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>1. The table shows no rows.
+          <t xml:space="preserve">1. The table shows no rows.
 2. An empty state is displayed saying no results were found for the current filters (see the Empty State cases for its full content).
 3. The app does not show an error.
 ---
-This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S2-N3, S8-R3).</t>
+This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S2-N3, S8-R3).
+AUTOMATION: READY
+</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
@@ -1005,12 +1023,14 @@
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>1. The table switches to showing imported work orders only.
+          <t xml:space="preserve">1. The table switches to showing imported work orders only.
 2. While Imported is ticked, the other filter chips are greyed out and cannot be used.
 3. Imported cannot be combined with other statuses - selecting it works alone.
 4. Unticking Imported re-enables the other chips and the normal list returns.
 ---
-This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S2-R7, S2-N4).</t>
+This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S2-R7, S2-N4).
+AUTOMATION: READY
+</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
@@ -1064,14 +1084,16 @@
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>&lt;ol&gt;
+          <t xml:space="preserve">&lt;ol&gt;
 &lt;li&gt;A dropdown panel opens under the Customer chip.&lt;/li&gt;
 &lt;li&gt;A search box with the placeholder 'Search' is at the top of the panel. Click it before you type - it is not focused for you automatically.&lt;/li&gt;
 &lt;li&gt;Below it is a scrollable list of customer names.&lt;/li&gt;
 &lt;li&gt;A 'Clear Selection' action is shown at the bottom of the panel.&lt;/li&gt;
 &lt;/ol&gt;
 ---
-This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S3-R1).</t>
+This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S3-R1).
+AUTOMATION: READY
+</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
@@ -1118,11 +1140,13 @@
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>1. The customer list narrows as you type, showing only names that match what you entered.
+          <t xml:space="preserve">1. The customer list narrows as you type, showing only names that match what you entered.
 2. Customers that do not match are removed from the list.
 3. Deleting the text brings the full list back.
 ---
-This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S3-R2).</t>
+This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S3-R2).
+AUTOMATION: READY
+</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
@@ -1176,14 +1200,16 @@
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>&lt;ol&gt;
+          <t xml:space="preserve">&lt;ol&gt;
 &lt;li&gt;Each selected customer appears as a tag (small chip) with an x in the input area at the top of the dropdown.&lt;/li&gt;
 &lt;li&gt;Each selected customer's row in the list shows a checkmark on the right.&lt;/li&gt;
 &lt;li&gt;Long customer names on tags are shortened with an ellipsis (for example 'Texas Truck And Aut...').&lt;/li&gt;
 &lt;li&gt;You can keep selecting as many customers as needed - there is no selection limit.&lt;/li&gt;
 &lt;/ol&gt;
 ---
-This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S3-R3, S3-R4).</t>
+This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S3-R3, S3-R4).
+AUTOMATION: READY
+</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
@@ -1230,12 +1256,14 @@
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>1. That customer's tag disappears from the input area.
+          <t xml:space="preserve">1. That customer's tag disappears from the input area.
 2. The checkmark next to that customer in the list is removed.
 3. The other selected customers keep their tags and checkmarks.
 4. The table updates to no longer include that customer's work orders.
 ---
-This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S3-R5).</t>
+This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S3-R5).
+AUTOMATION: READY
+</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
@@ -1282,11 +1310,13 @@
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>1. The table shows only work orders whose customer is one of the two selected customers.
+          <t xml:space="preserve">1. The table shows only work orders whose customer is one of the two selected customers.
 2. Work orders belonging to any other customer are hidden.
 3. The table updates in real time as you make the selections (no apply button on desktop).
 ---
-This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S3-R6, S2-R6).</t>
+This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S3-R6, S2-R6).
+AUTOMATION: READY
+</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
@@ -1334,12 +1364,14 @@
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>1. All customer tags are removed from the input area.
+          <t xml:space="preserve">1. All customer tags are removed from the input area.
 2. All checkmarks in the list are removed.
 3. The Customer filter is removed and the table shows work orders of all customers again.
 4. Other active filters (if any) are not affected.
 ---
-This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S3-R7, S8-R2).</t>
+This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S3-R7, S8-R2).
+AUTOMATION: READY
+</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
@@ -1386,11 +1418,13 @@
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>1. The dropdown closes when you click outside it.
+          <t xml:space="preserve">1. The dropdown closes when you click outside it.
 2. The Customer chip stays in the active (blue) state showing the selection and the table stays filtered.
 3. When reopened, the selected customers' tags are still visible in the input area.
 ---
-This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S3-R8).</t>
+This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S3-R8).
+AUTOMATION: READY
+</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
@@ -1442,13 +1476,15 @@
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>&lt;ol&gt;
+          <t xml:space="preserve">&lt;ol&gt;
 &lt;li&gt;The list shows a message saying there are no results (instead of an empty gap).&lt;/li&gt;
 &lt;li&gt;The app does not show an error.&lt;/li&gt;
 &lt;li&gt;Clearing the search text brings the customer list back.&lt;/li&gt;
 &lt;/ol&gt;
 ---
-This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S3-N1).</t>
+This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S3-N1).
+AUTOMATION: READY
+</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
@@ -1496,11 +1532,13 @@
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>1. The customer with no work orders IS shown in the filter list (they are not hidden).
+          <t xml:space="preserve">1. The customer with no work orders IS shown in the filter list (they are not hidden).
 2. After selecting only that customer, the table shows no rows and the filtered empty state is displayed.
 3. No error is shown.
 ---
-This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S3-E1, S3-N2, S8-R3).</t>
+This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S3-E1, S3-N2, S8-R3).
+AUTOMATION: READY
+</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
@@ -1553,14 +1591,16 @@
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>&lt;ol&gt;
+          <t xml:space="preserve">&lt;ol&gt;
 &lt;li&gt;A dropdown panel opens under the Lead Technician chip.&lt;/li&gt;
 &lt;li&gt;A search input with the placeholder 'Search' is at the top.&lt;/li&gt;
 &lt;li&gt;Below it is a scrollable list of technician names.&lt;/li&gt;
 &lt;li&gt;A 'Clear Selection' action is shown at the bottom.&lt;/li&gt;
 &lt;/ol&gt;
 ---
-This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S4-R1).</t>
+This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S4-R1).
+AUTOMATION: READY
+</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
@@ -1606,10 +1646,12 @@
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>1. The technician list narrows to only the names matching what you typed.
+          <t xml:space="preserve">1. The technician list narrows to only the names matching what you typed.
 2. Deleting the text brings the full list back.
 ---
-This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S4-R2).</t>
+This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S4-R2).
+AUTOMATION: READY
+</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
@@ -1656,12 +1698,14 @@
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>1. Selected technicians show a checkmark on the row, and as a small removable tag above the list in the list.
+          <t xml:space="preserve">1. Selected technicians show a checkmark on the row, and as a small removable tag above the list in the list.
 2. The table shows only work orders where one of the selected technicians is assigned as the LEAD technician.
 3. A work order where the technician is assigned only in a non-lead role does not appear.
 4. The table updates in real time as you select.
 ---
-This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S4-R3, S4-R4).</t>
+This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S4-R3, S4-R4).
+AUTOMATION: READY
+</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">
@@ -1708,11 +1752,13 @@
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>1. All technician selections are removed (checkboxes unticked).
+          <t xml:space="preserve">1. All technician selections are removed (checkboxes unticked).
 2. The Lead Technician filter no longer restricts the table.
 3. Other active filters are not affected.
 ---
-This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S4-R5, S8-R2).</t>
+This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S4-R5, S8-R2).
+AUTOMATION: READY
+</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr">
@@ -1758,10 +1804,12 @@
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>1. The dropdown closes.
+          <t xml:space="preserve">1. The dropdown closes.
 2. The selection stays applied - the chip stays active and the table stays filtered.
 ---
-This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S4-R6).</t>
+This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S4-R6).
+AUTOMATION: READY
+</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
@@ -1808,10 +1856,12 @@
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>1. The table shows no rows and the filtered empty state is displayed.
+          <t xml:space="preserve">1. The table shows no rows and the filtered empty state is displayed.
 2. No error is shown.
 ---
-This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S4-N1, S8-R3).</t>
+This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S4-N1, S8-R3).
+AUTOMATION: READY
+</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr">
@@ -1859,10 +1909,12 @@
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>1. The deactivated technician is NOT shown in the filter list.
+          <t xml:space="preserve">1. The deactivated technician is NOT shown in the filter list.
 2. Active technicians are still listed normally.
 ---
-This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S4-E1).</t>
+This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S4-E1).
+AUTOMATION: READY
+</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr">
@@ -1915,14 +1967,16 @@
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>&lt;ol&gt;
+          <t xml:space="preserve">&lt;ol&gt;
 &lt;li&gt;A dropdown panel opens under the Service Advisor chip.&lt;/li&gt;
 &lt;li&gt;A search input with the placeholder 'Search' is at the top.&lt;/li&gt;
 &lt;li&gt;Below it is a scrollable list of advisor names.&lt;/li&gt;
 &lt;li&gt;A 'Clear Selection' action is shown at the bottom.&lt;/li&gt;
 &lt;/ol&gt;
 ---
-This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S5-R1).</t>
+This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S5-R1).
+AUTOMATION: READY
+</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr">
@@ -1968,10 +2022,12 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>1. The advisor list narrows to only the names matching what you typed.
+          <t xml:space="preserve">1. The advisor list narrows to only the names matching what you typed.
 2. Deleting the text brings the full list back.
 ---
-This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S5-R2).</t>
+This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S5-R2).
+AUTOMATION: READY
+</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -2018,11 +2074,13 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>1. Selected advisors show a checkmark on the row, and as a small removable tag above the list in the list.
+          <t xml:space="preserve">1. Selected advisors show a checkmark on the row, and as a small removable tag above the list in the list.
 2. The table shows only work orders assigned to any of the selected advisors.
 3. The table updates in real time as you select.
 ---
-This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S5-R3, S5-R4).</t>
+This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S5-R3, S5-R4).
+AUTOMATION: READY
+</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -2069,11 +2127,13 @@
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>1. All advisor selections are removed.
+          <t xml:space="preserve">1. All advisor selections are removed.
 2. The Service Advisor filter no longer restricts the table.
 3. Other active filters are not affected.
 ---
-This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S5-R5, S8-R2).</t>
+This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S5-R5, S8-R2).
+AUTOMATION: READY
+</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr">
@@ -2119,10 +2179,12 @@
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>1. The dropdown closes.
+          <t xml:space="preserve">1. The dropdown closes.
 2. The selection stays applied - the chip stays active and the table stays filtered.
 ---
-This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S5-R6).</t>
+This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S5-R6).
+AUTOMATION: READY
+</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr">
@@ -2169,10 +2231,12 @@
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>1. The table shows no rows and the filtered empty state is displayed.
+          <t xml:space="preserve">1. The table shows no rows and the filtered empty state is displayed.
 2. No error is shown.
 ---
-This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S5-N1, S8-R3).</t>
+This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S5-N1, S8-R3).
+AUTOMATION: READY
+</t>
         </is>
       </c>
       <c r="H33" s="2" t="inlineStr">
@@ -2220,10 +2284,12 @@
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>1. The deactivated advisor is NOT shown in the filter list.
+          <t xml:space="preserve">1. The deactivated advisor is NOT shown in the filter list.
 2. Active advisors are still listed normally.
 ---
-This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S5-E1).</t>
+This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S5-E1).
+AUTOMATION: READY
+</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr">
@@ -2269,12 +2335,14 @@
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>1. A small dropdown panel opens under the Asset on Site chip.
+          <t xml:space="preserve">1. A small dropdown panel opens under the Asset on Site chip.
 2. It contains exactly two options: Yes and No.
 3. A 'Clear Selection' action is shown at the bottom.
 4. It is a dropdown (like the other filters), not an on/off toggle.
 ---
-This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S6-R1).</t>
+This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S6-R1).
+AUTOMATION: READY
+</t>
         </is>
       </c>
       <c r="H35" s="2" t="inlineStr">
@@ -2321,10 +2389,12 @@
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>1. The table shows only work orders whose asset is currently on site.
+          <t xml:space="preserve">1. The table shows only work orders whose asset is currently on site.
 2. Work orders whose asset is not on site are hidden.
 ---
-This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S6-R2).</t>
+This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S6-R2).
+AUTOMATION: READY
+</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr">
@@ -2371,11 +2441,13 @@
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>1. No becomes the selected option and Yes is deselected automatically - only one option can be selected at a time.
+          <t xml:space="preserve">1. No becomes the selected option and Yes is deselected automatically - only one option can be selected at a time.
 2. The table switches to showing only the not-on-site work orders.
 3. The chip shows the currently selected value.
 ---
-This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S6-R3).</t>
+This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S6-R3).
+AUTOMATION: READY
+</t>
         </is>
       </c>
       <c r="H37" s="2" t="inlineStr">
@@ -2421,11 +2493,13 @@
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>1. The selection is removed and the chip returns to its default (inactive) state.
+          <t xml:space="preserve">1. The selection is removed and the chip returns to its default (inactive) state.
 2. The table shows work orders regardless of on-site status again.
 3. Other active filters are not affected.
 ---
-This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S6-R4, S8-R2).</t>
+This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S6-R4, S8-R2).
+AUTOMATION: READY
+</t>
         </is>
       </c>
       <c r="H38" s="2" t="inlineStr">
@@ -2471,10 +2545,12 @@
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>1. The dropdown closes.
+          <t xml:space="preserve">1. The dropdown closes.
 2. The Yes selection stays applied - the chip stays active and the table stays filtered.
 ---
-This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S6-R5).</t>
+This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S6-R5).
+AUTOMATION: READY
+</t>
         </is>
       </c>
       <c r="H39" s="2" t="inlineStr">
@@ -2521,10 +2597,12 @@
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>1. The table shows no rows and the filtered empty state is displayed.
+          <t xml:space="preserve">1. The table shows no rows and the filtered empty state is displayed.
 2. No error is shown.
 ---
-This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S6-N1, S8-R3).</t>
+This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S6-N1, S8-R3).
+AUTOMATION: READY
+</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr">
@@ -2572,11 +2650,13 @@
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>1. Only work orders whose asset is NOT on site remain in the list.
+          <t xml:space="preserve">1. Only work orders whose asset is NOT on site remain in the list.
 2. Every work order with the asset on site is excluded.
 3. The chip shows the active No selection.
 ---
-This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S6-R2).</t>
+This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S6-R2).
+AUTOMATION: READY
+</t>
         </is>
       </c>
       <c r="H41" s="2" t="inlineStr">
@@ -2622,11 +2702,13 @@
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>1. The Status chip changes to an active/highlighted look (blue pill).
+          <t xml:space="preserve">1. The Status chip changes to an active/highlighted look (blue pill).
 2. The chip displays the selected value (for example 'Status: Estimate').
 3. The other chips stay in their default state.
 ---
-This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S7-R1).</t>
+This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S7-R1).
+AUTOMATION: READY
+</t>
         </is>
       </c>
       <c r="H42" s="2" t="inlineStr">
@@ -2672,10 +2754,12 @@
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>1. The chip lists the selected values starting with the first one and shortens the label when it gets too long (the design shows 'Status: Estimate, In progress, Approved...').
+          <t xml:space="preserve">1. The chip lists the selected values starting with the first one and shortens the label when it gets too long (the design shows 'Status: Estimate, In progress, Approved...').
 2. The chip stays a single compact pill - it does not grow to show every value in full.
 ---
-This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S7-R2).</t>
+This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S7-R2).
+AUTOMATION: READY
+</t>
         </is>
       </c>
       <c r="H43" s="2" t="inlineStr">
@@ -2723,11 +2807,13 @@
       </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>1. With no filters active, no 'Clear Filters' button/link is shown (there is nothing to click).
+          <t xml:space="preserve">1. With no filters active, no 'Clear Filters' button/link is shown (there is nothing to click).
 2. As soon as one filter is active, a blue 'Clear Filters' link appears at the right end of the chip row.
 3. When the last active filter is removed, 'Clear Filters' disappears again.
 ---
-This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S7-R3, S7-N1, S8-N1).</t>
+This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S7-R3, S7-N1, S8-N1).
+AUTOMATION: READY
+</t>
         </is>
       </c>
       <c r="H44" s="2" t="inlineStr">
@@ -2775,12 +2861,14 @@
       </c>
       <c r="G45" s="2" t="inlineStr">
         <is>
-          <t>1. Every active filter is cleared in one click.
+          <t xml:space="preserve">1. Every active filter is cleared in one click.
 2. All chips return to their default (inactive) look with no values shown.
 3. The table shows the full unfiltered list again (no text is in the page Search box, so nothing else is narrowing it).
 4. The 'Clear Filters' link disappears.
 ---
-This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S8-R1, S13-R13).</t>
+This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S8-R1, S13-R13).
+AUTOMATION: READY
+</t>
         </is>
       </c>
       <c r="H45" s="2" t="inlineStr">
@@ -2827,11 +2915,13 @@
       </c>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t>1. Only the Status filter is cleared - its chip returns to default.
+          <t xml:space="preserve">1. Only the Status filter is cleared - its chip returns to default.
 2. The Customer filter stays selected and active (blue) and keeps filtering the table.
 3. 'Clear Filters' remains visible because a filter is still active.
 ---
-This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S8-R2).</t>
+This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S8-R2).
+AUTOMATION: READY
+</t>
         </is>
       </c>
       <c r="H46" s="2" t="inlineStr">
@@ -2879,11 +2969,13 @@
       </c>
       <c r="G47" s="2" t="inlineStr">
         <is>
-          <t>1. Only customer A's Estimate work order is shown.
+          <t xml:space="preserve">1. Only customer A's Estimate work order is shown.
 2. Customer A's Approved work order is hidden (wrong status) and customer B's Estimate work order is hidden (wrong customer) - each additional filter narrows the result further.
 3. Both chips are in the active state and 'Clear Filters' is visible.
 ---
-This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S8-R3).</t>
+This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S8-R3).
+AUTOMATION: READY
+</t>
         </is>
       </c>
       <c r="H47" s="2" t="inlineStr">
@@ -2930,11 +3022,13 @@
       </c>
       <c r="G48" s="2" t="inlineStr">
         <is>
-          <t>1. The filter bar row is hidden.
+          <t xml:space="preserve">1. The filter bar row is hidden.
 2. The work order table moves up and uses the reclaimed vertical space.
 3. The filter icon shows a pressed/active look while the bar is collapsed.
 ---
-This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S1-R4, S1-R5).</t>
+This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S1-R4, S1-R5).
+AUTOMATION: READY
+</t>
         </is>
       </c>
       <c r="H48" s="2" t="inlineStr">
@@ -2981,12 +3075,14 @@
       </c>
       <c r="G49" s="2" t="inlineStr">
         <is>
-          <t>1. The filter bar reappears below the tab row.
+          <t xml:space="preserve">1. The filter bar reappears below the tab row.
 2. The previously selected filters are still shown on their chips in the active (blue) state - nothing was lost while collapsed.
 3. The 'Clear Filters' link is still shown at the right end of the chip row.
 Known and accepted: on the build tested collapsing the bar does not move the table up, because the buttons share the tab row. The product behaves this way on purpose for now. Do not raise this as a new problem.
 ---
-This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S1-R6).</t>
+This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S1-R6).
+AUTOMATION: READY - EXPECT FAIL (SV-8843 - closed as accepted, will not be fixed)
+</t>
         </is>
       </c>
       <c r="H49" s="2" t="inlineStr">
@@ -3034,10 +3130,12 @@
       </c>
       <c r="G50" s="2" t="inlineStr">
         <is>
-          <t>1. After step 2 the filter bar is still collapsed (your choice was remembered).
+          <t xml:space="preserve">1. After step 2 the filter bar is still collapsed (your choice was remembered).
 2. After step 4 the filter bar is expanded again when you return - whichever state you left it in is restored.
 ---
-This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S1-R7, S10-R1).</t>
+This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S1-R7, S10-R1).
+AUTOMATION: READY
+</t>
         </is>
       </c>
       <c r="H50" s="2" t="inlineStr">
@@ -3084,10 +3182,12 @@
       </c>
       <c r="G51" s="2" t="inlineStr">
         <is>
-          <t>1. After step 1 the filter icon shows no special indicator (only its normal pressed look).
+          <t xml:space="preserve">1. After step 1 the filter icon shows no special indicator (only its normal pressed look).
 2. After step 3 the filter icon shows a visual indicator (filters icon in primary blue) signalling that active filters are in effect while the bar is hidden.
 ---
-This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S7-R4, S7-N2).</t>
+This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S7-R4, S7-N2).
+AUTOMATION: READY
+</t>
         </is>
       </c>
       <c r="H51" s="2" t="inlineStr">
@@ -3134,10 +3234,12 @@
       </c>
       <c r="G52" s="2" t="inlineStr">
         <is>
-          <t>1. The table content does not change when the bar collapses - it still shows only the work orders matching the active filters.
+          <t xml:space="preserve">1. The table content does not change when the bar collapses - it still shows only the work orders matching the active filters.
 2. Hiding the bar only hides the chips; it does not remove or pause the filtering.
 ---
-This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S7-R5).</t>
+This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S7-R5).
+AUTOMATION: READY
+</t>
         </is>
       </c>
       <c r="H52" s="2" t="inlineStr">
@@ -3184,12 +3286,14 @@
       </c>
       <c r="G53" s="2" t="inlineStr">
         <is>
-          <t>1. The table body is replaced by an empty state (not just a bare empty grid).
+          <t xml:space="preserve">1. The table body is replaced by an empty state (not just a bare empty grid).
 2. The empty state shows a message indicating no results were found for the current filters.
 3. No error message or broken layout appears.
 Known and accepted: when only a search is active the message still says "filters" and the only link offered is Clear Filters. The product behaves this way on purpose for now. Do not raise this as a new problem.
 ---
-This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S8-R3).</t>
+This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S8-R3).
+AUTOMATION: READY - EXPECT FAIL (SV-8847 - closed as accepted, will not be fixed)
+</t>
         </is>
       </c>
       <c r="H53" s="2" t="inlineStr">
@@ -3237,12 +3341,14 @@
       </c>
       <c r="G54" s="2" t="inlineStr">
         <is>
-          <t>1. The empty state includes a prompt or link to clear the filters.
+          <t xml:space="preserve">1. The empty state includes a prompt or link to clear the filters.
 2. Clicking it removes the active filters and the full work order list is shown again (with no text in the Search box, nothing else is narrowing the list).
 3. The chips return to their default state.
 Known and accepted: the empty screen offers no way to clear the search on its own. The product behaves this way on purpose for now. Do not raise this as a new problem.
 ---
-This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S8-R4, S8-R5).</t>
+This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S8-R4, S8-R5).
+AUTOMATION: READY - EXPECT FAIL (SV-8847 - closed as accepted, will not be fixed)
+</t>
         </is>
       </c>
       <c r="H54" s="2" t="inlineStr">
@@ -3291,12 +3397,14 @@
       </c>
       <c r="G55" s="2" t="inlineStr">
         <is>
-          <t>1. The table is replaced by a no-results message that mentions BOTH the current filters and the search - not the filters alone.
+          <t xml:space="preserve">1. The table is replaced by a no-results message that mentions BOTH the current filters and the search - not the filters alone.
 2. The message offers a way to clear the filters and, because a search is active, a separate way to clear the search.
 3. Clearing the search brings back the list as narrowed by the filter only - the filter is still on.
 4. Clearing the filters leaves your typed word in the box and still applied - each is cleared on its own without wiping the other.
 ---
-This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S8-R3, S8-R4, S8-R5, S13-N1, S13-N2).</t>
+This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S8-R3, S8-R4, S8-R5, S13-N1, S13-N2).
+AUTOMATION: READY
+</t>
         </is>
       </c>
       <c r="H55" s="2" t="inlineStr">
@@ -3342,10 +3450,12 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>1. All five chips are shown: Status, Customer, Lead Technician, Service Advisor, Asset on Site.
+          <t xml:space="preserve">1. All five chips are shown: Status, Customer, Lead Technician, Service Advisor, Asset on Site.
 2. Each chip opens its dropdown and can be used.
 ---
-This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S9-R1).</t>
+This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S9-R1).
+AUTOMATION: READY
+</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
@@ -3395,11 +3505,13 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>1. The Status chip is not shown on this tab at all - only four chips appear. The tab already pre-filters the list to Estimate.
+          <t xml:space="preserve">1. The Status chip is not shown on this tab at all - only four chips appear. The tab already pre-filters the list to Estimate.
 2. Customer, Lead Technician, Service Advisor and Asset on Site chips are shown and usable.
 3. After step 4 the table shows only that customer's ESTIMATE work orders - the customer filter narrows the pre-filtered Estimates list.
 ---
-This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S9-R2, S2-N1). Note: an earlier answer of 2026-07-17 and the design frame both show the Status button greyed out and pre-filled on this tab; the specification and the build both hide it, and the specification is the newer source, so this test follows the specification and the build.</t>
+This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S9-R2, S2-N1). Note: an earlier answer of 2026-07-17 and the design frame both show the Status button greyed out and pre-filled on this tab; the specification and the build both hide it, and the specification is the newer source, so this test follows the specification and the build.
+AUTOMATION: READY
+</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -3449,11 +3561,13 @@
       </c>
       <c r="G58" s="2" t="inlineStr">
         <is>
-          <t>1. The Status chip is not shown on this tab at all - only four chips appear. The tab already pre-filters the list to Complete.
+          <t xml:space="preserve">1. The Status chip is not shown on this tab at all - only four chips appear. The tab already pre-filters the list to Complete.
 2. Customer, Lead Technician, Service Advisor and Asset on Site chips are shown and usable.
 3. After step 4 the table shows only that customer's COMPLETE work orders.
 ---
-This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S9-R3, S2-N2). Note: an earlier answer of 2026-07-17 and the design frame both show the Status button greyed out and pre-filled on this tab; the specification and the build both hide it, and the specification is the newer source, so this test follows the specification and the build.</t>
+This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S9-R3, S2-N2). Note: an earlier answer of 2026-07-17 and the design frame both show the Status button greyed out and pre-filled on this tab; the specification and the build both hide it, and the specification is the newer source, so this test follows the specification and the build.
+AUTOMATION: READY
+</t>
         </is>
       </c>
       <c r="H58" s="2" t="inlineStr">
@@ -3501,11 +3615,13 @@
       </c>
       <c r="G59" s="2" t="inlineStr">
         <is>
-          <t>1. All five filter chips are shown on the My Work Orders tab.
+          <t xml:space="preserve">1. All five filter chips are shown on the My Work Orders tab.
 2. The table only ever shows work orders assigned to you (the tab's own scope stays).
 3. After step 2 it shows only YOUR work orders in the ticked status - the filters narrow the user-scoped list, they do not widen it to other users' work orders.
 ---
-This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S9-R4).</t>
+This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S9-R4).
+AUTOMATION: READY
+</t>
         </is>
       </c>
       <c r="H59" s="2" t="inlineStr">
@@ -3552,11 +3668,13 @@
       </c>
       <c r="G60" s="2" t="inlineStr">
         <is>
-          <t>1. On the Estimates tab your Status choice is not applied and cannot be changed - the Status chip is not shown on that tab. The Customer selection is still shown and still filters the list.
+          <t xml:space="preserve">1. On the Estimates tab your Status choice is not applied and cannot be changed - the Status chip is not shown on that tab. The Customer selection is still shown and still filters the list.
 2. Back on the All tab the Status chip reappears with the SAME selection (Approved) still applied - the selection was retained in memory, not lost.
 3. The Customer selection is unchanged throughout.
 ---
-This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S9-R5, S9-N1, S9-R2).</t>
+This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S9-R5, S9-N1, S9-R2).
+AUTOMATION: READY
+</t>
         </is>
       </c>
       <c r="H60" s="2" t="inlineStr">
@@ -3603,10 +3721,12 @@
       </c>
       <c r="G61" s="2" t="inlineStr">
         <is>
-          <t>1. On the very first visit the Estimates tab is the selected one, even though All is the FIRST tab in the row (order and default are different on purpose).
+          <t xml:space="preserve">1. On the very first visit the Estimates tab is the selected one, even though All is the FIRST tab in the row (order and default are different on purpose).
 2. After switching to All and returning, the All tab is selected - the app remembers your last-used tab per account.
 ---
-This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch) and epic SV-8785. The Filters specification version 1.6 as revised on 4 August 2026 has no numbered requirement for this, so there is no requirement reference to give. The position on this point comes from Branko's answers, in this file: build/filters/branko-answers-2026-08-04/answers-ingested.md (https://github.com/bmuzamil-shopview/Manual-test-Cases/blob/main/build/filters/branko-answers-2026-08-04/answers-ingested.md)</t>
+This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch) and epic SV-8785. The Filters specification version 1.6 as revised on 4 August 2026 has no numbered requirement for this, so there is no requirement reference to give. The position on this point comes from Branko's answers, in this file: build/filters/branko-answers-2026-08-04/answers-ingested.md (https://github.com/bmuzamil-shopview/Manual-test-Cases/blob/main/build/filters/branko-answers-2026-08-04/answers-ingested.md)
+AUTOMATION: READY
+</t>
         </is>
       </c>
       <c r="H61" s="2" t="inlineStr">
@@ -3660,7 +3780,7 @@
       </c>
       <c r="G62" s="2" t="inlineStr">
         <is>
-          <t>&lt;ol&gt;
+          <t xml:space="preserve">&lt;ol&gt;
 &lt;li&gt;After step 2 the same Status and Customer selections are still applied - chips active with the same values, table filtered the same way.&lt;/li&gt;
 &lt;li&gt;The filter bar is still expanded (as you left it).&lt;/li&gt;
 &lt;li&gt;After step 4 the filter bar comes back collapsed - the collapsed/expanded state is restored too.&lt;/li&gt;
@@ -3669,7 +3789,9 @@
 &lt;p&gt;This is the expected behaviour as per epic SV-8785 and the Filters specification version 1.6 (S10-R1, S1-R7).&lt;/p&gt;
 Known issue: on the build tested the Customer, Lead Technician and Service Advisor buttons come back switched on but WITHOUT the name of the value you picked - the button reads just "Customer" instead of "Customer: Iibay Landscaping". The list is still filtered correctly. The Status and Asset on Site buttons keep their value. Until it is fixed this test is expected to fail on that point - it is already reported. Ticket: https://shopview.atlassian.net/browse/SV-8871
 ---
-This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S10-R1, S1-R7).</t>
+This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S10-R1, S1-R7).
+AUTOMATION: READY - EXPECT FAIL (SV-8871)
+</t>
         </is>
       </c>
       <c r="H62" s="2" t="inlineStr">
@@ -3719,11 +3841,13 @@
       </c>
       <c r="G63" s="2" t="inlineStr">
         <is>
-          <t>1. After moving around the app (step 2) the filter selections are still applied - you do not have to re-apply them.
+          <t xml:space="preserve">1. After moving around the app (step 2) the filter selections are still applied - you do not have to re-apply them.
 2. After closing the browser completely and signing back in (step 5) the same filter selections are still applied - the app remembers your filters for you permanently, not just for one browser session.
 3. The same filter selections are applied on the other computer too - the filters are saved to your account, not to one computer or browser (to confirm live once built).
 ---
-This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S10-R2, S10-R3, S10-R1).</t>
+This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S10-R2, S10-R3, S10-R1).
+AUTOMATION: READY
+</t>
         </is>
       </c>
       <c r="H63" s="2" t="inlineStr">
@@ -3770,10 +3894,12 @@
       </c>
       <c r="G64" s="2" t="inlineStr">
         <is>
-          <t>1. User B does not see user A's filters - user B's page opens with user B's own (or no) filters.
+          <t xml:space="preserve">1. User B does not see user A's filters - user B's page opens with user B's own (or no) filters.
 2. User B's new filter does not change what user A sees; each user keeps their own saved filter state.
 ---
-This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S10-R3).</t>
+This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S10-R3).
+AUTOMATION: READY
+</t>
         </is>
       </c>
       <c r="H64" s="2" t="inlineStr">
@@ -3820,12 +3946,14 @@
       </c>
       <c r="G65" s="2" t="inlineStr">
         <is>
-          <t>1. The deleted customer is silently ignored - no error or warning appears.
+          <t xml:space="preserve">1. The deleted customer is silently ignored - no error or warning appears.
 2. The Customer filter now reflects only the still-valid selection (the real customer).
 3. The table is filtered by the remaining valid selection only.
 Known issue: on the build tested the deleted customer is hidden from the dropdown but is STILL used to filter the table - the address bar and the request to the server both still carry it. So step 3 above is expected to fail. It is already reported. Ticket: https://shopview.atlassian.net/browse/SV-8832
 ---
-This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S10-N1).</t>
+This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S10-N1).
+AUTOMATION: READY - EXPECT FAIL (SV-8832)
+</t>
         </is>
       </c>
       <c r="H65" s="2" t="inlineStr">
@@ -3873,11 +4001,13 @@
       </c>
       <c r="G66" s="2" t="inlineStr">
         <is>
-          <t>1. The second Parts view does NOT show the first view's selections - each view keeps its own.
+          <t xml:space="preserve">1. The second Parts view does NOT show the first view's selections - each view keeps its own.
 2. Returning to the first view restores that view's own selections.
 3. Report tabs likewise keep separate filter choices, each remembered and restored on its own tab.
 ---
-This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S10-R4).</t>
+This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S10-R4).
+AUTOMATION: READY
+</t>
         </is>
       </c>
       <c r="H66" s="2" t="inlineStr">
@@ -3923,10 +4053,12 @@
       </c>
       <c r="G67" s="2" t="inlineStr">
         <is>
-          <t>1. The old saved choices appear in the new filter bar on the first visit - the update does not lose them (old status choices show in the Status chip, the old asset-here choice shows as Asset on Site: Yes, the old My-Work-Orders toggle maps to the My Work Orders tab, columns and sorting stay).
+          <t xml:space="preserve">1. The old saved choices appear in the new filter bar on the first visit - the update does not lose them (old status choices show in the Status chip, the old asset-here choice shows as Asset on Site: Yes, the old My-Work-Orders toggle maps to the My Work Orders tab, columns and sorting stay).
 2. Those carried-over choices are now saved to the account: the other computer shows them too.
 ---
-This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S10-R2).</t>
+This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S10-R2).
+AUTOMATION: READY
+</t>
         </is>
       </c>
       <c r="H67" s="2" t="inlineStr">
@@ -3973,10 +4105,12 @@
       </c>
       <c r="G68" s="2" t="inlineStr">
         <is>
-          <t>1. After step 1 the URL changes to include the active filter state.
+          <t xml:space="preserve">1. After step 1 the URL changes to include the active filter state.
 2. After step 3 the filter part of the URL is removed again.
 ---
-This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S11-R1).</t>
+This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S11-R1).
+AUTOMATION: READY
+</t>
         </is>
       </c>
       <c r="H68" s="2" t="inlineStr">
@@ -4022,12 +4156,14 @@
       </c>
       <c r="G69" s="2" t="inlineStr">
         <is>
-          <t>1. The page opens with the same filters already applied - chips active with the same values.
+          <t xml:space="preserve">1. The page opens with the same filters already applied - chips active with the same values.
 2. The table is already filtered accordingly on load (no need to re-apply anything).
 3. The same works from a saved bookmark.
 Known issue: two points on this test are expected to fail on the build tested. On a phone-sized screen a link carrying filters shows the buttons as on but lists the wrong work orders (ticket: https://shopview.atlassian.net/browse/SV-8845). And on a desktop screen a Customer, Lead Technician or Service Advisor button opened from a link comes back switched on but without the name of the value, so it reads just "Customer" (ticket: https://shopview.atlassian.net/browse/SV-8871). The list itself is filtered correctly on desktop. Both are already reported.
 ---
-This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S11-R2).</t>
+This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S11-R2).
+AUTOMATION: READY - EXPECT FAIL (SV-8845, SV-8871)
+</t>
         </is>
       </c>
       <c r="H69" s="2" t="inlineStr">
@@ -4074,12 +4210,14 @@
       </c>
       <c r="G70" s="2" t="inlineStr">
         <is>
-          <t>1. The page loads normally - no error.
+          <t xml:space="preserve">1. The page loads normally - no error.
 2. The deleted value is ignored; only the still-valid filter value is applied and shown on the chips.
 3. The table reflects only the valid filter.
 Known issue: a value in the address bar that no longer exists is still sent to the server, so you get an empty list instead of the list without that value. Until it is fixed this test is expected to fail on that point - it is already reported. Ticket: https://shopview.atlassian.net/browse/SV-8832
 ---
-This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S11-R3).</t>
+This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S11-R3).
+AUTOMATION: READY - EXPECT FAIL (SV-8832)
+</t>
         </is>
       </c>
       <c r="H70" s="2" t="inlineStr">
@@ -4126,12 +4264,14 @@
       </c>
       <c r="G71" s="2" t="inlineStr">
         <is>
-          <t>1. The Work Orders page loads normally.
+          <t xml:space="preserve">1. The Work Orders page loads normally.
 2. No filters are applied (chips in default state, full list shown) - the unrecognizable state is discarded.
 3. No error message or broken page appears.
 Known issue: a broken address is not fully ignored - a wrong tab value can switch the tab and a bad customer value is still sent to the server. Until it is fixed this test is expected to fail on that point - it is already reported. Ticket: https://shopview.atlassian.net/browse/SV-8832
 ---
-This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S11-N1).</t>
+This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S11-N1).
+AUTOMATION: READY - EXPECT FAIL (SV-8832)
+</t>
         </is>
       </c>
       <c r="H71" s="2" t="inlineStr">
@@ -4182,14 +4322,16 @@
       </c>
       <c r="G72" s="2" t="inlineStr">
         <is>
-          <t>1. The link's filters apply for viewing only - the page shows the shared view.
+          <t xml:space="preserve">1. The link's filters apply for viewing only - the page shows the shared view.
 2. Changes made during the link visit are also NOT saved to your account.
 3. A 'Back To My Saved Filters' option is shown while you are looking at the shared link. (If the wording on screen is slightly different, note what it says and carry on.)
 4. Clicking 'Back To My Saved Filters' brings back your own saved filters and removes the filter part from the web address.
 5. It also empties the Search box and removes your typed text - the search is not something that gets saved, so there is nothing to bring back.
 6. Returning normally later still shows your own saved filters, untouched by the link visit.
 ---
-This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S11-R6, S11-R7, S11-R8).</t>
+This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S11-R6, S11-R7, S11-R8).
+AUTOMATION: READY - EXPECT FAIL (SV-8828)
+</t>
         </is>
       </c>
       <c r="H72" s="2" t="inlineStr">
@@ -4239,12 +4381,14 @@
       </c>
       <c r="G73" s="2" t="inlineStr">
         <is>
-          <t>1. On your own view there is no 'Back To My Saved Filters' option anywhere - it only belongs to a shared-link visit.
+          <t xml:space="preserve">1. On your own view there is no 'Back To My Saved Filters' option anywhere - it only belongs to a shared-link visit.
 2. Changing your own filters does not make it appear.
 3. When you open the shared link, 'Back To My Saved Filters' does appear.
 4. After you click it and you are back on your own view, the option disappears again.
 ---
-This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S11-N3, S11-R7).</t>
+This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S11-N3, S11-R7).
+AUTOMATION: READY - EXPECT FAIL (SV-8828)
+</t>
         </is>
       </c>
       <c r="H73" s="2" t="inlineStr">
@@ -4670,12 +4814,14 @@
       </c>
       <c r="G81" s="2" t="inlineStr">
         <is>
-          <t>1. The chip for the applied filter shows the active state with the selected value(s), like on desktop.
+          <t xml:space="preserve">1. The chip for the applied filter shows the active state with the selected value(s), like on desktop.
 2. A 'Clear Filters' control appears while at least one filter is active.
 3. Using it removes all active filters, the chips return to default and the full list comes back.
 Known issue: on a phone there is no Clear Filters button at all while filters are on. Until it is fixed this test is expected to fail on that point - it is already reported. Ticket: https://shopview.atlassian.net/browse/SV-8846
 ---
-This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S12-R2, S7-R1, S8-R1).</t>
+This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S12-R2, S7-R1, S8-R1).
+AUTOMATION: READY - EXPECT FAIL (SV-8846)
+</t>
         </is>
       </c>
       <c r="H81" s="2" t="inlineStr">
@@ -4721,10 +4867,12 @@
       </c>
       <c r="G82" s="2" t="inlineStr">
         <is>
-          <t>1. There is no filter-bar collapse/expand (filter icon) toggle on mobile.
+          <t xml:space="preserve">1. There is no filter-bar collapse/expand (filter icon) toggle on mobile.
 2. The filter chip row is always visible on the mobile Work Orders page.
 ---
-This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S12-R4).</t>
+This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S12-R4).
+AUTOMATION: READY - EXPECT FAIL (no ticket - reported to the QA lead as one design item, not filed)
+</t>
         </is>
       </c>
       <c r="H82" s="2" t="inlineStr">
@@ -4830,7 +4978,7 @@
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>1. Inventory shows four filter buttons: Bin Location, Category, Supply and Vendor.
+          <t xml:space="preserve">1. Inventory shows four filter buttons: Bin Location, Category, Supply and Vendor.
 2. Part Sales shows four filter buttons: Status, Customer, Created by and Date.
 3. Catalog shows two filter buttons: Manufacturer and Category.
 4. The Returns tab shows three filter buttons: Vendor, Category and Part Type.
@@ -4845,7 +4993,9 @@
 13. Still to check on the live build: what the filter icon and the column/layout icon do (the written description does not cover the toolbar icons).
 Not built yet on the build tested: a filter bar exists on Inventory, Part Sales, Catalog and Returns, but Purchase Orders, Vendor Invoices and Vendors have no filter bar at all. If the filter bar is missing on the view you are testing, mark this test BLOCKED - do not mark it failed.
 ---
-This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch) and epic SV-8785. The Filters specification version 1.6 as revised on 4 August 2026 has no numbered requirement for this, so there is no requirement reference to give. The position on this point comes from Branko's answers, in this file: build/filters/branko-answers-2026-08-04/answers-ingested.md (https://github.com/bmuzamil-shopview/Manual-test-Cases/blob/main/build/filters/branko-answers-2026-08-04/answers-ingested.md)</t>
+This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch) and epic SV-8785. The Filters specification version 1.6 as revised on 4 August 2026 has no numbered requirement for this, so there is no requirement reference to give. The position on this point comes from Branko's answers, in this file: build/filters/branko-answers-2026-08-04/answers-ingested.md (https://github.com/bmuzamil-shopview/Manual-test-Cases/blob/main/build/filters/branko-answers-2026-08-04/answers-ingested.md)
+AUTOMATION: HOLD - the feature is not in the product yet
+</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr">
@@ -4893,13 +5043,15 @@
       </c>
       <c r="G85" s="2" t="inlineStr">
         <is>
-          <t>1. A small menu opens with two options: Core and Non Core.
+          <t xml:space="preserve">1. A small menu opens with two options: Core and Non Core.
 2. A Clear Selection action is shown at the bottom of the menu.
 3. You can tick both Core and Non Core at the same time - this filter allows more than one choice.
 4. As soon as you tick a choice the list below narrows to matching parts straight away, with no Apply button to press; Clear Selection puts the list back.
 Not built yet on the build tested: a filter bar exists on Inventory, Part Sales, Catalog and Returns, but Purchase Orders, Vendor Invoices and Vendors have no filter bar at all. If the filter bar is missing on the view you are testing, mark this test BLOCKED - do not mark it failed.
 ---
-This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch) and epic SV-8785. The Filters specification version 1.6 as revised on 4 August 2026 has no numbered requirement for this, so there is no requirement reference to give. The position on this point comes from Branko's answers, in this file: build/filters/branko-answers-2026-08-04/answers-ingested.md (https://github.com/bmuzamil-shopview/Manual-test-Cases/blob/main/build/filters/branko-answers-2026-08-04/answers-ingested.md)</t>
+This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch) and epic SV-8785. The Filters specification version 1.6 as revised on 4 August 2026 has no numbered requirement for this, so there is no requirement reference to give. The position on this point comes from Branko's answers, in this file: build/filters/branko-answers-2026-08-04/answers-ingested.md (https://github.com/bmuzamil-shopview/Manual-test-Cases/blob/main/build/filters/branko-answers-2026-08-04/answers-ingested.md)
+AUTOMATION: HOLD - the feature is not in the product yet
+</t>
         </is>
       </c>
       <c r="H85" s="2" t="inlineStr">
@@ -4946,12 +5098,14 @@
       </c>
       <c r="G86" s="2" t="inlineStr">
         <is>
-          <t>1. The table updates to show only the rows that match the chosen filter value.
+          <t xml:space="preserve">1. The table updates to show only the rows that match the chosen filter value.
 2. The chosen value is shown on the filter button so you can see what is applied.
 3. The list narrows as soon as you pick the value - there is no Apply or Search button to press. Every filter button on every Parts page works this way.
 Not built yet on the build tested: a filter bar exists on Inventory, Part Sales, Catalog and Returns, but Purchase Orders, Vendor Invoices and Vendors have no filter bar at all. If the filter bar is missing on the view you are testing, mark this test BLOCKED - do not mark it failed.
 ---
-This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch) and epic SV-8785. The Filters specification version 1.6 as revised on 4 August 2026 has no numbered requirement for this, so there is no requirement reference to give. The position on this point comes from Branko's answers, in this file: build/filters/branko-answers-2026-08-04/answers-ingested.md (https://github.com/bmuzamil-shopview/Manual-test-Cases/blob/main/build/filters/branko-answers-2026-08-04/answers-ingested.md)</t>
+This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch) and epic SV-8785. The Filters specification version 1.6 as revised on 4 August 2026 has no numbered requirement for this, so there is no requirement reference to give. The position on this point comes from Branko's answers, in this file: build/filters/branko-answers-2026-08-04/answers-ingested.md (https://github.com/bmuzamil-shopview/Manual-test-Cases/blob/main/build/filters/branko-answers-2026-08-04/answers-ingested.md)
+AUTOMATION: HOLD - the feature is not in the product yet
+</t>
         </is>
       </c>
       <c r="H86" s="2" t="inlineStr">
@@ -4998,12 +5152,14 @@
       </c>
       <c r="G87" s="2" t="inlineStr">
         <is>
-          <t>1. More than one value can be chosen inside the filter, and the button shows what you picked.
+          <t xml:space="preserve">1. More than one value can be chosen inside the filter, and the button shows what you picked.
 2. Clear Selection removes the choices for that one filter.
 3. A Clear Filters button appears in the filter bar while any filter is set, and using it clears them all at once - exactly as it works on the Work Orders page.
 Not built yet on the build tested: a filter bar exists on Inventory, Part Sales, Catalog and Returns, but Purchase Orders, Vendor Invoices and Vendors have no filter bar at all. If the filter bar is missing on the view you are testing, mark this test BLOCKED - do not mark it failed.
 ---
-This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch) and epic SV-8785. The Filters specification version 1.6 as revised on 4 August 2026 has no numbered requirement for this, so there is no requirement reference to give. The position on this point comes from Branko's answers, in this file: build/filters/branko-answers-2026-08-04/answers-ingested.md (https://github.com/bmuzamil-shopview/Manual-test-Cases/blob/main/build/filters/branko-answers-2026-08-04/answers-ingested.md)</t>
+This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch) and epic SV-8785. The Filters specification version 1.6 as revised on 4 August 2026 has no numbered requirement for this, so there is no requirement reference to give. The position on this point comes from Branko's answers, in this file: build/filters/branko-answers-2026-08-04/answers-ingested.md (https://github.com/bmuzamil-shopview/Manual-test-Cases/blob/main/build/filters/branko-answers-2026-08-04/answers-ingested.md)
+AUTOMATION: HOLD - the feature is not in the product yet
+</t>
         </is>
       </c>
       <c r="H87" s="2" t="inlineStr">
@@ -5053,12 +5209,14 @@
       </c>
       <c r="G88" s="2" t="inlineStr">
         <is>
-          <t>1. Every filter the page offered before is still offered - nothing has been taken away.
+          <t xml:space="preserve">1. Every filter the page offered before is still offered - nothing has been taken away.
 2. Every choice each of those filters offered before is still available inside the new button.
 3. If any filter or choice is missing, write down exactly which page, which filter and which choice - that is a bug worth reporting.
 Not built yet on the build tested: a filter bar exists on Inventory, Part Sales, Catalog and Returns, but Purchase Orders, Vendor Invoices and Vendors have no filter bar at all. If the filter bar is missing on the view you are testing, mark this test BLOCKED - do not mark it failed.
 ---
-This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch) and epic SV-8785. The Filters specification version 1.6 as revised on 4 August 2026 has no numbered requirement for this, so there is no requirement reference to give. The position on this point comes from Branko's answers, in this file: build/filters/branko-answers-2026-08-04/answers-ingested.md (https://github.com/bmuzamil-shopview/Manual-test-Cases/blob/main/build/filters/branko-answers-2026-08-04/answers-ingested.md)</t>
+This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch) and epic SV-8785. The Filters specification version 1.6 as revised on 4 August 2026 has no numbered requirement for this, so there is no requirement reference to give. The position on this point comes from Branko's answers, in this file: build/filters/branko-answers-2026-08-04/answers-ingested.md (https://github.com/bmuzamil-shopview/Manual-test-Cases/blob/main/build/filters/branko-answers-2026-08-04/answers-ingested.md)
+AUTOMATION: HOLD - the feature is not in the product yet
+</t>
         </is>
       </c>
       <c r="H88" s="2" t="inlineStr">
@@ -5118,7 +5276,7 @@
       </c>
       <c r="G89" s="2" t="inlineStr">
         <is>
-          <t>1. Timesheet Activities shows four filter buttons: Staff, Date, Status and Modified by.
+          <t xml:space="preserve">1. Timesheet Activities shows four filter buttons: Staff, Date, Status and Modified by.
 2. Payroll Timesheet shows two filter buttons: Employee and Date.
 3. Sales shows two filter buttons: Customer and Date.
 4. Technician Efficiency shows three filter buttons: Customer, Technician and Date — the same three on both of its view tabs, Invoiced and Completed. 'Technician' is spelled correctly here.
@@ -5144,7 +5302,9 @@
 24. Still to check on the live build: the real columns of the Sales Tax report and of the six A/R and A/P aging reports. The design uses sample placeholder tables for those, and the written description does not list their columns.
 Not built yet on the build tested: only the first report tab (Timesheet Activities) has a filter bar, with a Date Range and a Filter by Staff button, and no report tab has a page search box. If the controls this test needs are missing, mark this test BLOCKED - do not mark it failed.
 ---
-This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch) and epic SV-8785. The Filters specification version 1.6 as revised on 4 August 2026 has no numbered requirement for this, so there is no requirement reference to give. The position on this point comes from Branko's answers, in this file: build/filters/branko-answers-2026-08-04/answers-ingested.md (https://github.com/bmuzamil-shopview/Manual-test-Cases/blob/main/build/filters/branko-answers-2026-08-04/answers-ingested.md)</t>
+This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch) and epic SV-8785. The Filters specification version 1.6 as revised on 4 August 2026 has no numbered requirement for this, so there is no requirement reference to give. The position on this point comes from Branko's answers, in this file: build/filters/branko-answers-2026-08-04/answers-ingested.md (https://github.com/bmuzamil-shopview/Manual-test-Cases/blob/main/build/filters/branko-answers-2026-08-04/answers-ingested.md)
+AUTOMATION: HOLD - the feature is not in the product yet
+</t>
         </is>
       </c>
       <c r="H89" s="2" t="inlineStr">
@@ -5191,11 +5351,13 @@
       </c>
       <c r="G90" s="2" t="inlineStr">
         <is>
-          <t>1. The report updates to show only the rows matching the chosen filter value, and the chosen value is shown on the filter button.
+          <t xml:space="preserve">1. The report updates to show only the rows matching the chosen filter value, and the chosen value is shown on the filter button.
 2. The report narrows as soon as you pick the value - there is no Apply or Run button to press. Every filter button on every report works this way.
 Not built yet on the build tested: only the first report tab (Timesheet Activities) has a filter bar, with a Date Range and a Filter by Staff button, and no report tab has a page search box. If the controls this test needs are missing, mark this test BLOCKED - do not mark it failed.
 ---
-This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch) and epic SV-8785. The Filters specification version 1.6 as revised on 4 August 2026 has no numbered requirement for this, so there is no requirement reference to give. The position on this point comes from Branko's answers, in this file: build/filters/branko-answers-2026-08-04/answers-ingested.md (https://github.com/bmuzamil-shopview/Manual-test-Cases/blob/main/build/filters/branko-answers-2026-08-04/answers-ingested.md)</t>
+This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch) and epic SV-8785. The Filters specification version 1.6 as revised on 4 August 2026 has no numbered requirement for this, so there is no requirement reference to give. The position on this point comes from Branko's answers, in this file: build/filters/branko-answers-2026-08-04/answers-ingested.md (https://github.com/bmuzamil-shopview/Manual-test-Cases/blob/main/build/filters/branko-answers-2026-08-04/answers-ingested.md)
+AUTOMATION: HOLD - the feature is not in the product yet
+</t>
         </is>
       </c>
       <c r="H90" s="2" t="inlineStr">
@@ -5248,14 +5410,16 @@
       </c>
       <c r="G91" s="2" t="inlineStr">
         <is>
-          <t>&lt;ol&gt;
+          <t xml:space="preserve">&lt;ol&gt;
 &lt;li&gt;Each of these filter buttons - Location, Transaction Type, Invoice Status, Type, User and Mention - opens a list of choices, lets you tick more than one, and narrows the report straight away with no Apply button.&lt;/li&gt;
 &lt;li&gt;The choices inside each filter come from your own shop's data (for example your real vendors or categories), so there is no fixed list to compare against - check that the choices you see match the data in your shop.&lt;/li&gt;
 &lt;li&gt;Write down the choices you actually see behind each of these six buttons. They have not been written down anywhere yet, so your list becomes the record.&lt;/li&gt;
 &lt;/ol&gt;
 Not built yet on the build tested: only the first report tab (Timesheet Activities) has a filter bar, with a Date Range and a Filter by Staff button, and no report tab has a page search box. If the controls this test needs are missing, mark this test BLOCKED - do not mark it failed.
 ---
-This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch) and epic SV-8785. The Filters specification version 1.6 as revised on 4 August 2026 has no numbered requirement for this, so there is no requirement reference to give. The position on this point comes from Branko's answers, in this file: build/filters/branko-answers-2026-08-04/answers-ingested.md (https://github.com/bmuzamil-shopview/Manual-test-Cases/blob/main/build/filters/branko-answers-2026-08-04/answers-ingested.md)</t>
+This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch) and epic SV-8785. The Filters specification version 1.6 as revised on 4 August 2026 has no numbered requirement for this, so there is no requirement reference to give. The position on this point comes from Branko's answers, in this file: build/filters/branko-answers-2026-08-04/answers-ingested.md (https://github.com/bmuzamil-shopview/Manual-test-Cases/blob/main/build/filters/branko-answers-2026-08-04/answers-ingested.md)
+AUTOMATION: HOLD - the feature is not in the product yet
+</t>
         </is>
       </c>
       <c r="H91" s="2" t="inlineStr">
@@ -5307,7 +5471,7 @@
       </c>
       <c r="G92" s="2" t="inlineStr">
         <is>
-          <t>1. The panel that opens offers a set of ready-made periods to choose from - on the build tested these are Today, Yesterday, This week, Last week, This month, Last month, This quarter, Last quarter, This year, Last year - plus a Custom option and a Clear Selection link. The exact set of ready-made periods may differ per report, so check the ones your report offers rather than expecting this list.
+          <t xml:space="preserve">1. The panel that opens offers a set of ready-made periods to choose from - on the build tested these are Today, Yesterday, This week, Last week, This month, Last month, This quarter, Last quarter, This year, Last year - plus a Custom option and a Clear Selection link. The exact set of ready-made periods may differ per report, so check the ones your report offers rather than expecting this list.
 2. A period is already filled in when the panel first opens (on Timesheet Activities it is This month), and the button reads that period, for example "Date Range: This month".
 3. Choosing a ready-made period applies it straight away: the results update, the button reads the period you chose, and the web address records it.
 4. Choosing Custom shows a From box and a To box. After you fill in only the From date the results do NOT change yet.
@@ -5316,7 +5480,9 @@
 Note: dates are typed in month/day/year order, the way the build shows them (for example 07/01/2026).
 Where to run this on the build tested: the Reports area has this date button on the Timesheet Activities report. Other report tabs do not have a filter bar yet - if the report you open has no date button, mark this test BLOCKED, not failed.
 ---
-This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch) and epic SV-8785. It follows the NEWER wording of the Filters specification version 1.6, in the revision published on the afternoon of 4 August 2026, which changed the date filter description in the Feature Overview and in the Key Decisions section: the date button now offers standard ready-made periods and starts with the current default range already filled in. An earlier revision of the same specification said the opposite, and this test follows the newer one. The specification does not give this a numbered requirement, so there is no requirement number to quote.</t>
+This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch) and epic SV-8785. It follows the NEWER wording of the Filters specification version 1.6, in the revision published on the afternoon of 4 August 2026, which changed the date filter description in the Feature Overview and in the Key Decisions section: the date button now offers standard ready-made periods and starts with the current default range already filled in. An earlier revision of the same specification said the opposite, and this test follows the newer one. The specification does not give this a numbered requirement, so there is no requirement number to quote.
+AUTOMATION: READY
+</t>
         </is>
       </c>
       <c r="H92" s="2" t="inlineStr">
@@ -5366,12 +5532,14 @@
       </c>
       <c r="G93" s="2" t="inlineStr">
         <is>
-          <t>1. The control expands in place into a small search box showing the placeholder 'Type to search'.
+          <t xml:space="preserve">1. The control expands in place into a small search box showing the placeholder 'Type to search'.
 2. The list narrows as you type, after a brief pause - and ONLY this page's list changes, nothing else in the app.
 3. The round x clears the text and the full list returns.
 4. Clicking away with an empty box collapses it back to the Search button; with text in it, the box stays open.
 ---
-This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S13-R1, S13-R9, S13-R12, S13-R15).</t>
+This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S13-R1, S13-R9, S13-R12, S13-R15).
+AUTOMATION: READY - EXPECT FAIL (no ticket - reported to the QA lead as one design item, not filed)
+</t>
         </is>
       </c>
       <c r="H93" s="2" t="inlineStr">
@@ -5419,11 +5587,13 @@
       </c>
       <c r="G94" s="2" t="inlineStr">
         <is>
-          <t>1. With both active, the results match the filter AND the search together (both narrow the list at once).
+          <t xml:space="preserve">1. With both active, the results match the filter AND the search together (both narrow the list at once).
 2. Clearing the search keeps the filter applied.
 3. Clearing the filter keeps the search applied - each is cleared by its own control without wiping the other.
 ---
-This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S13-R10, S13-R13, S8-R5).</t>
+This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S13-R10, S13-R13, S8-R5).
+AUTOMATION: READY - EXPECT FAIL (no ticket - reported to the QA lead as one design item, not filed)
+</t>
         </is>
       </c>
       <c r="H94" s="2" t="inlineStr">
@@ -5473,12 +5643,14 @@
       </c>
       <c r="G95" s="2" t="inlineStr">
         <is>
-          <t>1. Sorting and paging keep your search applied - your text stays in the box and the list stays narrowed.
+          <t xml:space="preserve">1. Sorting and paging keep your search applied - your text stays in the box and the list stays narrowed.
 2. Leaving the page and coming back also keeps your text in the box and the list still narrowed.
 3. The second browser tab starts clean: its Search box is empty and it shows the full list. Each tab keeps its own search.
 4. After closing the browser and coming back, the Search box is empty and the list is unsearched - a typed search is never remembered for next time (your filters, unlike the search, ARE remembered).
 ---
-This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S13-R14, S13-R25, S13-N4, S10-R5).</t>
+This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S13-R14, S13-R25, S13-N4, S10-R5).
+AUTOMATION: READY
+</t>
         </is>
       </c>
       <c r="H95" s="2" t="inlineStr">
@@ -5525,12 +5697,14 @@
       </c>
       <c r="G96" s="2" t="inlineStr">
         <is>
-          <t>1. The address contains the search term after step 1.
+          <t xml:space="preserve">1. The address contains the search term after step 1.
 2. The fresh tab opens with the search box filled and the list already narrowed.
 3. The malformed part is ignored - the page loads cleanly without an error.
 4. A search arriving via a link is view-only, the same as filters from a link - it does not overwrite your own remembered search.
 ---
-This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S11-R4, S11-R5, S11-N2, S11-R8).</t>
+This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S11-R4, S11-R5, S11-N2, S11-R8).
+AUTOMATION: READY
+</t>
         </is>
       </c>
       <c r="H96" s="2" t="inlineStr">
@@ -5578,13 +5752,15 @@
       </c>
       <c r="G97" s="2" t="inlineStr">
         <is>
-          <t>1. The search expands inline inside the toolbar - no separate popup window opens.
+          <t xml:space="preserve">1. The search expands inline inside the toolbar - no separate popup window opens.
 2. The list narrows as you type, same as desktop.
 3. To make room, the page's main button no longer stretches full-width, and pages with two or more small icon buttons collapse them into a single 'more' menu.
 4. The box stretches to fill the space left in the action row instead of staying the narrow desktop size, and every other toolbar button stays visible and in the same place while you search.
 5. There is no extra 'search is on' badge on mobile: with text in it the box simply stays open showing your text, and an empty box closes back to the Search button when you tap elsewhere - exactly as on desktop.
 ---
-This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S13-R16, S13-R17, S13-R18, S13-R19, S13-R20, S12-R5).</t>
+This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S13-R16, S13-R17, S13-R18, S13-R19, S13-R20, S12-R5).
+AUTOMATION: READY
+</t>
         </is>
       </c>
       <c r="H97" s="2" t="inlineStr">
@@ -5635,12 +5811,14 @@
       </c>
       <c r="G98" s="2" t="inlineStr">
         <is>
-          <t>1. Every table listed above has its own Search box - no table lost the ability to narrow by text.
+          <t xml:space="preserve">1. Every table listed above has its own Search box - no table lost the ability to narrow by text.
 2. Each Search box narrows only its own table; nothing else in the app changes.
 3. Where the table sits inside a dialog (the Work Order Log, the Line Log, the audit log dialog), the Search box is inside that dialog and works there.
 4. The work order Parts tab keeps the local search input it already had - it was deliberately left as it is.
 ---
-This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S14-R6, S14-R5, S13-R22, S14-N1).</t>
+This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S14-R6, S14-R5, S13-R22, S14-N1).
+AUTOMATION: READY
+</t>
         </is>
       </c>
       <c r="H98" s="2" t="inlineStr">
@@ -5688,11 +5866,13 @@
       </c>
       <c r="G99" s="2" t="inlineStr">
         <is>
-          <t>1. The page list does NOT narrow while you type in the navigation search - only its dropdown of matching records appears.
+          <t xml:space="preserve">1. The page list does NOT narrow while you type in the navigation search - only its dropdown of matching records appears.
 2. The same holds on the other pages checked.
 3. Picking a dropdown result still takes you to that record - the navigation search keeps its find-and-open role.
 ---
-This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S14-R1, S14-R2, S14-R4, S14-R5).</t>
+This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S14-R1, S14-R2, S14-R4, S14-R5).
+AUTOMATION: READY
+</t>
         </is>
       </c>
       <c r="H99" s="2" t="inlineStr">
@@ -5741,14 +5921,16 @@
       </c>
       <c r="G100" s="2" t="inlineStr">
         <is>
-          <t>1. A 'Search' button is shown with a small magnifier icon next to the word 'Search'; it is plain text on a see-through background, with no border and no fill.
+          <t xml:space="preserve">1. A 'Search' button is shown with a small magnifier icon next to the word 'Search'; it is plain text on a see-through background, with no border and no fill.
 2. Hovering over it gives it a light grey background; the word 'Search' keeps its own colour.
 3. Clicking it turns the button into a small text box in the same spot (the design sets it at 180 pixels wide), the typing cursor is already inside it, and the box grows towards the left so the other toolbar buttons do not move.
 4. While the box is empty it shows the magnifier icon and the grey placeholder text 'Type to search'.
 5. As soon as you type, your text shows in a dark grey and a small round x appears at the right-hand end of the box.
 6. A very long sentence does not make the box grow and does not cut the text off - the text scrolls sideways inside the box and the cursor stays where you are typing.
 ---
-This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S13-R2, S13-R3, S13-R4, S13-R5, S13-R6, S13-R8).</t>
+This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S13-R2, S13-R3, S13-R4, S13-R5, S13-R6, S13-R8).
+AUTOMATION: READY - EXPECT FAIL (no ticket - reported to the QA lead as one design item, not filed)
+</t>
         </is>
       </c>
       <c r="H100" s="2" t="inlineStr">
@@ -5798,14 +5980,16 @@
       </c>
       <c r="G101" s="2" t="inlineStr">
         <is>
-          <t>1. The list narrows on its own a moment after you stop typing (about a third of a second) - you never press Enter or any button.
+          <t xml:space="preserve">1. The list narrows on its own a moment after you stop typing (about a third of a second) - you never press Enter or any button.
 2. The matching rows appear in the table you were already looking at; no separate results page, results list or pop-up window opens.
 3. There is no Apply or Submit button anywhere next to the Search box.
 4. Pressing Enter changes nothing that has not already happened - the same rows stay listed and no page reload happens.
 5. Parts Inventory behaves the same way, only it waits a fraction longer before reacting; that longer wait is on purpose because that page carries more data.
 Known and accepted: the empty screen offers no way to clear the search on its own. The product behaves this way on purpose for now. Do not raise this as a new problem.
 ---
-This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S13-R7, S13-R12).</t>
+This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S13-R7, S13-R12).
+AUTOMATION: READY - EXPECT FAIL (SV-8847 - closed as accepted, will not be fixed)
+</t>
         </is>
       </c>
       <c r="H101" s="2" t="inlineStr">
@@ -5854,12 +6038,14 @@
       </c>
       <c r="G102" s="2" t="inlineStr">
         <is>
-          <t>1. On the All tab only the rows matching your word remain.
+          <t xml:space="preserve">1. On the All tab only the rows matching your word remain.
 2. On the Estimates tab your word is still in the Search box, and the list shows only Estimates rows that match it - no rows from the other tabs appear.
 3. The Completed tab behaves the same way: your word is still there and only that tab's matching rows are listed.
 4. Clearing the search clears it for all the Work Orders tabs - they share one search - and each tab shows its full list again.
 ---
-This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S13-R11, S13-R24).</t>
+This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S13-R11, S13-R24).
+AUTOMATION: READY
+</t>
         </is>
       </c>
       <c r="H102" s="2" t="inlineStr">
@@ -5908,12 +6094,14 @@
       </c>
       <c r="G103" s="2" t="inlineStr">
         <is>
-          <t>1. The second Parts view opens with an empty Search box and its full list - the word you typed on the first view is not carried over.
+          <t xml:space="preserve">1. The second Parts view opens with an empty Search box and its full list - the word you typed on the first view is not carried over.
 2. Going back to the first view brings its own word back and narrows its list again.
 3. Each report tab behaves the same way: a word typed on one tab stays on that tab only, and each tab remembers its own.
 4. No search is ever applied to a table it was not typed on.
 ---
-This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S13-R24, S13-R11, S10-R4).</t>
+This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S13-R24, S13-R11, S10-R4).
+AUTOMATION: READY
+</t>
         </is>
       </c>
       <c r="H103" s="2" t="inlineStr">
@@ -5961,12 +6149,14 @@
       </c>
       <c r="G104" s="2" t="inlineStr">
         <is>
-          <t>1. The page opens with the normal list for your own saved filters - the old search word does NOT narrow the list.
+          <t xml:space="preserve">1. The page opens with the normal list for your own saved filters - the old search word does NOT narrow the list.
 2. The page's own Search box is empty; nothing was carried into it.
 3. No error is shown - the leftover search part in the address is simply ignored. (Whether it also disappears from the address is not important; note what you see.)
 4. After typing in the top-of-screen search and reloading, the list is still not narrowed and nothing about that word was remembered for the list.
 ---
-This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S14-R3, S14-R2, S14-R1).</t>
+This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S14-R3, S14-R2, S14-R1).
+AUTOMATION: READY
+</t>
         </is>
       </c>
       <c r="H104" s="2" t="inlineStr">
@@ -6014,11 +6204,13 @@
       </c>
       <c r="G105" s="2" t="inlineStr">
         <is>
-          <t>1. The list stays narrowed by your word - collapsing the filter bar does not cancel the search.
+          <t xml:space="preserve">1. The list stays narrowed by your word - collapsing the filter bar does not cancel the search.
 2. The Search box stays in the toolbar row with your word still showing; it is not tucked away with the filter bar, because the search sits in the toolbar row and the chips sit in the row below.
 3. Expanding the bar again changes nothing about the search or the narrowed list.
 ---
-This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S13-E1).</t>
+This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S13-E1).
+AUTOMATION: READY
+</t>
         </is>
       </c>
       <c r="H105" s="2" t="inlineStr">
@@ -6065,11 +6257,13 @@
       </c>
       <c r="G106" s="2" t="inlineStr">
         <is>
-          <t>1. The list request includes the active filter selections as request parameters (status values and customer identifiers).
+          <t xml:space="preserve">1. The list request includes the active filter selections as request parameters (status values and customer identifiers).
 2. The request succeeds (HTTP 200).
 3. The response contains only work orders matching the filters - the filtering is done by the backend, not just hidden client-side.
 ---
-This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S2-R2, S3-R6).</t>
+This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S2-R2, S3-R6).
+AUTOMATION: READY
+</t>
         </is>
       </c>
       <c r="H106" s="2" t="inlineStr">
@@ -6115,11 +6309,13 @@
       </c>
       <c r="G107" s="2" t="inlineStr">
         <is>
-          <t>1. One request carries both filters together (both statuses and the customer).
+          <t xml:space="preserve">1. One request carries both filters together (both statuses and the customer).
 2. The response returns customer A's Estimate and Approved work orders only.
 3. Customer B's work orders are absent - the customer filter and status filter both restrict the result, while the two statuses combine as either-or.
 ---
-This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S2-R2, S3-R6, S8-R3).</t>
+This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S2-R2, S3-R6, S8-R3).
+AUTOMATION: READY
+</t>
         </is>
       </c>
       <c r="H107" s="2" t="inlineStr">
@@ -6165,12 +6361,14 @@
       </c>
       <c r="G108" s="2" t="inlineStr">
         <is>
-          <t>1. The backend does not fail with a server error (no HTTP 5xx).
+          <t xml:space="preserve">1. The backend does not fail with a server error (no HTTP 5xx).
 2. The response is a normal, successful list response - the invalid value is ignored or simply matches nothing.
 3. Any still-valid filter values in the same request are applied normally.
 Known issue: the server does not fail, but the value that no longer exists is still applied instead of being dropped. Until it is fixed this test is expected to fail on that point - it is already reported. Ticket: https://shopview.atlassian.net/browse/SV-8832
 ---
-This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S10-N1, S11-R3).</t>
+This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S10-N1, S11-R3).
+AUTOMATION: READY - EXPECT FAIL (SV-8832)
+</t>
         </is>
       </c>
       <c r="H108" s="2" t="inlineStr">
@@ -6217,11 +6415,13 @@
       </c>
       <c r="G109" s="2" t="inlineStr">
         <is>
-          <t>1. The backend responds gracefully - no HTTP 5xx / crash; either a normal (unfiltered or empty) list or a clean validation response.
+          <t xml:space="preserve">1. The backend responds gracefully - no HTTP 5xx / crash; either a normal (unfiltered or empty) list or a clean validation response.
 2. In the browser the page still loads without filters and without an error message, matching the malformed-URL requirement.
 Known issue: the server does not fail, but a broken address is not fully ignored by the page. Until it is fixed this test is expected to fail on that point - it is already reported. Ticket: https://shopview.atlassian.net/browse/SV-8832
 ---
-This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S11-N1).</t>
+This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S11-N1).
+AUTOMATION: READY - EXPECT FAIL (SV-8832)
+</t>
         </is>
       </c>
       <c r="H109" s="2" t="inlineStr">
@@ -6267,11 +6467,13 @@
       </c>
       <c r="G110" s="2" t="inlineStr">
         <is>
-          <t>1. The request succeeds (HTTP 200).
+          <t xml:space="preserve">1. The request succeeds (HTTP 200).
 2. The response contains an empty result set (zero work orders) - an empty match is a normal outcome, not an error.
 3. The page renders the no-results empty state from this response.
 ---
-This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S8-R3, S2-N3).</t>
+This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S8-R3, S2-N3).
+AUTOMATION: READY
+</t>
         </is>
       </c>
       <c r="H110" s="2" t="inlineStr">
@@ -6319,13 +6521,15 @@
       </c>
       <c r="G111" s="2" t="inlineStr">
         <is>
-          <t>1. Changing a filter sends a save (PUT) to the per-user page-preferences service carrying the page's state, and it succeeds (HTTP 200).
+          <t xml:space="preserve">1. Changing a filter sends a save (PUT) to the per-user page-preferences service carrying the page's state, and it succeeds (HTTP 200).
 2. On reload the page requests the saved state back (GET, HTTP 200) and applies it - the filters return without you redoing them.
 3. The second user does NOT receive the first user's saved state - each account's saved filters are isolated.
 4. Asking for a never-saved key returns success with an empty value, not an error page.
 Step 3 needs a SECOND sign-in of your own. We could not run it for you: impersonating another user on this branch returns an error, and a new staff member cannot finish signing up because the invitation email cannot be received here. If you have a second account, run step 3 normally. If you do not, mark this test BLOCKED - do not mark it failed. Steps 1, 2 and 4 were confirmed working.
 ---
-This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S10-R2, S10-R3).</t>
+This is the expected behaviour as per the build tested on 8/5/2026 (ShopView v3.4.2-d00239b on the Filters QA branch), epic SV-8785 and the Filters specification version 1.6 as revised on 4 August 2026 (S10-R2, S10-R3).
+AUTOMATION: HOLD - needs a second test login to prove one person's saved filters do not reach another
+</t>
         </is>
       </c>
       <c r="H111" s="2" t="inlineStr">

</xml_diff>